<commit_message>
feat: add figure code
</commit_message>
<xml_diff>
--- a/data/proteomics/physiology_collection.xlsx
+++ b/data/proteomics/physiology_collection.xlsx
@@ -5,17 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Documents/GitHub/De-nevo-protein-3D-structure-yeast/data/proteomics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{919ACB8D-611B-ED4E-B284-53643CDCB86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67790435-58F9-4644-8DFA-12F03F5D194D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26880" yWindow="500" windowWidth="40960" windowHeight="22540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="26880" windowHeight="15220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
-    <sheet name="Supplementary File 1e vip" sheetId="1" r:id="rId3"/>
+    <sheet name="Supplementary File 1e vip" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$S$1:$S$77</definedName>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="113">
   <si>
     <t>sample</t>
   </si>
@@ -373,9 +372,6 @@
   </si>
   <si>
     <t>D=0.027_M</t>
-  </si>
-  <si>
-    <t>r_1992</t>
   </si>
 </sst>
 </file>
@@ -385,7 +381,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -527,11 +523,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri (Body)"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -565,7 +556,7 @@
       <name val="Times Roman"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -769,6 +760,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -953,63 +950,63 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="24" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="10" xfId="6" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="6" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4272,12 +4269,14 @@
         <v>0.42361575000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:23" s="20" customFormat="1">
-      <c r="A48" s="18" t="s">
+    <row r="48" spans="1:23" s="26" customFormat="1">
+      <c r="A48" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="B48" s="19"/>
-      <c r="P48" s="21"/>
+      <c r="B48" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="P48" s="27"/>
     </row>
     <row r="49" spans="1:16" s="7" customFormat="1">
       <c r="A49" s="4" t="s">
@@ -4345,25 +4344,37 @@
       <c r="A53" s="1" t="s">
         <v>66</v>
       </c>
+      <c r="B53" s="12">
+        <v>0.1</v>
+      </c>
       <c r="P53" s="11"/>
     </row>
     <row r="54" spans="1:16" s="12" customFormat="1">
       <c r="A54" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D54" s="22"/>
+      <c r="B54" s="12">
+        <v>0.1</v>
+      </c>
+      <c r="D54" s="18"/>
       <c r="P54" s="11"/>
     </row>
     <row r="55" spans="1:16" s="12" customFormat="1">
       <c r="A55" s="1" t="s">
         <v>68</v>
       </c>
+      <c r="B55" s="12">
+        <v>0.1</v>
+      </c>
       <c r="P55" s="11"/>
     </row>
     <row r="56" spans="1:16" s="12" customFormat="1">
       <c r="A56" s="1" t="s">
         <v>69</v>
       </c>
+      <c r="B56" s="12">
+        <v>0.1</v>
+      </c>
       <c r="P56" s="11"/>
     </row>
     <row r="57" spans="1:16" s="12" customFormat="1">
@@ -4438,300 +4449,300 @@
       </c>
       <c r="P68" s="11"/>
     </row>
-    <row r="69" spans="1:23" s="23" customFormat="1">
+    <row r="69" spans="1:23" s="19" customFormat="1">
       <c r="A69" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B69" s="23">
+      <c r="B69" s="19">
         <v>2.7E-2</v>
       </c>
-      <c r="C69" s="24">
+      <c r="C69" s="20">
         <v>-0.33700000000000002</v>
       </c>
-      <c r="D69" s="24">
+      <c r="D69" s="20">
         <v>-0.151308114750691</v>
       </c>
-      <c r="I69" s="24">
-        <v>0</v>
-      </c>
-      <c r="N69" s="24">
+      <c r="I69" s="20">
+        <v>0</v>
+      </c>
+      <c r="N69" s="20">
         <v>0.878</v>
       </c>
-      <c r="O69" s="25">
+      <c r="O69" s="21">
         <v>-0.86358170086251695</v>
       </c>
-      <c r="P69" s="26"/>
-      <c r="Q69" s="23" t="s">
+      <c r="P69" s="22"/>
+      <c r="Q69" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S69" s="23" t="s">
+      <c r="S69" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W69" s="23">
+      <c r="W69" s="19">
         <v>0.29899999999999999</v>
       </c>
     </row>
-    <row r="70" spans="1:23" s="25" customFormat="1">
+    <row r="70" spans="1:23" s="21" customFormat="1">
       <c r="A70" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="B70" s="25">
+      <c r="B70" s="21">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="C70" s="24">
+      <c r="C70" s="20">
         <v>-0.52300000000000002</v>
       </c>
-      <c r="D70" s="24">
+      <c r="D70" s="20">
         <v>-0.22220072795676099</v>
       </c>
-      <c r="I70" s="24">
-        <v>0</v>
-      </c>
-      <c r="N70" s="24">
+      <c r="I70" s="20">
+        <v>0</v>
+      </c>
+      <c r="N70" s="20">
         <v>1.458</v>
       </c>
-      <c r="O70" s="25">
+      <c r="O70" s="21">
         <v>-1.4368262739973601</v>
       </c>
-      <c r="P70" s="27"/>
-      <c r="Q70" s="23" t="s">
+      <c r="P70" s="23"/>
+      <c r="Q70" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S70" s="23" t="s">
+      <c r="S70" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W70" s="25">
+      <c r="W70" s="21">
         <v>0.312</v>
       </c>
     </row>
-    <row r="71" spans="1:23" s="25" customFormat="1">
+    <row r="71" spans="1:23" s="21" customFormat="1">
       <c r="A71" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B71" s="25">
+      <c r="B71" s="21">
         <v>0.10199999999999999</v>
       </c>
-      <c r="C71" s="24">
+      <c r="C71" s="20">
         <v>-1.171</v>
       </c>
-      <c r="D71" s="24">
+      <c r="D71" s="20">
         <v>-0.59240301221006997</v>
       </c>
-      <c r="I71" s="24">
-        <v>0</v>
-      </c>
-      <c r="N71" s="24">
+      <c r="I71" s="20">
+        <v>0</v>
+      </c>
+      <c r="N71" s="20">
         <v>2.5470000000000002</v>
       </c>
-      <c r="O71" s="25">
+      <c r="O71" s="21">
         <v>-2.4905493340587901</v>
       </c>
-      <c r="P71" s="27"/>
-      <c r="Q71" s="23" t="s">
+      <c r="P71" s="23"/>
+      <c r="Q71" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S71" s="23" t="s">
+      <c r="S71" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W71" s="25">
+      <c r="W71" s="21">
         <v>0.371</v>
       </c>
     </row>
-    <row r="72" spans="1:23" s="25" customFormat="1">
+    <row r="72" spans="1:23" s="21" customFormat="1">
       <c r="A72" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="B72" s="25">
+      <c r="B72" s="21">
         <v>0.152</v>
       </c>
-      <c r="C72" s="24">
+      <c r="C72" s="20">
         <v>-1.6830000000000001</v>
       </c>
-      <c r="D72" s="24">
+      <c r="D72" s="20">
         <v>-0.81572561388224996</v>
       </c>
-      <c r="I72" s="24">
-        <v>0</v>
-      </c>
-      <c r="N72" s="24">
+      <c r="I72" s="20">
+        <v>0</v>
+      </c>
+      <c r="N72" s="20">
         <v>3.81518914277475</v>
       </c>
-      <c r="O72" s="25">
+      <c r="O72" s="21">
         <v>-3.855</v>
       </c>
-      <c r="P72" s="27"/>
-      <c r="Q72" s="23" t="s">
+      <c r="P72" s="23"/>
+      <c r="Q72" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S72" s="23" t="s">
+      <c r="S72" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W72" s="25">
+      <c r="W72" s="21">
         <v>0.41899999999999998</v>
       </c>
     </row>
-    <row r="73" spans="1:23" s="25" customFormat="1">
+    <row r="73" spans="1:23" s="21" customFormat="1">
       <c r="A73" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="B73" s="25">
+      <c r="B73" s="21">
         <v>0.214</v>
       </c>
-      <c r="C73" s="24">
+      <c r="C73" s="20">
         <v>-2.4769999999999999</v>
       </c>
-      <c r="D73" s="24">
+      <c r="D73" s="20">
         <v>-1.22567508688439</v>
       </c>
-      <c r="I73" s="24">
+      <c r="I73" s="20">
         <v>-3.4044364549679102E-12</v>
       </c>
-      <c r="N73" s="24">
+      <c r="N73" s="20">
         <v>5.5949999999999998</v>
       </c>
-      <c r="O73" s="25">
+      <c r="O73" s="21">
         <v>-5.4782042149448502</v>
       </c>
-      <c r="P73" s="27"/>
-      <c r="Q73" s="23" t="s">
+      <c r="P73" s="23"/>
+      <c r="Q73" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S73" s="23" t="s">
+      <c r="S73" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W73" s="25">
+      <c r="W73" s="21">
         <v>0.32</v>
       </c>
     </row>
-    <row r="74" spans="1:23" s="25" customFormat="1">
+    <row r="74" spans="1:23" s="21" customFormat="1">
       <c r="A74" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B74" s="25">
+      <c r="B74" s="21">
         <v>0.254</v>
       </c>
-      <c r="C74" s="24">
+      <c r="C74" s="20">
         <v>-2.8620000000000001</v>
       </c>
-      <c r="D74" s="24">
+      <c r="D74" s="20">
         <v>-1.4136198692773401</v>
       </c>
-      <c r="I74" s="24">
+      <c r="I74" s="20">
         <v>7.3805128675275E-12</v>
       </c>
-      <c r="N74" s="24">
+      <c r="N74" s="20">
         <v>6.484</v>
       </c>
-      <c r="O74" s="25">
+      <c r="O74" s="21">
         <v>-6.2489999999999997</v>
       </c>
-      <c r="P74" s="27"/>
-      <c r="Q74" s="23" t="s">
+      <c r="P74" s="23"/>
+      <c r="Q74" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S74" s="23" t="s">
+      <c r="S74" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W74" s="25">
+      <c r="W74" s="21">
         <v>0.37799999999999995</v>
       </c>
     </row>
-    <row r="75" spans="1:23" s="25" customFormat="1">
+    <row r="75" spans="1:23" s="21" customFormat="1">
       <c r="A75" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B75" s="25">
+      <c r="B75" s="21">
         <v>0.28399999999999997</v>
       </c>
-      <c r="C75" s="24">
+      <c r="C75" s="20">
         <v>-3.2050000000000001</v>
       </c>
-      <c r="D75" s="24">
+      <c r="D75" s="20">
         <v>-1.47353470842518</v>
       </c>
-      <c r="I75" s="24">
+      <c r="I75" s="20">
         <v>-3.4111879987364099E-12</v>
       </c>
-      <c r="N75" s="24">
+      <c r="N75" s="20">
         <v>8.0890000000000004</v>
       </c>
-      <c r="O75" s="25">
+      <c r="O75" s="21">
         <v>-7.9485854277214001</v>
       </c>
-      <c r="P75" s="27"/>
-      <c r="Q75" s="23" t="s">
+      <c r="P75" s="23"/>
+      <c r="Q75" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S75" s="23" t="s">
+      <c r="S75" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W75" s="25">
+      <c r="W75" s="21">
         <v>0.39100000000000001</v>
       </c>
     </row>
-    <row r="76" spans="1:23" s="25" customFormat="1">
+    <row r="76" spans="1:23" s="21" customFormat="1">
       <c r="A76" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B76" s="25">
+      <c r="B76" s="21">
         <v>0.33400000000000002</v>
       </c>
-      <c r="C76" s="24">
+      <c r="C76" s="20">
         <v>-5.2350000000000003</v>
       </c>
-      <c r="D76" s="24">
+      <c r="D76" s="20">
         <v>-1.99253212300414</v>
       </c>
-      <c r="I76" s="24">
+      <c r="I76" s="20">
         <v>2.0830000000081101</v>
       </c>
-      <c r="N76" s="24">
+      <c r="N76" s="20">
         <v>11.872999999999999</v>
       </c>
-      <c r="O76" s="25">
+      <c r="O76" s="21">
         <v>-9.6077296533960403</v>
       </c>
-      <c r="P76" s="27"/>
-      <c r="Q76" s="23" t="s">
+      <c r="P76" s="23"/>
+      <c r="Q76" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S76" s="23" t="s">
+      <c r="S76" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W76" s="25">
+      <c r="W76" s="21">
         <v>0.41899999999999998</v>
       </c>
     </row>
-    <row r="77" spans="1:23" s="25" customFormat="1">
+    <row r="77" spans="1:23" s="21" customFormat="1">
       <c r="A77" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="B77" s="25">
+      <c r="B77" s="21">
         <v>0.379</v>
       </c>
-      <c r="C77" s="24">
+      <c r="C77" s="20">
         <v>-6.9569999999999999</v>
       </c>
-      <c r="D77" s="24">
+      <c r="D77" s="20">
         <v>-2.0155334705947299</v>
       </c>
-      <c r="I77" s="24">
+      <c r="I77" s="20">
         <v>5.5389999999999997</v>
       </c>
-      <c r="N77" s="24">
+      <c r="N77" s="20">
         <v>14.304133448972699</v>
       </c>
-      <c r="O77" s="25">
+      <c r="O77" s="21">
         <v>-8.8979999999999997</v>
       </c>
-      <c r="P77" s="27"/>
-      <c r="Q77" s="23" t="s">
+      <c r="P77" s="23"/>
+      <c r="Q77" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S77" s="23" t="s">
+      <c r="S77" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W77" s="25">
+      <c r="W77" s="21">
         <v>0.39100000000000001</v>
       </c>
     </row>
@@ -4741,93 +4752,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E49AD3A4-3FFD-6442-B843-C2A9D40041A1}">
-  <dimension ref="A1:J12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B1">
-        <v>-0.86358170086251695</v>
-      </c>
-      <c r="C1">
-        <v>-1.4368262739973601</v>
-      </c>
-      <c r="D1">
-        <v>-2.4905493340587901</v>
-      </c>
-      <c r="E1">
-        <v>-3.855</v>
-      </c>
-      <c r="F1">
-        <v>-5.4782042149448502</v>
-      </c>
-      <c r="G1">
-        <v>-6.2489999999999997</v>
-      </c>
-      <c r="H1">
-        <v>-7.9485854277214001</v>
-      </c>
-      <c r="I1">
-        <v>-9.6077296533960403</v>
-      </c>
-      <c r="J1">
-        <v>-8.8979999999999997</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="D4">
-        <v>-0.86358170086251695</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="D5">
-        <v>-1.4368262739973601</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="D6">
-        <v>-2.4905493340587901</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="D7">
-        <v>-3.855</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="D8">
-        <v>-5.4782042149448502</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="D9">
-        <v>-6.2489999999999997</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="D10">
-        <v>-7.9485854277214001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="D11">
-        <v>-9.6077296533960403</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="D12">
-        <v>-8.8979999999999997</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>

</xml_diff>

<commit_message>
feat: analyse the different dataset sources
</commit_message>
<xml_diff>
--- a/data/proteomics/physiology_collection.xlsx
+++ b/data/proteomics/physiology_collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Documents/GitHub/De-nevo-protein-3D-structure-yeast/data/proteomics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67790435-58F9-4644-8DFA-12F03F5D194D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5CD058E-38E8-0946-888A-DB788D917361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="26880" windowHeight="15220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Supplementary File 1e vip" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$S$1:$S$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$T$1:$T$77</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="116">
   <si>
     <t>sample</t>
   </si>
@@ -372,6 +372,15 @@
   </si>
   <si>
     <t>D=0.027_M</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>sysbio</t>
+  </si>
+  <si>
+    <t>other_lab</t>
   </si>
 </sst>
 </file>
@@ -1364,3385 +1373,3617 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E8F22EE-2E06-6741-B451-D4EA064EAB2E}">
-  <dimension ref="A1:Y77"/>
+  <dimension ref="A1:Z77"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="37.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="21.6640625" customWidth="1"/>
-    <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="22.1640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="28" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="30.5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="23.83203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="26" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="23" customWidth="1"/>
+    <col min="2" max="2" width="32.1640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" customWidth="1"/>
+    <col min="4" max="4" width="22" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="30.5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="26" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="12" customFormat="1">
+    <row r="1" spans="1:26" s="12" customFormat="1">
       <c r="A1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="D1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="E1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="F1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="G1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="H1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="I1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="J1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="K1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="L1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="M1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="12" t="s">
+      <c r="N1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="O1" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="P1" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="Q1" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="Q1" s="12" t="s">
+      <c r="R1" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="R1" s="12" t="s">
+      <c r="S1" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="S1" s="12" t="s">
+      <c r="T1" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="T1" s="12" t="s">
+      <c r="U1" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="U1" s="12" t="s">
+      <c r="V1" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="V1" s="12" t="s">
+      <c r="W1" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="W1" s="12" t="s">
+      <c r="X1" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="X1" s="12" t="s">
+      <c r="Y1" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="Y1" s="12" t="s">
+      <c r="Z1" s="12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:25" s="12" customFormat="1">
+    <row r="2" spans="1:26" s="12" customFormat="1">
       <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="11"/>
-    </row>
-    <row r="3" spans="1:25" s="12" customFormat="1">
+      <c r="B2" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q2" s="11"/>
+    </row>
+    <row r="3" spans="1:26" s="12" customFormat="1">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="P3" s="11"/>
-    </row>
-    <row r="4" spans="1:25" s="12" customFormat="1">
+      <c r="B3" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q3" s="11"/>
+    </row>
+    <row r="4" spans="1:26" s="12" customFormat="1">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="11"/>
-    </row>
-    <row r="5" spans="1:25" s="13" customFormat="1">
+      <c r="B4" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q4" s="11"/>
+    </row>
+    <row r="5" spans="1:26" s="13" customFormat="1">
       <c r="A5" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C5" s="13">
         <v>0.42399999999999999</v>
       </c>
-      <c r="C5" s="13">
+      <c r="D5" s="13">
         <v>18.79</v>
       </c>
-      <c r="I5" s="13">
+      <c r="J5" s="13">
         <v>26.97</v>
       </c>
-      <c r="J5" s="13">
+      <c r="K5" s="13">
         <v>0.56599999999999995</v>
       </c>
-      <c r="K5" s="13">
+      <c r="L5" s="13">
         <v>0.16300000000000001</v>
       </c>
-      <c r="L5" s="13">
+      <c r="M5" s="13">
         <v>3.6499999999999998E-2</v>
       </c>
-      <c r="M5" s="13">
+      <c r="N5" s="13">
         <v>1.4690000000000001</v>
       </c>
-      <c r="N5" s="13">
+      <c r="O5" s="13">
         <v>24.501999999999999</v>
       </c>
-      <c r="O5" s="13">
+      <c r="P5" s="13">
         <v>2.919</v>
       </c>
-      <c r="P5" s="14"/>
-    </row>
-    <row r="6" spans="1:25" s="15" customFormat="1">
+      <c r="Q5" s="14"/>
+    </row>
+    <row r="6" spans="1:26" s="15" customFormat="1">
       <c r="A6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="15">
         <v>0.05</v>
       </c>
-      <c r="C6" s="16">
+      <c r="D6" s="16">
         <v>0.82299999999999995</v>
       </c>
-      <c r="D6" s="16">
+      <c r="E6" s="16">
         <v>0.13100000000000001</v>
       </c>
-      <c r="E6" s="16"/>
       <c r="F6" s="16"/>
       <c r="G6" s="16"/>
-      <c r="H6" s="16">
+      <c r="H6" s="16"/>
+      <c r="I6" s="16">
         <v>0.13100000000000001</v>
       </c>
-      <c r="I6" s="16">
-        <v>0</v>
-      </c>
       <c r="J6" s="16">
         <v>0</v>
       </c>
       <c r="K6" s="16">
+        <v>0</v>
+      </c>
+      <c r="L6" s="16">
         <v>7.2308500000000005E-4</v>
       </c>
-      <c r="L6" s="16">
-        <v>0</v>
-      </c>
       <c r="M6" s="16">
+        <v>0</v>
+      </c>
+      <c r="N6" s="16">
         <v>4.0285879999999996E-3</v>
       </c>
-      <c r="N6" s="16">
+      <c r="O6" s="16">
         <v>2.4449999999999998</v>
       </c>
-      <c r="O6" s="16">
+      <c r="P6" s="16">
         <v>2.3620000000000001</v>
       </c>
-      <c r="P6" s="17">
+      <c r="Q6" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q6" s="15" t="s">
+      <c r="R6" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R6" s="15">
+      <c r="S6" s="15">
         <v>0.5</v>
       </c>
-      <c r="S6" s="15" t="s">
+      <c r="T6" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T6" s="15">
+      <c r="U6" s="15">
         <v>30</v>
       </c>
-      <c r="U6" s="15" t="s">
+      <c r="V6" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V6" s="15">
+      <c r="W6" s="15">
         <v>2.1734E-2</v>
       </c>
-      <c r="W6" s="15">
+      <c r="X6" s="15">
         <v>0.27251471399999999</v>
       </c>
     </row>
-    <row r="7" spans="1:25" s="15" customFormat="1">
+    <row r="7" spans="1:26" s="15" customFormat="1">
       <c r="A7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C7" s="15">
         <v>0.05</v>
       </c>
-      <c r="C7" s="16">
+      <c r="D7" s="16">
         <v>0.70399999999999996</v>
       </c>
-      <c r="D7" s="16">
+      <c r="E7" s="16">
         <v>8.6999999999999994E-2</v>
       </c>
-      <c r="E7" s="16"/>
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
-      <c r="H7" s="16">
+      <c r="H7" s="16"/>
+      <c r="I7" s="16">
         <v>8.6999999999999994E-2</v>
       </c>
-      <c r="I7" s="16">
-        <v>0</v>
-      </c>
       <c r="J7" s="16">
         <v>0</v>
       </c>
       <c r="K7" s="16">
+        <v>0</v>
+      </c>
+      <c r="L7" s="16">
         <v>1.6583900000000001E-4</v>
       </c>
-      <c r="L7" s="16">
-        <v>0</v>
-      </c>
       <c r="M7" s="16">
+        <v>0</v>
+      </c>
+      <c r="N7" s="16">
         <v>6.6796169999999997E-3</v>
       </c>
-      <c r="N7" s="16">
+      <c r="O7" s="16">
         <v>2.105</v>
       </c>
-      <c r="O7" s="16">
+      <c r="P7" s="16">
         <v>2.2759999999999998</v>
       </c>
-      <c r="P7" s="17">
+      <c r="Q7" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q7" s="15" t="s">
+      <c r="R7" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R7" s="15">
+      <c r="S7" s="15">
         <v>0.5</v>
       </c>
-      <c r="S7" s="15" t="s">
+      <c r="T7" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T7" s="15">
+      <c r="U7" s="15">
         <v>30</v>
       </c>
-      <c r="U7" s="15" t="s">
+      <c r="V7" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V7" s="15">
+      <c r="W7" s="15">
         <v>2.4941000000000001E-2</v>
       </c>
-      <c r="W7" s="15">
+      <c r="X7" s="15">
         <v>0.25082010700000001</v>
       </c>
     </row>
-    <row r="8" spans="1:25" s="15" customFormat="1">
+    <row r="8" spans="1:26" s="15" customFormat="1">
       <c r="A8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" s="15">
         <v>0.05</v>
       </c>
-      <c r="C8" s="16">
+      <c r="D8" s="16">
         <v>0.76800000000000002</v>
       </c>
-      <c r="D8" s="16">
+      <c r="E8" s="16">
         <v>0.14000000000000001</v>
       </c>
-      <c r="E8" s="16"/>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
-      <c r="H8" s="16">
+      <c r="H8" s="16"/>
+      <c r="I8" s="16">
         <v>0.14000000000000001</v>
       </c>
-      <c r="I8" s="16">
-        <v>0</v>
-      </c>
       <c r="J8" s="16">
         <v>0</v>
       </c>
       <c r="K8" s="16">
+        <v>0</v>
+      </c>
+      <c r="L8" s="16">
         <v>3.81541E-4</v>
       </c>
-      <c r="L8" s="16">
-        <v>0</v>
-      </c>
       <c r="M8" s="16">
+        <v>0</v>
+      </c>
+      <c r="N8" s="16">
         <v>9.7823159999999992E-3</v>
       </c>
-      <c r="N8" s="16">
+      <c r="O8" s="16">
         <v>2.383</v>
       </c>
-      <c r="O8" s="16">
+      <c r="P8" s="16">
         <v>1.6240000000000001</v>
       </c>
-      <c r="P8" s="17">
+      <c r="Q8" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q8" s="15" t="s">
+      <c r="R8" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R8" s="15">
+      <c r="S8" s="15">
         <v>0.5</v>
       </c>
-      <c r="S8" s="15" t="s">
+      <c r="T8" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T8" s="15">
+      <c r="U8" s="15">
         <v>30</v>
       </c>
-      <c r="U8" s="15" t="s">
+      <c r="V8" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V8" s="15">
+      <c r="W8" s="15">
         <v>2.5831E-2</v>
       </c>
-      <c r="W8" s="15">
+      <c r="X8" s="15">
         <v>0.26109650000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:25" s="15" customFormat="1">
+    <row r="9" spans="1:26" s="15" customFormat="1">
       <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C9" s="15">
         <v>0.1</v>
       </c>
-      <c r="C9" s="16">
+      <c r="D9" s="16">
         <v>1.18</v>
       </c>
-      <c r="D9" s="16">
+      <c r="E9" s="16">
         <v>2.2029999999999998</v>
       </c>
-      <c r="E9" s="16"/>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
-      <c r="H9" s="16">
+      <c r="H9" s="16"/>
+      <c r="I9" s="16">
         <v>2.2029999999999998</v>
       </c>
-      <c r="I9" s="16">
-        <v>0</v>
-      </c>
       <c r="J9" s="16">
         <v>0</v>
       </c>
       <c r="K9" s="16">
+        <v>0</v>
+      </c>
+      <c r="L9" s="16">
         <v>1.2795499999999999E-4</v>
       </c>
-      <c r="L9" s="16">
-        <v>0</v>
-      </c>
       <c r="M9" s="16">
         <v>0</v>
       </c>
       <c r="N9" s="16">
+        <v>0</v>
+      </c>
+      <c r="O9" s="16">
         <v>1.93</v>
       </c>
-      <c r="O9" s="16">
+      <c r="P9" s="16">
         <v>2.44</v>
       </c>
-      <c r="P9" s="17">
+      <c r="Q9" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q9" s="15" t="s">
+      <c r="R9" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R9" s="15">
+      <c r="S9" s="15">
         <v>5</v>
       </c>
-      <c r="S9" s="15" t="s">
+      <c r="T9" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T9" s="15">
+      <c r="U9" s="15">
         <v>3</v>
       </c>
-      <c r="U9" s="15" t="s">
+      <c r="V9" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V9" s="15">
+      <c r="W9" s="15">
         <v>5.3443999999999998E-2</v>
       </c>
-      <c r="W9" s="15">
+      <c r="X9" s="15">
         <v>0.35967375000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:25" s="15" customFormat="1">
+    <row r="10" spans="1:26" s="15" customFormat="1">
       <c r="A10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C10" s="15">
         <v>0.1</v>
       </c>
-      <c r="C10" s="16">
+      <c r="D10" s="16">
         <v>1.127</v>
       </c>
-      <c r="D10" s="16">
+      <c r="E10" s="16">
         <v>2.0979999999999999</v>
       </c>
-      <c r="E10" s="16"/>
       <c r="F10" s="16"/>
       <c r="G10" s="16"/>
-      <c r="H10" s="16">
+      <c r="H10" s="16"/>
+      <c r="I10" s="16">
         <v>2.0979999999999999</v>
       </c>
-      <c r="I10" s="16">
+      <c r="J10" s="16">
         <v>1.6766474999999999E-2</v>
       </c>
-      <c r="J10" s="16">
-        <v>0</v>
-      </c>
       <c r="K10" s="16">
+        <v>0</v>
+      </c>
+      <c r="L10" s="16">
         <v>1.5726999999999999E-4</v>
       </c>
-      <c r="L10" s="16">
-        <v>0</v>
-      </c>
       <c r="M10" s="16">
         <v>0</v>
       </c>
       <c r="N10" s="16">
+        <v>0</v>
+      </c>
+      <c r="O10" s="16">
         <v>2.0699999999999998</v>
       </c>
-      <c r="O10" s="16">
+      <c r="P10" s="16">
         <v>2.39</v>
       </c>
-      <c r="P10" s="17">
+      <c r="Q10" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q10" s="15" t="s">
+      <c r="R10" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R10" s="15">
+      <c r="S10" s="15">
         <v>5</v>
       </c>
-      <c r="S10" s="15" t="s">
+      <c r="T10" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T10" s="15">
+      <c r="U10" s="15">
         <v>3</v>
       </c>
-      <c r="U10" s="15" t="s">
+      <c r="V10" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V10" s="15">
+      <c r="W10" s="15">
         <v>5.0594E-2</v>
       </c>
-      <c r="W10" s="15">
+      <c r="X10" s="15">
         <v>0.377942893</v>
       </c>
     </row>
-    <row r="11" spans="1:25" s="15" customFormat="1">
+    <row r="11" spans="1:26" s="15" customFormat="1">
       <c r="A11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C11" s="15">
         <v>0.1</v>
       </c>
-      <c r="C11" s="16">
+      <c r="D11" s="16">
         <v>1.0980000000000001</v>
       </c>
-      <c r="D11" s="16">
+      <c r="E11" s="16">
         <v>2.0550000000000002</v>
       </c>
-      <c r="E11" s="16"/>
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
-      <c r="H11" s="16">
+      <c r="H11" s="16"/>
+      <c r="I11" s="16">
         <v>2.0550000000000002</v>
       </c>
-      <c r="I11" s="16">
-        <v>0</v>
-      </c>
       <c r="J11" s="16">
         <v>0</v>
       </c>
       <c r="K11" s="16">
+        <v>0</v>
+      </c>
+      <c r="L11" s="16">
         <v>1.3422099999999999E-4</v>
       </c>
-      <c r="L11" s="16">
-        <v>0</v>
-      </c>
       <c r="M11" s="16">
         <v>0</v>
       </c>
       <c r="N11" s="16">
+        <v>0</v>
+      </c>
+      <c r="O11" s="16">
         <v>1.97</v>
       </c>
-      <c r="O11" s="16">
+      <c r="P11" s="16">
         <v>2.1800000000000002</v>
       </c>
-      <c r="P11" s="17">
+      <c r="Q11" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q11" s="15" t="s">
+      <c r="R11" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R11" s="15">
+      <c r="S11" s="15">
         <v>5</v>
       </c>
-      <c r="S11" s="15" t="s">
+      <c r="T11" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T11" s="15">
+      <c r="U11" s="15">
         <v>3</v>
       </c>
-      <c r="U11" s="15" t="s">
+      <c r="V11" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V11" s="15">
+      <c r="W11" s="15">
         <v>4.5962000000000003E-2</v>
       </c>
-      <c r="W11" s="15">
+      <c r="X11" s="15">
         <v>0.33645671399999999</v>
       </c>
     </row>
-    <row r="12" spans="1:25" s="15" customFormat="1">
+    <row r="12" spans="1:26" s="15" customFormat="1">
       <c r="A12" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C12" s="15">
         <v>0.1</v>
       </c>
-      <c r="C12" s="16">
+      <c r="D12" s="16">
         <v>1.51</v>
       </c>
-      <c r="D12" s="16">
+      <c r="E12" s="16">
         <v>0.308</v>
       </c>
-      <c r="E12" s="16"/>
       <c r="F12" s="16"/>
       <c r="G12" s="16"/>
-      <c r="H12" s="16">
+      <c r="H12" s="16"/>
+      <c r="I12" s="16">
         <v>0.308</v>
       </c>
-      <c r="I12" s="16">
-        <v>0</v>
-      </c>
       <c r="J12" s="16">
+        <v>0</v>
+      </c>
+      <c r="K12" s="16">
         <v>7.5614127000000003E-2</v>
       </c>
-      <c r="K12" s="16">
+      <c r="L12" s="16">
         <v>1.7982350000000001E-2</v>
       </c>
-      <c r="L12" s="16">
-        <v>0</v>
-      </c>
       <c r="M12" s="16">
         <v>0</v>
       </c>
       <c r="N12" s="16">
+        <v>0</v>
+      </c>
+      <c r="O12" s="16">
         <v>3.4660000000000002</v>
       </c>
-      <c r="O12" s="16">
+      <c r="P12" s="16">
         <v>3.6160000000000001</v>
       </c>
-      <c r="P12" s="17">
+      <c r="Q12" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q12" s="15" t="s">
+      <c r="R12" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R12" s="15">
+      <c r="S12" s="15">
         <v>0.5</v>
       </c>
-      <c r="S12" s="15" t="s">
+      <c r="T12" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T12" s="15">
+      <c r="U12" s="15">
         <v>30</v>
       </c>
-      <c r="U12" s="15" t="s">
+      <c r="V12" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="V12" s="15">
+      <c r="W12" s="15">
         <v>2.2624999999999999E-2</v>
       </c>
-      <c r="W12" s="15">
+      <c r="X12" s="15">
         <v>0.209333929</v>
       </c>
     </row>
-    <row r="13" spans="1:25" s="15" customFormat="1">
+    <row r="13" spans="1:26" s="15" customFormat="1">
       <c r="A13" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="15">
+      <c r="B13" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C13" s="15">
         <v>0.1</v>
       </c>
-      <c r="C13" s="16">
+      <c r="D13" s="16">
         <v>1.5109999999999999</v>
       </c>
-      <c r="D13" s="16">
+      <c r="E13" s="16">
         <v>0.308</v>
       </c>
-      <c r="E13" s="16"/>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
-      <c r="H13" s="16">
+      <c r="H13" s="16"/>
+      <c r="I13" s="16">
         <v>0.308</v>
       </c>
-      <c r="I13" s="16">
-        <v>0</v>
-      </c>
       <c r="J13" s="16">
+        <v>0</v>
+      </c>
+      <c r="K13" s="16">
         <v>4.9087042999999997E-2</v>
       </c>
-      <c r="K13" s="16">
+      <c r="L13" s="16">
         <v>1.38432E-2</v>
       </c>
-      <c r="L13" s="16">
-        <v>0</v>
-      </c>
       <c r="M13" s="16">
         <v>0</v>
       </c>
       <c r="N13" s="16">
+        <v>0</v>
+      </c>
+      <c r="O13" s="16">
         <v>3.1360000000000001</v>
       </c>
-      <c r="O13" s="16">
+      <c r="P13" s="16">
         <v>3.5219999999999998</v>
       </c>
-      <c r="P13" s="17">
+      <c r="Q13" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q13" s="15" t="s">
+      <c r="R13" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R13" s="15">
+      <c r="S13" s="15">
         <v>0.5</v>
       </c>
-      <c r="S13" s="15" t="s">
+      <c r="T13" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T13" s="15">
+      <c r="U13" s="15">
         <v>30</v>
       </c>
-      <c r="U13" s="15" t="s">
+      <c r="V13" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="V13" s="15">
+      <c r="W13" s="15">
         <v>2.6009999999999998E-2</v>
       </c>
-      <c r="W13" s="15">
+      <c r="X13" s="15">
         <v>0.22151335699999999</v>
       </c>
     </row>
-    <row r="14" spans="1:25" s="15" customFormat="1">
+    <row r="14" spans="1:26" s="15" customFormat="1">
       <c r="A14" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" s="15">
         <v>0.1</v>
       </c>
-      <c r="C14" s="16">
+      <c r="D14" s="16">
         <v>1.4890000000000001</v>
       </c>
-      <c r="D14" s="16">
+      <c r="E14" s="16">
         <v>0.30399999999999999</v>
       </c>
-      <c r="E14" s="16"/>
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
-      <c r="H14" s="16">
+      <c r="H14" s="16"/>
+      <c r="I14" s="16">
         <v>0.30399999999999999</v>
       </c>
-      <c r="I14" s="16">
-        <v>0</v>
-      </c>
       <c r="J14" s="16">
+        <v>0</v>
+      </c>
+      <c r="K14" s="16">
         <v>6.6037847999999996E-2</v>
       </c>
-      <c r="K14" s="16">
+      <c r="L14" s="16">
         <v>1.602926E-2</v>
       </c>
-      <c r="L14" s="16">
-        <v>0</v>
-      </c>
       <c r="M14" s="16">
         <v>0</v>
       </c>
       <c r="N14" s="16">
+        <v>0</v>
+      </c>
+      <c r="O14" s="16">
         <v>3.161</v>
       </c>
-      <c r="O14" s="16">
+      <c r="P14" s="16">
         <v>3.8239999999999998</v>
       </c>
-      <c r="P14" s="17">
+      <c r="Q14" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q14" s="15" t="s">
+      <c r="R14" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R14" s="15">
+      <c r="S14" s="15">
         <v>0.5</v>
       </c>
-      <c r="S14" s="15" t="s">
+      <c r="T14" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T14" s="15">
+      <c r="U14" s="15">
         <v>30</v>
       </c>
-      <c r="U14" s="15" t="s">
+      <c r="V14" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="V14" s="15">
+      <c r="W14" s="15">
         <v>2.7257E-2</v>
       </c>
-      <c r="W14" s="15">
+      <c r="X14" s="15">
         <v>0.24587221400000001</v>
       </c>
     </row>
-    <row r="15" spans="1:25" s="15" customFormat="1">
+    <row r="15" spans="1:26" s="15" customFormat="1">
       <c r="A15" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C15" s="15">
         <v>0.13</v>
       </c>
-      <c r="C15" s="16">
+      <c r="D15" s="16">
         <v>2.0190000000000001</v>
       </c>
-      <c r="D15" s="16">
+      <c r="E15" s="16">
         <v>0.41499999999999998</v>
       </c>
-      <c r="E15" s="16"/>
       <c r="F15" s="16"/>
       <c r="G15" s="16"/>
-      <c r="H15" s="16">
+      <c r="H15" s="16"/>
+      <c r="I15" s="16">
         <v>0.41499999999999998</v>
       </c>
-      <c r="I15" s="16">
+      <c r="J15" s="16">
         <v>0.14387805000000001</v>
       </c>
-      <c r="J15" s="16">
+      <c r="K15" s="16">
         <v>0.23128044</v>
       </c>
-      <c r="K15" s="16">
+      <c r="L15" s="16">
         <v>2.4418572999999999E-2</v>
       </c>
-      <c r="L15" s="16">
+      <c r="M15" s="16">
         <v>7.3894399999999995E-4</v>
       </c>
-      <c r="M15" s="16">
+      <c r="N15" s="16">
         <v>4.2122905000000002E-2</v>
       </c>
-      <c r="N15" s="16">
+      <c r="O15" s="16">
         <v>5.51</v>
       </c>
-      <c r="O15" s="16">
+      <c r="P15" s="16">
         <v>5.2519999999999998</v>
       </c>
-      <c r="P15" s="17">
+      <c r="Q15" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q15" s="15" t="s">
+      <c r="R15" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R15" s="15">
+      <c r="S15" s="15">
         <v>0.5</v>
       </c>
-      <c r="S15" s="15" t="s">
+      <c r="T15" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T15" s="15">
+      <c r="U15" s="15">
         <v>30</v>
       </c>
-      <c r="U15" s="15" t="s">
+      <c r="V15" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V15" s="15">
+      <c r="W15" s="15">
         <v>2.6366000000000001E-2</v>
       </c>
-      <c r="W15" s="15">
+      <c r="X15" s="15">
         <v>0.30372450000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:25" s="15" customFormat="1">
+    <row r="16" spans="1:26" s="15" customFormat="1">
       <c r="A16" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C16" s="15">
         <v>0.13</v>
       </c>
-      <c r="C16" s="16">
+      <c r="D16" s="16">
         <v>2.0590000000000002</v>
       </c>
-      <c r="D16" s="16">
+      <c r="E16" s="16">
         <v>0.42499999999999999</v>
       </c>
-      <c r="E16" s="16"/>
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
-      <c r="H16" s="16">
+      <c r="H16" s="16"/>
+      <c r="I16" s="16">
         <v>0.42499999999999999</v>
       </c>
-      <c r="I16" s="16">
+      <c r="J16" s="16">
         <v>0.13916811300000001</v>
       </c>
-      <c r="J16" s="16">
+      <c r="K16" s="16">
         <v>0.22761730999999999</v>
       </c>
-      <c r="K16" s="16">
+      <c r="L16" s="16">
         <v>2.5077986E-2</v>
       </c>
-      <c r="L16" s="16">
+      <c r="M16" s="16">
         <v>2.152588E-3</v>
       </c>
-      <c r="M16" s="16">
+      <c r="N16" s="16">
         <v>3.3899711999999999E-2</v>
       </c>
-      <c r="N16" s="16">
+      <c r="O16" s="16">
         <v>5.3739999999999997</v>
       </c>
-      <c r="O16" s="16">
+      <c r="P16" s="16">
         <v>4.5460000000000003</v>
       </c>
-      <c r="P16" s="17">
+      <c r="Q16" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q16" s="15" t="s">
+      <c r="R16" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R16" s="15">
+      <c r="S16" s="15">
         <v>0.5</v>
       </c>
-      <c r="S16" s="15" t="s">
+      <c r="T16" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T16" s="15">
+      <c r="U16" s="15">
         <v>30</v>
       </c>
-      <c r="U16" s="15" t="s">
+      <c r="V16" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V16" s="15">
+      <c r="W16" s="15">
         <v>2.5831E-2</v>
       </c>
-      <c r="W16" s="15">
+      <c r="X16" s="15">
         <v>0.25690982099999998</v>
       </c>
     </row>
-    <row r="17" spans="1:24" s="15" customFormat="1">
+    <row r="17" spans="1:25" s="15" customFormat="1">
       <c r="A17" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C17" s="15">
         <v>0.13</v>
       </c>
-      <c r="C17" s="16">
+      <c r="D17" s="16">
         <v>2.1349999999999998</v>
       </c>
-      <c r="D17" s="16">
+      <c r="E17" s="16">
         <v>0.438</v>
       </c>
-      <c r="E17" s="16"/>
       <c r="F17" s="16"/>
       <c r="G17" s="16"/>
-      <c r="H17" s="16">
+      <c r="H17" s="16"/>
+      <c r="I17" s="16">
         <v>0.438</v>
       </c>
-      <c r="I17" s="16">
+      <c r="J17" s="16">
         <v>0.13267562499999999</v>
       </c>
-      <c r="J17" s="16">
+      <c r="K17" s="16">
         <v>0.25727792100000002</v>
       </c>
-      <c r="K17" s="16">
+      <c r="L17" s="16">
         <v>2.6121129999999999E-2</v>
       </c>
-      <c r="L17" s="16">
-        <v>0</v>
-      </c>
       <c r="M17" s="16">
+        <v>0</v>
+      </c>
+      <c r="N17" s="16">
         <v>4.1071206999999998E-2</v>
       </c>
-      <c r="N17" s="16">
+      <c r="O17" s="16">
         <v>5.3019999999999996</v>
       </c>
-      <c r="O17" s="16">
+      <c r="P17" s="16">
         <v>5.07</v>
       </c>
-      <c r="P17" s="17">
+      <c r="Q17" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q17" s="15" t="s">
+      <c r="R17" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R17" s="15">
+      <c r="S17" s="15">
         <v>0.5</v>
       </c>
-      <c r="S17" s="15" t="s">
+      <c r="T17" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T17" s="15">
+      <c r="U17" s="15">
         <v>30</v>
       </c>
-      <c r="U17" s="15" t="s">
+      <c r="V17" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V17" s="15">
+      <c r="W17" s="15">
         <v>2.5297E-2</v>
       </c>
-      <c r="W17" s="15">
+      <c r="X17" s="15">
         <v>0.26642500000000002</v>
       </c>
     </row>
-    <row r="18" spans="1:24" s="15" customFormat="1">
+    <row r="18" spans="1:25" s="15" customFormat="1">
       <c r="A18" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="15">
+      <c r="B18" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C18" s="15">
         <v>0.18</v>
       </c>
-      <c r="C18" s="16">
+      <c r="D18" s="16">
         <v>3.266</v>
       </c>
-      <c r="D18" s="16">
+      <c r="E18" s="16">
         <v>0.66900000000000004</v>
       </c>
-      <c r="E18" s="16"/>
       <c r="F18" s="16"/>
       <c r="G18" s="16"/>
-      <c r="H18" s="16">
+      <c r="H18" s="16"/>
+      <c r="I18" s="16">
         <v>0.66900000000000004</v>
       </c>
-      <c r="I18" s="16">
+      <c r="J18" s="16">
         <v>1.2813869950000001</v>
       </c>
-      <c r="J18" s="16">
+      <c r="K18" s="16">
         <v>0.18048138799999999</v>
       </c>
-      <c r="K18" s="16">
+      <c r="L18" s="16">
         <v>3.2745818000000003E-2</v>
       </c>
-      <c r="L18" s="16">
-        <v>0</v>
-      </c>
       <c r="M18" s="16">
+        <v>0</v>
+      </c>
+      <c r="N18" s="16">
         <v>5.6452840000000004E-3</v>
       </c>
-      <c r="N18" s="16">
+      <c r="O18" s="16">
         <v>7.2619999999999996</v>
       </c>
-      <c r="O18" s="16">
+      <c r="P18" s="16">
         <v>5.42</v>
       </c>
-      <c r="P18" s="17">
+      <c r="Q18" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q18" s="15" t="s">
+      <c r="R18" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R18" s="15">
+      <c r="S18" s="15">
         <v>0.5</v>
       </c>
-      <c r="S18" s="15" t="s">
+      <c r="T18" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T18" s="15">
+      <c r="U18" s="15">
         <v>30</v>
       </c>
-      <c r="U18" s="15" t="s">
+      <c r="V18" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V18" s="15">
+      <c r="W18" s="15">
         <v>3.9014E-2</v>
       </c>
-      <c r="W18" s="15">
+      <c r="X18" s="15">
         <v>0.28926142900000001</v>
       </c>
     </row>
-    <row r="19" spans="1:24" s="15" customFormat="1">
+    <row r="19" spans="1:25" s="15" customFormat="1">
       <c r="A19" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="15">
+      <c r="B19" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C19" s="15">
         <v>0.18</v>
       </c>
-      <c r="C19" s="16">
+      <c r="D19" s="16">
         <v>3.202</v>
       </c>
-      <c r="D19" s="16">
+      <c r="E19" s="16">
         <v>0.65900000000000003</v>
       </c>
-      <c r="E19" s="16"/>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
-      <c r="H19" s="16">
+      <c r="H19" s="16"/>
+      <c r="I19" s="16">
         <v>0.65900000000000003</v>
       </c>
-      <c r="I19" s="16">
+      <c r="J19" s="16">
         <v>1.4870797280000001</v>
       </c>
-      <c r="J19" s="16">
+      <c r="K19" s="16">
         <v>0.41515672300000001</v>
       </c>
-      <c r="K19" s="16">
+      <c r="L19" s="16">
         <v>3.1272250000000001E-2</v>
       </c>
-      <c r="L19" s="16">
+      <c r="M19" s="16">
         <v>2.6969479999999998E-3</v>
       </c>
-      <c r="M19" s="16">
+      <c r="N19" s="16">
         <v>1.6418242E-2</v>
       </c>
-      <c r="N19" s="16">
+      <c r="O19" s="16">
         <v>7.3049999999999997</v>
       </c>
-      <c r="O19" s="16">
+      <c r="P19" s="16">
         <v>6.0170000000000003</v>
       </c>
-      <c r="P19" s="17">
+      <c r="Q19" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q19" s="15" t="s">
+      <c r="R19" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R19" s="15">
+      <c r="S19" s="15">
         <v>0.5</v>
       </c>
-      <c r="S19" s="15" t="s">
+      <c r="T19" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T19" s="15">
+      <c r="U19" s="15">
         <v>30</v>
       </c>
-      <c r="U19" s="15" t="s">
+      <c r="V19" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V19" s="15">
+      <c r="W19" s="15">
         <v>3.8657999999999998E-2</v>
       </c>
-      <c r="W19" s="15">
+      <c r="X19" s="15">
         <v>0.28202989299999998</v>
       </c>
     </row>
-    <row r="20" spans="1:24" s="15" customFormat="1">
+    <row r="20" spans="1:25" s="15" customFormat="1">
       <c r="A20" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="15">
+      <c r="B20" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C20" s="15">
         <v>0.18</v>
       </c>
-      <c r="C20" s="16">
+      <c r="D20" s="16">
         <v>2.83</v>
       </c>
-      <c r="D20" s="16">
+      <c r="E20" s="16">
         <v>0.58099999999999996</v>
       </c>
-      <c r="E20" s="16"/>
       <c r="F20" s="16"/>
       <c r="G20" s="16"/>
-      <c r="H20" s="16">
+      <c r="H20" s="16"/>
+      <c r="I20" s="16">
         <v>0.58099999999999996</v>
       </c>
-      <c r="I20" s="16">
+      <c r="J20" s="16">
         <v>1.069367508</v>
       </c>
-      <c r="J20" s="16">
+      <c r="K20" s="16">
         <v>0.18424942899999999</v>
       </c>
-      <c r="K20" s="16">
+      <c r="L20" s="16">
         <v>2.652065E-2</v>
       </c>
-      <c r="L20" s="16">
-        <v>0</v>
-      </c>
       <c r="M20" s="16">
+        <v>0</v>
+      </c>
+      <c r="N20" s="16">
         <v>1.5674206999999999E-2</v>
       </c>
-      <c r="N20" s="16">
+      <c r="O20" s="16">
         <v>6.2510000000000003</v>
       </c>
-      <c r="O20" s="16">
+      <c r="P20" s="16">
         <v>5.2640000000000002</v>
       </c>
-      <c r="P20" s="17">
+      <c r="Q20" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q20" s="15" t="s">
+      <c r="R20" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R20" s="15">
+      <c r="S20" s="15">
         <v>0.5</v>
       </c>
-      <c r="S20" s="15" t="s">
+      <c r="T20" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T20" s="15">
+      <c r="U20" s="15">
         <v>30</v>
       </c>
-      <c r="U20" s="15" t="s">
+      <c r="V20" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V20" s="15">
+      <c r="W20" s="15">
         <v>3.7945E-2</v>
       </c>
-      <c r="W20" s="15">
+      <c r="X20" s="15">
         <v>0.288119607</v>
       </c>
     </row>
-    <row r="21" spans="1:24" s="15" customFormat="1">
+    <row r="21" spans="1:25" s="15" customFormat="1">
       <c r="A21" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B21" s="15">
+      <c r="B21" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C21" s="15">
         <v>0.3</v>
       </c>
-      <c r="C21" s="16">
+      <c r="D21" s="16">
         <v>7.9909999999999997</v>
       </c>
-      <c r="D21" s="16">
+      <c r="E21" s="16">
         <v>1.6479999999999999</v>
       </c>
-      <c r="E21" s="16"/>
       <c r="F21" s="16"/>
       <c r="G21" s="16"/>
-      <c r="H21" s="16">
+      <c r="H21" s="16"/>
+      <c r="I21" s="16">
         <v>1.6479999999999999</v>
       </c>
-      <c r="I21" s="16">
+      <c r="J21" s="16">
         <v>7.0441347099999998</v>
       </c>
-      <c r="J21" s="16">
+      <c r="K21" s="16">
         <v>0.31251037799999998</v>
       </c>
-      <c r="K21" s="16">
+      <c r="L21" s="16">
         <v>5.1692219999999997E-2</v>
       </c>
-      <c r="L21" s="16">
+      <c r="M21" s="16">
         <v>1.1339925000000001E-2</v>
       </c>
-      <c r="M21" s="16">
-        <v>0</v>
-      </c>
       <c r="N21" s="16">
+        <v>0</v>
+      </c>
+      <c r="O21" s="16">
         <v>14.086</v>
       </c>
-      <c r="O21" s="16">
+      <c r="P21" s="16">
         <v>8.3010000000000002</v>
       </c>
-      <c r="P21" s="17">
+      <c r="Q21" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q21" s="15" t="s">
+      <c r="R21" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R21" s="15">
+      <c r="S21" s="15">
         <v>0.5</v>
       </c>
-      <c r="S21" s="15" t="s">
+      <c r="T21" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T21" s="15">
+      <c r="U21" s="15">
         <v>30</v>
       </c>
-      <c r="U21" s="15" t="s">
+      <c r="V21" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V21" s="15">
+      <c r="W21" s="15">
         <v>4.7031000000000003E-2</v>
       </c>
-      <c r="W21" s="15">
+      <c r="X21" s="15">
         <v>0.42247392900000003</v>
       </c>
     </row>
-    <row r="22" spans="1:24" s="15" customFormat="1">
+    <row r="22" spans="1:25" s="15" customFormat="1">
       <c r="A22" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C22" s="15">
         <v>0.3</v>
       </c>
-      <c r="C22" s="16">
+      <c r="D22" s="16">
         <v>8.2759999999999998</v>
       </c>
-      <c r="D22" s="16">
+      <c r="E22" s="16">
         <v>1.6950000000000001</v>
       </c>
-      <c r="E22" s="16"/>
       <c r="F22" s="16"/>
       <c r="G22" s="16"/>
-      <c r="H22" s="16">
+      <c r="H22" s="16"/>
+      <c r="I22" s="16">
         <v>1.6950000000000001</v>
       </c>
-      <c r="I22" s="16">
+      <c r="J22" s="16">
         <v>6.6847254490000001</v>
       </c>
-      <c r="J22" s="16">
+      <c r="K22" s="16">
         <v>0.27229536399999998</v>
       </c>
-      <c r="K22" s="16">
+      <c r="L22" s="16">
         <v>4.4478275999999997E-2</v>
       </c>
-      <c r="L22" s="16">
+      <c r="M22" s="16">
         <v>3.4668667E-2</v>
       </c>
-      <c r="M22" s="16">
-        <v>0</v>
-      </c>
       <c r="N22" s="16">
+        <v>0</v>
+      </c>
+      <c r="O22" s="16">
         <v>15.111000000000001</v>
       </c>
-      <c r="O22" s="16">
+      <c r="P22" s="16">
         <v>8.3870000000000005</v>
       </c>
-      <c r="P22" s="17">
+      <c r="Q22" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q22" s="15" t="s">
+      <c r="R22" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R22" s="15">
+      <c r="S22" s="15">
         <v>0.5</v>
       </c>
-      <c r="S22" s="15" t="s">
+      <c r="T22" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T22" s="15">
+      <c r="U22" s="15">
         <v>30</v>
       </c>
-      <c r="U22" s="15" t="s">
+      <c r="V22" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V22" s="15">
+      <c r="W22" s="15">
         <v>4.5606000000000001E-2</v>
       </c>
-      <c r="W22" s="15">
+      <c r="X22" s="15">
         <v>0.42133210700000001</v>
       </c>
     </row>
-    <row r="23" spans="1:24" s="15" customFormat="1">
+    <row r="23" spans="1:25" s="15" customFormat="1">
       <c r="A23" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C23" s="15">
         <v>0.3</v>
       </c>
-      <c r="C23" s="16">
+      <c r="D23" s="16">
         <v>8.9320000000000004</v>
       </c>
-      <c r="D23" s="16">
+      <c r="E23" s="16">
         <v>1.8660000000000001</v>
       </c>
-      <c r="E23" s="16"/>
       <c r="F23" s="16"/>
       <c r="G23" s="16"/>
-      <c r="H23" s="16">
+      <c r="H23" s="16"/>
+      <c r="I23" s="16">
         <v>1.8660000000000001</v>
       </c>
-      <c r="I23" s="16">
+      <c r="J23" s="16">
         <v>8.2124218889999998</v>
       </c>
-      <c r="J23" s="16">
+      <c r="K23" s="16">
         <v>0.61718923199999998</v>
       </c>
-      <c r="K23" s="16">
+      <c r="L23" s="16">
         <v>6.4337543999999997E-2</v>
       </c>
-      <c r="L23" s="16">
+      <c r="M23" s="16">
         <v>2.9481279999999999E-2</v>
       </c>
-      <c r="M23" s="16">
-        <v>0</v>
-      </c>
       <c r="N23" s="16">
+        <v>0</v>
+      </c>
+      <c r="O23" s="16">
         <v>16.956</v>
       </c>
-      <c r="O23" s="16">
+      <c r="P23" s="16">
         <v>9.34</v>
       </c>
-      <c r="P23" s="17">
+      <c r="Q23" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q23" s="15" t="s">
+      <c r="R23" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R23" s="15">
+      <c r="S23" s="15">
         <v>0.5</v>
       </c>
-      <c r="S23" s="15" t="s">
+      <c r="T23" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T23" s="15">
+      <c r="U23" s="15">
         <v>30</v>
       </c>
-      <c r="U23" s="15" t="s">
+      <c r="V23" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V23" s="15">
+      <c r="W23" s="15">
         <v>5.2019000000000003E-2</v>
       </c>
-      <c r="W23" s="15">
+      <c r="X23" s="15">
         <v>0.39963749999999998</v>
       </c>
     </row>
-    <row r="24" spans="1:24" s="15" customFormat="1">
+    <row r="24" spans="1:25" s="15" customFormat="1">
       <c r="A24" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" s="15">
         <v>0.35</v>
       </c>
-      <c r="C24" s="16">
+      <c r="D24" s="16">
         <v>12.936999999999999</v>
       </c>
-      <c r="D24" s="16">
+      <c r="E24" s="16">
         <v>2.7120000000000002</v>
       </c>
-      <c r="E24" s="16"/>
       <c r="F24" s="16"/>
       <c r="G24" s="16"/>
-      <c r="H24" s="16">
+      <c r="H24" s="16"/>
+      <c r="I24" s="16">
         <v>2.7120000000000002</v>
       </c>
-      <c r="I24" s="16">
+      <c r="J24" s="16">
         <v>11.927306959999999</v>
       </c>
-      <c r="J24" s="16">
+      <c r="K24" s="16">
         <v>0.47269426599999997</v>
       </c>
-      <c r="K24" s="16">
+      <c r="L24" s="16">
         <v>8.9757966999999994E-2</v>
       </c>
-      <c r="L24" s="16">
+      <c r="M24" s="16">
         <v>3.5944587E-2</v>
       </c>
-      <c r="M24" s="16">
-        <v>0</v>
-      </c>
       <c r="N24" s="16">
+        <v>0</v>
+      </c>
+      <c r="O24" s="16">
         <v>20.902000000000001</v>
       </c>
-      <c r="O24" s="16">
+      <c r="P24" s="16">
         <v>12.682</v>
       </c>
-      <c r="P24" s="17">
+      <c r="Q24" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q24" s="15" t="s">
+      <c r="R24" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R24" s="15">
+      <c r="S24" s="15">
         <v>0.5</v>
       </c>
-      <c r="S24" s="15" t="s">
+      <c r="T24" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T24" s="15">
+      <c r="U24" s="15">
         <v>30</v>
       </c>
-      <c r="U24" s="15" t="s">
+      <c r="V24" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V24" s="15">
+      <c r="W24" s="15">
         <v>7.3219000000000006E-2</v>
       </c>
-      <c r="W24" s="15">
+      <c r="X24" s="15">
         <v>0.48415467400000001</v>
       </c>
     </row>
-    <row r="25" spans="1:24" s="15" customFormat="1">
+    <row r="25" spans="1:25" s="15" customFormat="1">
       <c r="A25" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="15">
+      <c r="B25" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" s="15">
         <v>0.35</v>
       </c>
-      <c r="C25" s="16">
+      <c r="D25" s="16">
         <v>13.23</v>
       </c>
-      <c r="D25" s="16">
+      <c r="E25" s="16">
         <v>2.786</v>
       </c>
-      <c r="E25" s="16"/>
       <c r="F25" s="16"/>
       <c r="G25" s="16"/>
-      <c r="H25" s="16">
+      <c r="H25" s="16"/>
+      <c r="I25" s="16">
         <v>2.786</v>
       </c>
-      <c r="I25" s="16">
+      <c r="J25" s="16">
         <v>12.12470377</v>
       </c>
-      <c r="J25" s="16">
+      <c r="K25" s="16">
         <v>0.63692599999999999</v>
       </c>
-      <c r="K25" s="16">
+      <c r="L25" s="16">
         <v>0.104193063</v>
       </c>
-      <c r="L25" s="16">
+      <c r="M25" s="16">
         <v>3.3770889999999998E-2</v>
       </c>
-      <c r="M25" s="16">
-        <v>0</v>
-      </c>
       <c r="N25" s="16">
+        <v>0</v>
+      </c>
+      <c r="O25" s="16">
         <v>21.082999999999998</v>
       </c>
-      <c r="O25" s="16">
+      <c r="P25" s="16">
         <v>12.353999999999999</v>
       </c>
-      <c r="P25" s="17">
+      <c r="Q25" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q25" s="15" t="s">
+      <c r="R25" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R25" s="15">
+      <c r="S25" s="15">
         <v>0.5</v>
       </c>
-      <c r="S25" s="15" t="s">
+      <c r="T25" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T25" s="15">
+      <c r="U25" s="15">
         <v>30</v>
       </c>
-      <c r="U25" s="15" t="s">
+      <c r="V25" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V25" s="15">
+      <c r="W25" s="15">
         <v>7.0545999999999998E-2</v>
       </c>
-      <c r="W25" s="15">
+      <c r="X25" s="15">
         <v>0.48992198300000001</v>
       </c>
     </row>
-    <row r="26" spans="1:24" s="15" customFormat="1">
+    <row r="26" spans="1:25" s="15" customFormat="1">
       <c r="A26" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="15">
+      <c r="B26" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C26" s="15">
         <v>0.35</v>
       </c>
-      <c r="C26" s="16">
+      <c r="D26" s="16">
         <v>13.096</v>
       </c>
-      <c r="D26" s="16">
+      <c r="E26" s="16">
         <v>2.742</v>
       </c>
-      <c r="E26" s="16"/>
       <c r="F26" s="16"/>
       <c r="G26" s="16"/>
-      <c r="H26" s="16">
+      <c r="H26" s="16"/>
+      <c r="I26" s="16">
         <v>2.742</v>
       </c>
-      <c r="I26" s="16">
+      <c r="J26" s="16">
         <v>11.84780602</v>
       </c>
-      <c r="J26" s="16">
+      <c r="K26" s="16">
         <v>0.47734259699999998</v>
       </c>
-      <c r="K26" s="16">
+      <c r="L26" s="16">
         <v>9.1823417000000004E-2</v>
       </c>
-      <c r="L26" s="16">
-        <v>0</v>
-      </c>
       <c r="M26" s="16">
         <v>0</v>
       </c>
       <c r="N26" s="16">
+        <v>0</v>
+      </c>
+      <c r="O26" s="16">
         <v>21.097999999999999</v>
       </c>
-      <c r="O26" s="16">
+      <c r="P26" s="16">
         <v>12.977</v>
       </c>
-      <c r="P26" s="17">
+      <c r="Q26" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q26" s="15" t="s">
+      <c r="R26" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="R26" s="15">
+      <c r="S26" s="15">
         <v>0.5</v>
       </c>
-      <c r="S26" s="15" t="s">
+      <c r="T26" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T26" s="15">
+      <c r="U26" s="15">
         <v>30</v>
       </c>
-      <c r="U26" s="15" t="s">
+      <c r="V26" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="V26" s="15">
+      <c r="W26" s="15">
         <v>8.8717000000000004E-2</v>
       </c>
-      <c r="W26" s="15">
+      <c r="X26" s="15">
         <v>0.50886425499999999</v>
       </c>
     </row>
-    <row r="27" spans="1:24" s="15" customFormat="1">
+    <row r="27" spans="1:25" s="15" customFormat="1">
       <c r="A27" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="15">
+      <c r="B27" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C27" s="15">
         <v>0.1</v>
       </c>
-      <c r="C27" s="16">
+      <c r="D27" s="16">
         <v>0.82699999999999996</v>
       </c>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16">
+      <c r="E27" s="16"/>
+      <c r="F27" s="16">
         <v>0.747</v>
       </c>
-      <c r="F27" s="16"/>
       <c r="G27" s="16"/>
-      <c r="H27" s="16">
+      <c r="H27" s="16"/>
+      <c r="I27" s="16">
         <v>1.4930000000000001</v>
       </c>
-      <c r="I27" s="16">
-        <v>0</v>
-      </c>
       <c r="J27" s="16">
         <v>0</v>
       </c>
       <c r="K27" s="16">
+        <v>0</v>
+      </c>
+      <c r="L27" s="16">
         <v>8.7561730000000008E-3</v>
       </c>
-      <c r="L27" s="16">
-        <v>0</v>
-      </c>
       <c r="M27" s="16">
         <v>0</v>
       </c>
       <c r="N27" s="16">
+        <v>0</v>
+      </c>
+      <c r="O27" s="16">
         <v>2.7690000000000001</v>
       </c>
-      <c r="O27" s="16">
+      <c r="P27" s="16">
         <v>2.4500000000000002</v>
       </c>
-      <c r="P27" s="17">
+      <c r="Q27" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q27" s="15" t="s">
+      <c r="R27" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="R27" s="15">
+      <c r="S27" s="15">
         <v>5.53</v>
       </c>
-      <c r="S27" s="15" t="s">
+      <c r="T27" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T27" s="15">
+      <c r="U27" s="15">
         <v>5</v>
       </c>
-      <c r="U27" s="15" t="s">
+      <c r="V27" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V27" s="15">
+      <c r="W27" s="15">
         <v>7.1259000000000003E-2</v>
       </c>
-      <c r="W27" s="15">
+      <c r="X27" s="15">
         <v>0.49783414300000001</v>
       </c>
-      <c r="X27" s="15" t="s">
+      <c r="Y27" s="15" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="28" spans="1:24" s="15" customFormat="1">
+    <row r="28" spans="1:25" s="15" customFormat="1">
       <c r="A28" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B28" s="15">
+      <c r="B28" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C28" s="15">
         <v>0.1</v>
       </c>
-      <c r="C28" s="16">
+      <c r="D28" s="16">
         <v>0.78800000000000003</v>
       </c>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16">
+      <c r="E28" s="16"/>
+      <c r="F28" s="16">
         <v>0.71199999999999997</v>
       </c>
-      <c r="F28" s="16"/>
       <c r="G28" s="16"/>
-      <c r="H28" s="16">
+      <c r="H28" s="16"/>
+      <c r="I28" s="16">
         <v>1.423</v>
       </c>
-      <c r="I28" s="16">
-        <v>0</v>
-      </c>
       <c r="J28" s="16">
         <v>0</v>
       </c>
       <c r="K28" s="16">
+        <v>0</v>
+      </c>
+      <c r="L28" s="16">
         <v>5.5182690000000001E-3</v>
       </c>
-      <c r="L28" s="16">
-        <v>0</v>
-      </c>
       <c r="M28" s="16">
         <v>0</v>
       </c>
       <c r="N28" s="16">
+        <v>0</v>
+      </c>
+      <c r="O28" s="16">
         <v>2.7170000000000001</v>
       </c>
-      <c r="O28" s="16">
+      <c r="P28" s="16">
         <v>2.3530000000000002</v>
       </c>
-      <c r="P28" s="17">
+      <c r="Q28" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q28" s="15" t="s">
+      <c r="R28" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="R28" s="15">
+      <c r="S28" s="15">
         <v>5.53</v>
       </c>
-      <c r="S28" s="15" t="s">
+      <c r="T28" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T28" s="15">
+      <c r="U28" s="15">
         <v>5</v>
       </c>
-      <c r="U28" s="15" t="s">
+      <c r="V28" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V28" s="15">
+      <c r="W28" s="15">
         <v>5.8789000000000001E-2</v>
       </c>
-      <c r="W28" s="15">
+      <c r="X28" s="15">
         <v>0.58385135700000002</v>
       </c>
-      <c r="X28" s="15" t="s">
+      <c r="Y28" s="15" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="29" spans="1:24" s="15" customFormat="1">
+    <row r="29" spans="1:25" s="15" customFormat="1">
       <c r="A29" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B29" s="15">
+      <c r="B29" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C29" s="15">
         <v>0.1</v>
       </c>
-      <c r="C29" s="16">
+      <c r="D29" s="16">
         <v>0.76700000000000002</v>
       </c>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16">
+      <c r="E29" s="16"/>
+      <c r="F29" s="16">
         <v>0.69099999999999995</v>
       </c>
-      <c r="F29" s="16"/>
       <c r="G29" s="16"/>
-      <c r="H29" s="16">
+      <c r="H29" s="16"/>
+      <c r="I29" s="16">
         <v>1.3819999999999999</v>
       </c>
-      <c r="I29" s="16">
-        <v>0</v>
-      </c>
       <c r="J29" s="16">
         <v>0</v>
       </c>
       <c r="K29" s="16">
+        <v>0</v>
+      </c>
+      <c r="L29" s="16">
         <v>1.9902549999999998E-3</v>
       </c>
-      <c r="L29" s="16">
-        <v>0</v>
-      </c>
       <c r="M29" s="16">
         <v>0</v>
       </c>
       <c r="N29" s="16">
+        <v>0</v>
+      </c>
+      <c r="O29" s="16">
         <v>2.5739999999999998</v>
       </c>
-      <c r="O29" s="16">
+      <c r="P29" s="16">
         <v>2.25</v>
       </c>
-      <c r="P29" s="17">
+      <c r="Q29" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q29" s="15" t="s">
+      <c r="R29" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="R29" s="15">
+      <c r="S29" s="15">
         <v>5.53</v>
       </c>
-      <c r="S29" s="15" t="s">
+      <c r="T29" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T29" s="15">
+      <c r="U29" s="15">
         <v>5</v>
       </c>
-      <c r="U29" s="15" t="s">
+      <c r="V29" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V29" s="15">
+      <c r="W29" s="15">
         <v>6.4132999999999996E-2</v>
       </c>
-      <c r="W29" s="15">
+      <c r="X29" s="15">
         <v>0.59412774999999995</v>
       </c>
-      <c r="X29" s="15" t="s">
+      <c r="Y29" s="15" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="30" spans="1:24" s="15" customFormat="1">
+    <row r="30" spans="1:25" s="15" customFormat="1">
       <c r="A30" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B30" s="15">
+      <c r="B30" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C30" s="15">
         <v>0.1</v>
       </c>
-      <c r="C30" s="16">
+      <c r="D30" s="16">
         <v>0.80700000000000005</v>
       </c>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16">
+      <c r="E30" s="16"/>
+      <c r="F30" s="16">
         <v>4.92</v>
       </c>
-      <c r="F30" s="16"/>
       <c r="G30" s="16"/>
-      <c r="H30" s="16">
+      <c r="H30" s="16"/>
+      <c r="I30" s="16">
         <v>9.8390000000000004</v>
       </c>
-      <c r="I30" s="16">
-        <v>0</v>
-      </c>
       <c r="J30" s="16">
         <v>0</v>
       </c>
       <c r="K30" s="16">
+        <v>0</v>
+      </c>
+      <c r="L30" s="16">
         <v>3.9436786000000001E-2</v>
       </c>
-      <c r="L30" s="16">
-        <v>0</v>
-      </c>
       <c r="M30" s="16">
+        <v>0</v>
+      </c>
+      <c r="N30" s="16">
         <v>1.3630471999999999E-2</v>
       </c>
-      <c r="N30" s="16">
+      <c r="O30" s="16">
         <v>3.032</v>
       </c>
-      <c r="O30" s="16">
+      <c r="P30" s="16">
         <v>1.7749999999999999</v>
       </c>
-      <c r="P30" s="17">
+      <c r="Q30" s="17">
         <v>1.21</v>
       </c>
-      <c r="Q30" s="15" t="s">
+      <c r="R30" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="R30" s="15">
+      <c r="S30" s="15">
         <v>5.53</v>
       </c>
-      <c r="S30" s="15" t="s">
+      <c r="T30" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T30" s="15">
+      <c r="U30" s="15">
         <v>3</v>
       </c>
-      <c r="U30" s="15" t="s">
+      <c r="V30" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V30" s="15">
+      <c r="W30" s="15">
         <v>5.5581999999999999E-2</v>
       </c>
-      <c r="W30" s="15">
+      <c r="X30" s="15">
         <v>0.510013571</v>
       </c>
-      <c r="X30" s="15" t="s">
+      <c r="Y30" s="15" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="31" spans="1:24" s="15" customFormat="1">
+    <row r="31" spans="1:25" s="15" customFormat="1">
       <c r="A31" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B31" s="15">
+      <c r="B31" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C31" s="15">
         <v>0.1</v>
       </c>
-      <c r="C31" s="16">
+      <c r="D31" s="16">
         <v>0.64900000000000002</v>
       </c>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16">
+      <c r="E31" s="16"/>
+      <c r="F31" s="16">
         <v>3.9620000000000002</v>
       </c>
-      <c r="F31" s="16"/>
       <c r="G31" s="16"/>
-      <c r="H31" s="16">
+      <c r="H31" s="16"/>
+      <c r="I31" s="16">
         <v>7.9240000000000004</v>
       </c>
-      <c r="I31" s="16">
-        <v>0</v>
-      </c>
       <c r="J31" s="16">
         <v>0</v>
       </c>
       <c r="K31" s="16">
+        <v>0</v>
+      </c>
+      <c r="L31" s="16">
         <v>3.0460814999999999E-2</v>
       </c>
-      <c r="L31" s="16">
-        <v>0</v>
-      </c>
       <c r="M31" s="16">
+        <v>0</v>
+      </c>
+      <c r="N31" s="16">
         <v>9.5061450000000006E-3</v>
       </c>
-      <c r="N31" s="16">
+      <c r="O31" s="16">
         <v>1.9590000000000001</v>
       </c>
-      <c r="O31" s="16">
+      <c r="P31" s="16">
         <v>1.623</v>
       </c>
-      <c r="P31" s="17">
+      <c r="Q31" s="17">
         <v>1.21</v>
       </c>
-      <c r="Q31" s="15" t="s">
+      <c r="R31" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="R31" s="15">
+      <c r="S31" s="15">
         <v>5.53</v>
       </c>
-      <c r="S31" s="15" t="s">
+      <c r="T31" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T31" s="15">
+      <c r="U31" s="15">
         <v>3</v>
       </c>
-      <c r="U31" s="15" t="s">
+      <c r="V31" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V31" s="15">
+      <c r="W31" s="15">
         <v>5.4869000000000001E-2</v>
       </c>
-      <c r="W31" s="15">
+      <c r="X31" s="15">
         <v>0.29420932100000002</v>
       </c>
-      <c r="X31" s="15" t="s">
+      <c r="Y31" s="15" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="32" spans="1:24" s="15" customFormat="1">
+    <row r="32" spans="1:25" s="15" customFormat="1">
       <c r="A32" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B32" s="15">
+      <c r="B32" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C32" s="15">
         <v>0.1</v>
       </c>
-      <c r="C32" s="16">
+      <c r="D32" s="16">
         <v>0.76500000000000001</v>
       </c>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16">
+      <c r="E32" s="16"/>
+      <c r="F32" s="16">
         <v>4.6159999999999997</v>
       </c>
-      <c r="F32" s="16"/>
       <c r="G32" s="16"/>
-      <c r="H32" s="16">
+      <c r="H32" s="16"/>
+      <c r="I32" s="16">
         <v>9.2319999999999993</v>
       </c>
-      <c r="I32" s="16">
-        <v>0</v>
-      </c>
       <c r="J32" s="16">
         <v>0</v>
       </c>
       <c r="K32" s="16">
+        <v>0</v>
+      </c>
+      <c r="L32" s="16">
         <v>2.5119712999999998E-2</v>
       </c>
-      <c r="L32" s="16">
-        <v>0</v>
-      </c>
       <c r="M32" s="16">
         <v>0</v>
       </c>
       <c r="N32" s="16">
+        <v>0</v>
+      </c>
+      <c r="O32" s="16">
         <v>2.569</v>
       </c>
-      <c r="O32" s="16">
+      <c r="P32" s="16">
         <v>1.2909999999999999</v>
       </c>
-      <c r="P32" s="17">
+      <c r="Q32" s="17">
         <v>1.21</v>
       </c>
-      <c r="Q32" s="15" t="s">
+      <c r="R32" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="R32" s="15">
+      <c r="S32" s="15">
         <v>5.53</v>
       </c>
-      <c r="S32" s="15" t="s">
+      <c r="T32" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T32" s="15">
+      <c r="U32" s="15">
         <v>3</v>
       </c>
-      <c r="U32" s="15" t="s">
+      <c r="V32" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V32" s="15">
+      <c r="W32" s="15">
         <v>5.1663000000000001E-2</v>
       </c>
-      <c r="W32" s="15">
+      <c r="X32" s="15">
         <v>0.358912536</v>
       </c>
-      <c r="X32" s="15" t="s">
+      <c r="Y32" s="15" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="33" spans="1:23" s="15" customFormat="1">
+    <row r="33" spans="1:24" s="15" customFormat="1">
       <c r="A33" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B33" s="15">
+      <c r="B33" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C33" s="15">
         <v>0.1</v>
       </c>
-      <c r="C33" s="16">
+      <c r="D33" s="16">
         <v>1.381</v>
       </c>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16">
+      <c r="E33" s="16"/>
+      <c r="F33" s="16">
         <v>0.158</v>
       </c>
-      <c r="F33" s="16"/>
       <c r="G33" s="16"/>
-      <c r="H33" s="16">
+      <c r="H33" s="16"/>
+      <c r="I33" s="16">
         <v>0.317</v>
       </c>
-      <c r="I33" s="16">
+      <c r="J33" s="16">
         <v>1.8073279000000001E-2</v>
       </c>
-      <c r="J33" s="16">
+      <c r="K33" s="16">
         <v>7.8381013999999999E-2</v>
       </c>
-      <c r="K33" s="16">
+      <c r="L33" s="16">
         <v>0.86713414300000002</v>
       </c>
-      <c r="L33" s="16">
+      <c r="M33" s="16">
         <v>5.4564440000000004E-3</v>
       </c>
-      <c r="M33" s="16">
+      <c r="N33" s="16">
         <v>4.6616212999999997E-2</v>
       </c>
-      <c r="N33" s="16">
+      <c r="O33" s="16">
         <v>4.3209999999999997</v>
       </c>
-      <c r="O33" s="16">
+      <c r="P33" s="16">
         <v>3.883</v>
       </c>
-      <c r="P33" s="17">
+      <c r="Q33" s="17">
         <v>6.87</v>
       </c>
-      <c r="Q33" s="15" t="s">
+      <c r="R33" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="R33" s="15">
+      <c r="S33" s="15">
         <v>0.55000000000000004</v>
       </c>
-      <c r="S33" s="15" t="s">
+      <c r="T33" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T33" s="15">
+      <c r="U33" s="15">
         <v>30</v>
       </c>
-      <c r="U33" s="15" t="s">
+      <c r="V33" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V33" s="15">
+      <c r="W33" s="15">
         <v>2.6366000000000001E-2</v>
       </c>
-      <c r="W33" s="15">
+      <c r="X33" s="15">
         <v>0.20552785700000001</v>
       </c>
     </row>
-    <row r="34" spans="1:23" s="15" customFormat="1">
+    <row r="34" spans="1:24" s="15" customFormat="1">
       <c r="A34" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B34" s="15">
+      <c r="B34" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C34" s="15">
         <v>0.1</v>
       </c>
-      <c r="C34" s="16">
+      <c r="D34" s="16">
         <v>1.2589999999999999</v>
       </c>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16">
+      <c r="E34" s="16"/>
+      <c r="F34" s="16">
         <v>0.14199999999999999</v>
       </c>
-      <c r="F34" s="16"/>
       <c r="G34" s="16"/>
-      <c r="H34" s="16">
+      <c r="H34" s="16"/>
+      <c r="I34" s="16">
         <v>0.28399999999999997</v>
       </c>
-      <c r="I34" s="16">
-        <v>0</v>
-      </c>
       <c r="J34" s="16">
+        <v>0</v>
+      </c>
+      <c r="K34" s="16">
         <v>3.4333113999999998E-2</v>
       </c>
-      <c r="K34" s="16">
+      <c r="L34" s="16">
         <v>0.69158415699999998</v>
       </c>
-      <c r="L34" s="16">
-        <v>0</v>
-      </c>
       <c r="M34" s="16">
+        <v>0</v>
+      </c>
+      <c r="N34" s="16">
         <v>4.5041784000000001E-2</v>
       </c>
-      <c r="N34" s="16">
+      <c r="O34" s="16">
         <v>3.93</v>
       </c>
-      <c r="O34" s="16">
+      <c r="P34" s="16">
         <v>3.3959999999999999</v>
       </c>
-      <c r="P34" s="17">
+      <c r="Q34" s="17">
         <v>6.87</v>
       </c>
-      <c r="Q34" s="15" t="s">
+      <c r="R34" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="R34" s="15">
+      <c r="S34" s="15">
         <v>0.55000000000000004</v>
       </c>
-      <c r="S34" s="15" t="s">
+      <c r="T34" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T34" s="15">
+      <c r="U34" s="15">
         <v>30</v>
       </c>
-      <c r="U34" s="15" t="s">
+      <c r="V34" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V34" s="15">
+      <c r="W34" s="15">
         <v>2.2268E-2</v>
       </c>
-      <c r="W34" s="15">
+      <c r="X34" s="15">
         <v>0.35282282100000001</v>
       </c>
     </row>
-    <row r="35" spans="1:23" s="15" customFormat="1">
+    <row r="35" spans="1:24" s="15" customFormat="1">
       <c r="A35" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B35" s="15">
+      <c r="B35" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C35" s="15">
         <v>0.1</v>
       </c>
-      <c r="C35" s="16">
+      <c r="D35" s="16">
         <v>1.3</v>
       </c>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16">
+      <c r="E35" s="16"/>
+      <c r="F35" s="16">
         <v>0.14899999999999999</v>
       </c>
-      <c r="F35" s="16"/>
       <c r="G35" s="16"/>
-      <c r="H35" s="16">
+      <c r="H35" s="16"/>
+      <c r="I35" s="16">
         <v>0.29799999999999999</v>
       </c>
-      <c r="I35" s="16">
-        <v>0</v>
-      </c>
       <c r="J35" s="16">
+        <v>0</v>
+      </c>
+      <c r="K35" s="16">
         <v>7.6426068999999999E-2</v>
       </c>
-      <c r="K35" s="16">
+      <c r="L35" s="16">
         <v>0.84262339500000005</v>
       </c>
-      <c r="L35" s="16">
+      <c r="M35" s="16">
         <v>5.663179E-3</v>
       </c>
-      <c r="M35" s="16">
+      <c r="N35" s="16">
         <v>4.1991897E-2</v>
       </c>
-      <c r="N35" s="16">
+      <c r="O35" s="16">
         <v>4.077</v>
       </c>
-      <c r="O35" s="16">
+      <c r="P35" s="16">
         <v>3.3340000000000001</v>
       </c>
-      <c r="P35" s="17">
+      <c r="Q35" s="17">
         <v>6.87</v>
       </c>
-      <c r="Q35" s="15" t="s">
+      <c r="R35" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="R35" s="15">
+      <c r="S35" s="15">
         <v>0.55000000000000004</v>
       </c>
-      <c r="S35" s="15" t="s">
+      <c r="T35" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T35" s="15">
+      <c r="U35" s="15">
         <v>30</v>
       </c>
-      <c r="U35" s="15" t="s">
+      <c r="V35" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V35" s="15">
+      <c r="W35" s="15">
         <v>1.7815000000000001E-2</v>
       </c>
-      <c r="W35" s="15">
+      <c r="X35" s="15">
         <v>0.36195739300000002</v>
       </c>
     </row>
-    <row r="36" spans="1:23" s="15" customFormat="1">
+    <row r="36" spans="1:24" s="15" customFormat="1">
       <c r="A36" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B36" s="15">
+      <c r="B36" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C36" s="15">
         <v>0.1</v>
       </c>
-      <c r="C36" s="16">
+      <c r="D36" s="16">
         <v>1.4850000000000001</v>
       </c>
-      <c r="D36" s="16"/>
       <c r="E36" s="16"/>
-      <c r="F36" s="16">
+      <c r="F36" s="16"/>
+      <c r="G36" s="16">
         <v>2.8620000000000001</v>
       </c>
-      <c r="G36" s="16"/>
-      <c r="H36" s="16">
+      <c r="H36" s="16"/>
+      <c r="I36" s="16">
         <v>2.8620000000000001</v>
       </c>
-      <c r="I36" s="16">
-        <v>0</v>
-      </c>
       <c r="J36" s="16">
         <v>0</v>
       </c>
       <c r="K36" s="16">
+        <v>0</v>
+      </c>
+      <c r="L36" s="16">
         <v>6.3162172000000003E-2</v>
       </c>
-      <c r="L36" s="16">
-        <v>0</v>
-      </c>
       <c r="M36" s="16">
         <v>0</v>
       </c>
       <c r="N36" s="16">
+        <v>0</v>
+      </c>
+      <c r="O36" s="16">
         <v>5.7110000000000003</v>
       </c>
-      <c r="O36" s="16">
+      <c r="P36" s="16">
         <v>5.6040000000000001</v>
       </c>
-      <c r="P36" s="17">
+      <c r="Q36" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q36" s="15" t="s">
+      <c r="R36" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="R36" s="15">
+      <c r="S36" s="15">
         <v>12.35</v>
       </c>
-      <c r="S36" s="15" t="s">
+      <c r="T36" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T36" s="15">
+      <c r="U36" s="15">
         <v>3</v>
       </c>
-      <c r="U36" s="15" t="s">
+      <c r="V36" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V36" s="15">
+      <c r="W36" s="15">
         <v>1.9595999999999999E-2</v>
       </c>
-      <c r="W36" s="15">
+      <c r="X36" s="15">
         <v>0.425138179</v>
       </c>
     </row>
-    <row r="37" spans="1:23" s="15" customFormat="1">
+    <row r="37" spans="1:24" s="15" customFormat="1">
       <c r="A37" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B37" s="15">
+      <c r="B37" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C37" s="15">
         <v>0.1</v>
       </c>
-      <c r="C37" s="16">
+      <c r="D37" s="16">
         <v>1.6</v>
       </c>
-      <c r="D37" s="16"/>
       <c r="E37" s="16"/>
-      <c r="F37" s="16">
+      <c r="F37" s="16"/>
+      <c r="G37" s="16">
         <v>3.0840000000000001</v>
       </c>
-      <c r="G37" s="16"/>
-      <c r="H37" s="16">
+      <c r="H37" s="16"/>
+      <c r="I37" s="16">
         <v>3.0840000000000001</v>
       </c>
-      <c r="I37" s="16">
-        <v>0</v>
-      </c>
       <c r="J37" s="16">
         <v>0</v>
       </c>
       <c r="K37" s="16">
+        <v>0</v>
+      </c>
+      <c r="L37" s="16">
         <v>7.4209667000000007E-2</v>
       </c>
-      <c r="L37" s="16">
-        <v>0</v>
-      </c>
       <c r="M37" s="16">
         <v>0</v>
       </c>
       <c r="N37" s="16">
+        <v>0</v>
+      </c>
+      <c r="O37" s="16">
         <v>6.0389999999999997</v>
       </c>
-      <c r="O37" s="16">
+      <c r="P37" s="16">
         <v>5.8689999999999998</v>
       </c>
-      <c r="P37" s="17">
+      <c r="Q37" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q37" s="15" t="s">
+      <c r="R37" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="R37" s="15">
+      <c r="S37" s="15">
         <v>12.35</v>
       </c>
-      <c r="S37" s="15" t="s">
+      <c r="T37" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T37" s="15">
+      <c r="U37" s="15">
         <v>3</v>
       </c>
-      <c r="U37" s="15" t="s">
+      <c r="V37" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V37" s="15">
+      <c r="W37" s="15">
         <v>2.0309000000000001E-2</v>
       </c>
-      <c r="W37" s="15">
+      <c r="X37" s="15">
         <v>0.52028996400000005</v>
       </c>
     </row>
-    <row r="38" spans="1:23" s="15" customFormat="1">
+    <row r="38" spans="1:24" s="15" customFormat="1">
       <c r="A38" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B38" s="15">
+      <c r="B38" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C38" s="15">
         <v>0.1</v>
       </c>
-      <c r="C38" s="16">
+      <c r="D38" s="16">
         <v>1.4350000000000001</v>
       </c>
-      <c r="D38" s="16"/>
       <c r="E38" s="16"/>
-      <c r="F38" s="16">
+      <c r="F38" s="16"/>
+      <c r="G38" s="16">
         <v>2.7629999999999999</v>
       </c>
-      <c r="G38" s="16"/>
-      <c r="H38" s="16">
+      <c r="H38" s="16"/>
+      <c r="I38" s="16">
         <v>2.7629999999999999</v>
       </c>
-      <c r="I38" s="16">
-        <v>0</v>
-      </c>
       <c r="J38" s="16">
         <v>0</v>
       </c>
       <c r="K38" s="16">
+        <v>0</v>
+      </c>
+      <c r="L38" s="16">
         <v>7.4921513999999995E-2</v>
       </c>
-      <c r="L38" s="16">
-        <v>0</v>
-      </c>
       <c r="M38" s="16">
         <v>0</v>
       </c>
       <c r="N38" s="16">
+        <v>0</v>
+      </c>
+      <c r="O38" s="16">
         <v>5.32</v>
       </c>
-      <c r="O38" s="16">
+      <c r="P38" s="16">
         <v>5.0789999999999997</v>
       </c>
-      <c r="P38" s="17">
+      <c r="Q38" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q38" s="15" t="s">
+      <c r="R38" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="R38" s="15">
+      <c r="S38" s="15">
         <v>12.35</v>
       </c>
-      <c r="S38" s="15" t="s">
+      <c r="T38" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T38" s="15">
+      <c r="U38" s="15">
         <v>3</v>
       </c>
-      <c r="U38" s="15" t="s">
+      <c r="V38" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V38" s="15">
+      <c r="W38" s="15">
         <v>1.8171E-2</v>
       </c>
-      <c r="W38" s="15">
+      <c r="X38" s="15">
         <v>0.452161286</v>
       </c>
     </row>
-    <row r="39" spans="1:23" s="15" customFormat="1">
+    <row r="39" spans="1:24" s="15" customFormat="1">
       <c r="A39" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B39" s="15">
+      <c r="B39" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C39" s="15">
         <v>0.1</v>
       </c>
-      <c r="C39" s="16">
+      <c r="D39" s="16">
         <v>1.6779999999999999</v>
       </c>
-      <c r="D39" s="16"/>
       <c r="E39" s="16"/>
-      <c r="F39" s="16">
+      <c r="F39" s="16"/>
+      <c r="G39" s="16">
         <v>0.33400000000000002</v>
       </c>
-      <c r="G39" s="16"/>
-      <c r="H39" s="16">
+      <c r="H39" s="16"/>
+      <c r="I39" s="16">
         <v>0.33400000000000002</v>
       </c>
-      <c r="I39" s="16">
-        <v>0</v>
-      </c>
       <c r="J39" s="16">
         <v>0</v>
       </c>
       <c r="K39" s="16">
+        <v>0</v>
+      </c>
+      <c r="L39" s="16">
         <v>0.27117874199999997</v>
       </c>
-      <c r="L39" s="16">
-        <v>0</v>
-      </c>
       <c r="M39" s="16">
         <v>0</v>
       </c>
       <c r="N39" s="16">
+        <v>0</v>
+      </c>
+      <c r="O39" s="16">
         <v>5.7240000000000002</v>
       </c>
-      <c r="O39" s="16">
+      <c r="P39" s="16">
         <v>5.9080000000000004</v>
       </c>
-      <c r="P39" s="17">
+      <c r="Q39" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q39" s="15" t="s">
+      <c r="R39" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="R39" s="15">
+      <c r="S39" s="15">
         <v>1.24</v>
       </c>
-      <c r="S39" s="15" t="s">
+      <c r="T39" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T39" s="15">
+      <c r="U39" s="15">
         <v>30</v>
       </c>
-      <c r="U39" s="15" t="s">
+      <c r="V39" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V39" s="15">
+      <c r="W39" s="15">
         <v>2.3337E-2</v>
       </c>
-      <c r="W39" s="15">
+      <c r="X39" s="15">
         <v>0.41790664300000002</v>
       </c>
     </row>
-    <row r="40" spans="1:23" s="15" customFormat="1">
+    <row r="40" spans="1:24" s="15" customFormat="1">
       <c r="A40" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B40" s="15">
+      <c r="B40" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C40" s="15">
         <v>0.1</v>
       </c>
-      <c r="C40" s="16">
+      <c r="D40" s="16">
         <v>1.6930000000000001</v>
       </c>
-      <c r="D40" s="16"/>
       <c r="E40" s="16"/>
-      <c r="F40" s="16">
+      <c r="F40" s="16"/>
+      <c r="G40" s="16">
         <v>0.33700000000000002</v>
       </c>
-      <c r="G40" s="16"/>
-      <c r="H40" s="16">
+      <c r="H40" s="16"/>
+      <c r="I40" s="16">
         <v>0.33700000000000002</v>
       </c>
-      <c r="I40" s="16">
-        <v>0</v>
-      </c>
       <c r="J40" s="16">
         <v>0</v>
       </c>
       <c r="K40" s="16">
+        <v>0</v>
+      </c>
+      <c r="L40" s="16">
         <v>0.30716928599999999</v>
       </c>
-      <c r="L40" s="16">
-        <v>0</v>
-      </c>
       <c r="M40" s="16">
         <v>0</v>
       </c>
       <c r="N40" s="16">
+        <v>0</v>
+      </c>
+      <c r="O40" s="16">
         <v>5.9720000000000004</v>
       </c>
-      <c r="O40" s="16">
+      <c r="P40" s="16">
         <v>5.29</v>
       </c>
-      <c r="P40" s="17">
+      <c r="Q40" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q40" s="15" t="s">
+      <c r="R40" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="R40" s="15">
+      <c r="S40" s="15">
         <v>1.24</v>
       </c>
-      <c r="S40" s="15" t="s">
+      <c r="T40" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T40" s="15">
+      <c r="U40" s="15">
         <v>30</v>
       </c>
-      <c r="U40" s="15" t="s">
+      <c r="V40" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V40" s="15">
+      <c r="W40" s="15">
         <v>2.4941000000000001E-2</v>
       </c>
-      <c r="W40" s="15">
+      <c r="X40" s="15">
         <v>0.37870410700000001</v>
       </c>
     </row>
-    <row r="41" spans="1:23" s="15" customFormat="1">
+    <row r="41" spans="1:24" s="15" customFormat="1">
       <c r="A41" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B41" s="15">
+      <c r="B41" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C41" s="15">
         <v>0.1</v>
       </c>
-      <c r="C41" s="16">
+      <c r="D41" s="16">
         <v>1.647</v>
       </c>
-      <c r="D41" s="16"/>
       <c r="E41" s="16"/>
-      <c r="F41" s="16">
+      <c r="F41" s="16"/>
+      <c r="G41" s="16">
         <v>0.32700000000000001</v>
       </c>
-      <c r="G41" s="16"/>
-      <c r="H41" s="16">
+      <c r="H41" s="16"/>
+      <c r="I41" s="16">
         <v>0.32700000000000001</v>
       </c>
-      <c r="I41" s="16">
-        <v>0</v>
-      </c>
       <c r="J41" s="16">
         <v>0</v>
       </c>
       <c r="K41" s="16">
+        <v>0</v>
+      </c>
+      <c r="L41" s="16">
         <v>0.20397084300000001</v>
       </c>
-      <c r="L41" s="16">
-        <v>0</v>
-      </c>
       <c r="M41" s="16">
         <v>0</v>
       </c>
       <c r="N41" s="16">
+        <v>0</v>
+      </c>
+      <c r="O41" s="16">
         <v>6.1310000000000002</v>
       </c>
-      <c r="O41" s="16">
+      <c r="P41" s="16">
         <v>5.69</v>
       </c>
-      <c r="P41" s="17">
+      <c r="Q41" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q41" s="15" t="s">
+      <c r="R41" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="R41" s="15">
+      <c r="S41" s="15">
         <v>1.24</v>
       </c>
-      <c r="S41" s="15" t="s">
+      <c r="T41" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T41" s="15">
+      <c r="U41" s="15">
         <v>30</v>
       </c>
-      <c r="U41" s="15" t="s">
+      <c r="V41" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V41" s="15">
+      <c r="W41" s="15">
         <v>2.4406000000000001E-2</v>
       </c>
-      <c r="W41" s="15">
+      <c r="X41" s="15">
         <v>0.39887628600000002</v>
       </c>
     </row>
-    <row r="42" spans="1:23" s="15" customFormat="1">
+    <row r="42" spans="1:24" s="15" customFormat="1">
       <c r="A42" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B42" s="15">
+      <c r="B42" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C42" s="15">
         <v>0.1</v>
       </c>
-      <c r="C42" s="16">
+      <c r="D42" s="16">
         <v>1.4790000000000001</v>
       </c>
-      <c r="D42" s="16"/>
       <c r="E42" s="16"/>
       <c r="F42" s="16"/>
-      <c r="G42" s="16">
-        <v>2.919</v>
-      </c>
+      <c r="G42" s="16"/>
       <c r="H42" s="16">
         <v>2.919</v>
       </c>
       <c r="I42" s="16">
+        <v>2.919</v>
+      </c>
+      <c r="J42" s="16">
         <v>6.4434642E-2</v>
       </c>
-      <c r="J42" s="16">
-        <v>0</v>
-      </c>
       <c r="K42" s="16">
+        <v>0</v>
+      </c>
+      <c r="L42" s="16">
         <v>0.16559933199999999</v>
       </c>
-      <c r="L42" s="16">
-        <v>0</v>
-      </c>
       <c r="M42" s="16">
+        <v>0</v>
+      </c>
+      <c r="N42" s="16">
         <v>4.8736990000000004E-3</v>
       </c>
-      <c r="N42" s="16">
+      <c r="O42" s="16">
         <v>4.7869999999999999</v>
       </c>
-      <c r="O42" s="16">
+      <c r="P42" s="16">
         <v>4.5609999999999999</v>
       </c>
-      <c r="P42" s="17">
+      <c r="Q42" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q42" s="15" t="s">
+      <c r="R42" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="R42" s="15">
+      <c r="S42" s="15">
         <v>9.81</v>
       </c>
-      <c r="S42" s="15" t="s">
+      <c r="T42" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T42" s="15">
+      <c r="U42" s="15">
         <v>3</v>
       </c>
-      <c r="U42" s="15" t="s">
+      <c r="V42" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V42" s="15">
+      <c r="W42" s="15">
         <v>2.9215999999999999E-2</v>
       </c>
-      <c r="W42" s="15">
+      <c r="X42" s="15">
         <v>0.32085182099999998</v>
       </c>
     </row>
-    <row r="43" spans="1:23" s="15" customFormat="1">
+    <row r="43" spans="1:24" s="15" customFormat="1">
       <c r="A43" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B43" s="15">
+      <c r="B43" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43" s="15">
         <v>0.1</v>
       </c>
-      <c r="C43" s="16">
+      <c r="D43" s="16">
         <v>1.633</v>
       </c>
-      <c r="D43" s="16"/>
       <c r="E43" s="16"/>
       <c r="F43" s="16"/>
-      <c r="G43" s="16">
-        <v>3.2</v>
-      </c>
+      <c r="G43" s="16"/>
       <c r="H43" s="16">
         <v>3.2</v>
       </c>
       <c r="I43" s="16">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="J43" s="16">
         <v>0</v>
       </c>
       <c r="K43" s="16">
+        <v>0</v>
+      </c>
+      <c r="L43" s="16">
         <v>0.156217087</v>
       </c>
-      <c r="L43" s="16">
-        <v>0</v>
-      </c>
       <c r="M43" s="16">
         <v>0</v>
       </c>
       <c r="N43" s="16">
+        <v>0</v>
+      </c>
+      <c r="O43" s="16">
         <v>5.1379999999999999</v>
       </c>
-      <c r="O43" s="16">
+      <c r="P43" s="16">
         <v>4.9089999999999998</v>
       </c>
-      <c r="P43" s="17">
+      <c r="Q43" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q43" s="15" t="s">
+      <c r="R43" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="R43" s="15">
+      <c r="S43" s="15">
         <v>9.81</v>
       </c>
-      <c r="S43" s="15" t="s">
+      <c r="T43" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T43" s="15">
+      <c r="U43" s="15">
         <v>3</v>
       </c>
-      <c r="U43" s="15" t="s">
+      <c r="V43" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V43" s="15">
+      <c r="W43" s="15">
         <v>3.4738999999999999E-2</v>
       </c>
-      <c r="W43" s="15">
+      <c r="X43" s="15">
         <v>0.41866785699999998</v>
       </c>
     </row>
-    <row r="44" spans="1:23" s="15" customFormat="1">
+    <row r="44" spans="1:24" s="15" customFormat="1">
       <c r="A44" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B44" s="15">
+      <c r="B44" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C44" s="15">
         <v>0.1</v>
       </c>
-      <c r="C44" s="16">
+      <c r="D44" s="16">
         <v>1.571</v>
       </c>
-      <c r="D44" s="16"/>
       <c r="E44" s="16"/>
       <c r="F44" s="16"/>
-      <c r="G44" s="16">
-        <v>3.0830000000000002</v>
-      </c>
+      <c r="G44" s="16"/>
       <c r="H44" s="16">
         <v>3.0830000000000002</v>
       </c>
       <c r="I44" s="16">
+        <v>3.0830000000000002</v>
+      </c>
+      <c r="J44" s="16">
         <v>6.4504826000000001E-2</v>
       </c>
-      <c r="J44" s="16">
-        <v>0</v>
-      </c>
       <c r="K44" s="16">
+        <v>0</v>
+      </c>
+      <c r="L44" s="16">
         <v>0.15037355499999999</v>
       </c>
-      <c r="L44" s="16">
-        <v>0</v>
-      </c>
       <c r="M44" s="16">
+        <v>0</v>
+      </c>
+      <c r="N44" s="16">
         <v>5.596462E-3</v>
       </c>
-      <c r="N44" s="16">
+      <c r="O44" s="16">
         <v>4.9610000000000003</v>
       </c>
-      <c r="O44" s="16">
+      <c r="P44" s="16">
         <v>4.5490000000000004</v>
       </c>
-      <c r="P44" s="17">
+      <c r="Q44" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q44" s="15" t="s">
+      <c r="R44" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="R44" s="15">
+      <c r="S44" s="15">
         <v>9.81</v>
       </c>
-      <c r="S44" s="15" t="s">
+      <c r="T44" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="T44" s="15">
+      <c r="U44" s="15">
         <v>3</v>
       </c>
-      <c r="U44" s="15" t="s">
+      <c r="V44" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V44" s="15">
+      <c r="W44" s="15">
         <v>3.0641000000000002E-2</v>
       </c>
-      <c r="W44" s="15">
+      <c r="X44" s="15">
         <v>0.33150882100000001</v>
       </c>
     </row>
-    <row r="45" spans="1:23" s="15" customFormat="1">
+    <row r="45" spans="1:24" s="15" customFormat="1">
       <c r="A45" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B45" s="15">
+      <c r="B45" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C45" s="15">
         <v>0.1</v>
       </c>
-      <c r="C45" s="16">
+      <c r="D45" s="16">
         <v>1.4510000000000001</v>
       </c>
-      <c r="D45" s="16"/>
       <c r="E45" s="16"/>
       <c r="F45" s="16"/>
-      <c r="G45" s="16">
-        <v>0.29199999999999998</v>
-      </c>
+      <c r="G45" s="16"/>
       <c r="H45" s="16">
         <v>0.29199999999999998</v>
       </c>
       <c r="I45" s="16">
+        <v>0.29199999999999998</v>
+      </c>
+      <c r="J45" s="16">
         <v>0.16597783599999999</v>
       </c>
-      <c r="J45" s="16">
+      <c r="K45" s="16">
         <v>6.6479359000000002E-2</v>
       </c>
-      <c r="K45" s="16">
+      <c r="L45" s="16">
         <v>0.60819290000000004</v>
       </c>
-      <c r="L45" s="16">
-        <v>0</v>
-      </c>
       <c r="M45" s="16">
+        <v>0</v>
+      </c>
+      <c r="N45" s="16">
         <v>2.5725250000000002E-2</v>
       </c>
-      <c r="N45" s="16">
+      <c r="O45" s="16">
         <v>4.18</v>
       </c>
-      <c r="O45" s="16">
+      <c r="P45" s="16">
         <v>4.0129999999999999</v>
       </c>
-      <c r="P45" s="17">
+      <c r="Q45" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q45" s="15" t="s">
+      <c r="R45" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="R45" s="15">
+      <c r="S45" s="15">
         <v>0.98</v>
       </c>
-      <c r="S45" s="15" t="s">
+      <c r="T45" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T45" s="15">
+      <c r="U45" s="15">
         <v>30</v>
       </c>
-      <c r="U45" s="15" t="s">
+      <c r="V45" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V45" s="15">
+      <c r="W45" s="15">
         <v>2.4761999999999999E-2</v>
       </c>
-      <c r="W45" s="15">
+      <c r="X45" s="15">
         <v>0.43998185699999998</v>
       </c>
     </row>
-    <row r="46" spans="1:23" s="15" customFormat="1">
+    <row r="46" spans="1:24" s="15" customFormat="1">
       <c r="A46" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B46" s="15">
+      <c r="B46" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C46" s="15">
         <v>0.1</v>
       </c>
-      <c r="C46" s="16">
+      <c r="D46" s="16">
         <v>1.7090000000000001</v>
       </c>
-      <c r="D46" s="16"/>
       <c r="E46" s="16"/>
       <c r="F46" s="16"/>
-      <c r="G46" s="16">
-        <v>0.33900000000000002</v>
-      </c>
+      <c r="G46" s="16"/>
       <c r="H46" s="16">
         <v>0.33900000000000002</v>
       </c>
       <c r="I46" s="16">
+        <v>0.33900000000000002</v>
+      </c>
+      <c r="J46" s="16">
         <v>6.0174350000000001E-2</v>
       </c>
-      <c r="J46" s="16">
+      <c r="K46" s="16">
         <v>7.8079274000000004E-2</v>
       </c>
-      <c r="K46" s="16">
+      <c r="L46" s="16">
         <v>0.66867871400000001</v>
       </c>
-      <c r="L46" s="16">
-        <v>0</v>
-      </c>
       <c r="M46" s="16">
+        <v>0</v>
+      </c>
+      <c r="N46" s="16">
         <v>3.5868012999999997E-2</v>
       </c>
-      <c r="N46" s="16">
+      <c r="O46" s="16">
         <v>4.9020000000000001</v>
       </c>
-      <c r="O46" s="16">
+      <c r="P46" s="16">
         <v>4.45</v>
       </c>
-      <c r="P46" s="17">
+      <c r="Q46" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q46" s="15" t="s">
+      <c r="R46" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="R46" s="15">
+      <c r="S46" s="15">
         <v>0.98</v>
       </c>
-      <c r="S46" s="15" t="s">
+      <c r="T46" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T46" s="15">
+      <c r="U46" s="15">
         <v>30</v>
       </c>
-      <c r="U46" s="15" t="s">
+      <c r="V46" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V46" s="15">
+      <c r="W46" s="15">
         <v>2.1912000000000001E-2</v>
       </c>
-      <c r="W46" s="15">
+      <c r="X46" s="15">
         <v>0.448355214</v>
       </c>
     </row>
-    <row r="47" spans="1:23" s="15" customFormat="1">
+    <row r="47" spans="1:24" s="15" customFormat="1">
       <c r="A47" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B47" s="15">
+      <c r="B47" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C47" s="15">
         <v>0.1</v>
       </c>
-      <c r="C47" s="16">
+      <c r="D47" s="16">
         <v>1.6220000000000001</v>
       </c>
-      <c r="D47" s="16"/>
       <c r="E47" s="16"/>
       <c r="F47" s="16"/>
-      <c r="G47" s="16">
-        <v>0.32900000000000001</v>
-      </c>
+      <c r="G47" s="16"/>
       <c r="H47" s="16">
         <v>0.32900000000000001</v>
       </c>
       <c r="I47" s="16">
+        <v>0.32900000000000001</v>
+      </c>
+      <c r="J47" s="16">
         <v>0.18362290100000001</v>
       </c>
-      <c r="J47" s="16">
+      <c r="K47" s="16">
         <v>0.16825845</v>
       </c>
-      <c r="K47" s="16">
+      <c r="L47" s="16">
         <v>0.92271634599999997</v>
       </c>
-      <c r="L47" s="16">
-        <v>0</v>
-      </c>
       <c r="M47" s="16">
+        <v>0</v>
+      </c>
+      <c r="N47" s="16">
         <v>4.8272586999999999E-2</v>
       </c>
-      <c r="N47" s="16">
+      <c r="O47" s="16">
         <v>4.5620000000000003</v>
       </c>
-      <c r="O47" s="16">
+      <c r="P47" s="16">
         <v>4.2300000000000004</v>
       </c>
-      <c r="P47" s="17">
+      <c r="Q47" s="17">
         <v>7.5</v>
       </c>
-      <c r="Q47" s="15" t="s">
+      <c r="R47" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="R47" s="15">
+      <c r="S47" s="15">
         <v>0.98</v>
       </c>
-      <c r="S47" s="15" t="s">
+      <c r="T47" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="T47" s="15">
+      <c r="U47" s="15">
         <v>30</v>
       </c>
-      <c r="U47" s="15" t="s">
+      <c r="V47" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="V47" s="15">
+      <c r="W47" s="15">
         <v>2.4761999999999999E-2</v>
       </c>
-      <c r="W47" s="15">
+      <c r="X47" s="15">
         <v>0.42361575000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:23" s="26" customFormat="1">
+    <row r="48" spans="1:24" s="26" customFormat="1">
       <c r="A48" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="B48" s="25">
+      <c r="B48" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C48" s="25">
         <v>0.1</v>
       </c>
-      <c r="P48" s="27"/>
-    </row>
-    <row r="49" spans="1:16" s="7" customFormat="1">
+      <c r="Q48" s="27"/>
+    </row>
+    <row r="49" spans="1:17" s="7" customFormat="1">
       <c r="A49" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B49" s="5">
+      <c r="B49" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C49" s="5">
         <v>0.40653850000000002</v>
       </c>
-      <c r="C49" s="6">
+      <c r="D49" s="6">
         <v>-13.20185</v>
       </c>
-      <c r="I49" s="6">
+      <c r="J49" s="6">
         <v>15.979100000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:16" s="7" customFormat="1">
+    <row r="50" spans="1:17" s="7" customFormat="1">
       <c r="A50" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B50" s="5">
+      <c r="B50" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C50" s="5">
         <v>0.44837779999999999</v>
       </c>
-      <c r="C50" s="6">
+      <c r="D50" s="6">
         <v>-12.97245</v>
       </c>
-      <c r="I50" s="6">
+      <c r="J50" s="6">
         <v>17.642130000000002</v>
       </c>
     </row>
-    <row r="51" spans="1:16" s="7" customFormat="1">
+    <row r="51" spans="1:17" s="7" customFormat="1">
       <c r="A51" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B51" s="5">
+      <c r="B51" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C51" s="5">
         <v>0.32723469999999999</v>
       </c>
-      <c r="C51" s="6">
+      <c r="D51" s="6">
         <v>-18.39499</v>
       </c>
-      <c r="I51" s="6">
+      <c r="J51" s="6">
         <v>27.157050000000002</v>
       </c>
-      <c r="M51" s="5">
+      <c r="N51" s="5">
         <v>3.6701839999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:16" s="7" customFormat="1">
+    <row r="52" spans="1:17" s="7" customFormat="1">
       <c r="A52" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B52" s="5">
+      <c r="B52" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C52" s="5">
         <v>0.32866410000000001</v>
       </c>
-      <c r="C52" s="6">
+      <c r="D52" s="6">
         <v>-14.408200000000001</v>
       </c>
-      <c r="I52" s="6">
+      <c r="J52" s="6">
         <v>22.896090000000001</v>
       </c>
-      <c r="M52" s="5">
+      <c r="N52" s="5">
         <v>1.9558949999999999</v>
       </c>
     </row>
-    <row r="53" spans="1:16" s="12" customFormat="1">
+    <row r="53" spans="1:17" s="12" customFormat="1">
       <c r="A53" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B53" s="12">
+      <c r="B53" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C53" s="12">
         <v>0.1</v>
       </c>
-      <c r="P53" s="11"/>
-    </row>
-    <row r="54" spans="1:16" s="12" customFormat="1">
+      <c r="Q53" s="11"/>
+    </row>
+    <row r="54" spans="1:17" s="12" customFormat="1">
       <c r="A54" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B54" s="12">
+      <c r="B54" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C54" s="12">
         <v>0.1</v>
       </c>
-      <c r="D54" s="18"/>
-      <c r="P54" s="11"/>
-    </row>
-    <row r="55" spans="1:16" s="12" customFormat="1">
+      <c r="E54" s="18"/>
+      <c r="Q54" s="11"/>
+    </row>
+    <row r="55" spans="1:17" s="12" customFormat="1">
       <c r="A55" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B55" s="12">
+      <c r="B55" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C55" s="12">
         <v>0.1</v>
       </c>
-      <c r="P55" s="11"/>
-    </row>
-    <row r="56" spans="1:16" s="12" customFormat="1">
+      <c r="Q55" s="11"/>
+    </row>
+    <row r="56" spans="1:17" s="12" customFormat="1">
       <c r="A56" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B56" s="12">
+      <c r="B56" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C56" s="12">
         <v>0.1</v>
       </c>
-      <c r="P56" s="11"/>
-    </row>
-    <row r="57" spans="1:16" s="12" customFormat="1">
+      <c r="Q56" s="11"/>
+    </row>
+    <row r="57" spans="1:17" s="12" customFormat="1">
       <c r="A57" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="P57" s="11"/>
-    </row>
-    <row r="58" spans="1:16" s="12" customFormat="1">
+      <c r="B57" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q57" s="11"/>
+    </row>
+    <row r="58" spans="1:17" s="12" customFormat="1">
       <c r="A58" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="P58" s="11"/>
-    </row>
-    <row r="59" spans="1:16" s="12" customFormat="1">
+      <c r="B58" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q58" s="11"/>
+    </row>
+    <row r="59" spans="1:17" s="12" customFormat="1">
       <c r="A59" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="P59" s="11"/>
-    </row>
-    <row r="60" spans="1:16" s="12" customFormat="1">
+      <c r="B59" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q59" s="11"/>
+    </row>
+    <row r="60" spans="1:17" s="12" customFormat="1">
       <c r="A60" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="P60" s="11"/>
-    </row>
-    <row r="61" spans="1:16" s="12" customFormat="1">
+      <c r="B60" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q60" s="11"/>
+    </row>
+    <row r="61" spans="1:17" s="12" customFormat="1">
       <c r="A61" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="P61" s="11"/>
-    </row>
-    <row r="62" spans="1:16" s="12" customFormat="1">
+      <c r="B61" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q61" s="11"/>
+    </row>
+    <row r="62" spans="1:17" s="12" customFormat="1">
       <c r="A62" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="P62" s="11"/>
-    </row>
-    <row r="63" spans="1:16" s="12" customFormat="1">
+      <c r="B62" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q62" s="11"/>
+    </row>
+    <row r="63" spans="1:17" s="12" customFormat="1">
       <c r="A63" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="P63" s="11"/>
-    </row>
-    <row r="64" spans="1:16" s="12" customFormat="1">
+      <c r="B63" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q63" s="11"/>
+    </row>
+    <row r="64" spans="1:17" s="12" customFormat="1">
       <c r="A64" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="P64" s="11"/>
-    </row>
-    <row r="65" spans="1:23" s="12" customFormat="1">
+      <c r="B64" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q64" s="11"/>
+    </row>
+    <row r="65" spans="1:24" s="12" customFormat="1">
       <c r="A65" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="P65" s="11"/>
-    </row>
-    <row r="66" spans="1:23" s="12" customFormat="1">
+      <c r="B65" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q65" s="11"/>
+    </row>
+    <row r="66" spans="1:24" s="12" customFormat="1">
       <c r="A66" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="P66" s="11"/>
-    </row>
-    <row r="67" spans="1:23" s="12" customFormat="1">
+      <c r="B66" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q66" s="11"/>
+    </row>
+    <row r="67" spans="1:24" s="12" customFormat="1">
       <c r="A67" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="P67" s="11"/>
-    </row>
-    <row r="68" spans="1:23" s="12" customFormat="1">
+      <c r="B67" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q67" s="11"/>
+    </row>
+    <row r="68" spans="1:24" s="12" customFormat="1">
       <c r="A68" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="P68" s="11"/>
-    </row>
-    <row r="69" spans="1:23" s="19" customFormat="1">
+      <c r="B68" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q68" s="11"/>
+    </row>
+    <row r="69" spans="1:24" s="19" customFormat="1">
       <c r="A69" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B69" s="19">
+      <c r="B69" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C69" s="19">
         <v>2.7E-2</v>
       </c>
-      <c r="C69" s="20">
+      <c r="D69" s="20">
         <v>-0.33700000000000002</v>
       </c>
-      <c r="D69" s="20">
+      <c r="E69" s="20">
         <v>-0.151308114750691</v>
       </c>
-      <c r="I69" s="20">
-        <v>0</v>
-      </c>
-      <c r="N69" s="20">
+      <c r="J69" s="20">
+        <v>0</v>
+      </c>
+      <c r="O69" s="20">
         <v>0.878</v>
       </c>
-      <c r="O69" s="21">
-        <v>-0.86358170086251695</v>
-      </c>
-      <c r="P69" s="22"/>
-      <c r="Q69" s="19" t="s">
+      <c r="P69" s="21">
+        <v>0.86358170086251695</v>
+      </c>
+      <c r="Q69" s="22"/>
+      <c r="R69" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S69" s="19" t="s">
+      <c r="T69" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W69" s="19">
+      <c r="X69" s="19">
         <v>0.29899999999999999</v>
       </c>
     </row>
-    <row r="70" spans="1:23" s="21" customFormat="1">
+    <row r="70" spans="1:24" s="21" customFormat="1">
       <c r="A70" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="B70" s="21">
+      <c r="B70" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C70" s="21">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="C70" s="20">
+      <c r="D70" s="20">
         <v>-0.52300000000000002</v>
       </c>
-      <c r="D70" s="20">
+      <c r="E70" s="20">
         <v>-0.22220072795676099</v>
       </c>
-      <c r="I70" s="20">
-        <v>0</v>
-      </c>
-      <c r="N70" s="20">
+      <c r="J70" s="20">
+        <v>0</v>
+      </c>
+      <c r="O70" s="20">
         <v>1.458</v>
       </c>
-      <c r="O70" s="21">
-        <v>-1.4368262739973601</v>
-      </c>
-      <c r="P70" s="23"/>
-      <c r="Q70" s="19" t="s">
+      <c r="P70" s="21">
+        <v>1.4368262739973601</v>
+      </c>
+      <c r="Q70" s="23"/>
+      <c r="R70" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S70" s="19" t="s">
+      <c r="T70" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W70" s="21">
+      <c r="X70" s="21">
         <v>0.312</v>
       </c>
     </row>
-    <row r="71" spans="1:23" s="21" customFormat="1">
+    <row r="71" spans="1:24" s="21" customFormat="1">
       <c r="A71" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B71" s="21">
+      <c r="B71" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C71" s="21">
         <v>0.10199999999999999</v>
       </c>
-      <c r="C71" s="20">
+      <c r="D71" s="20">
         <v>-1.171</v>
       </c>
-      <c r="D71" s="20">
+      <c r="E71" s="20">
         <v>-0.59240301221006997</v>
       </c>
-      <c r="I71" s="20">
-        <v>0</v>
-      </c>
-      <c r="N71" s="20">
+      <c r="J71" s="20">
+        <v>0</v>
+      </c>
+      <c r="O71" s="20">
         <v>2.5470000000000002</v>
       </c>
-      <c r="O71" s="21">
-        <v>-2.4905493340587901</v>
-      </c>
-      <c r="P71" s="23"/>
-      <c r="Q71" s="19" t="s">
+      <c r="P71" s="21">
+        <v>2.4905493340587901</v>
+      </c>
+      <c r="Q71" s="23"/>
+      <c r="R71" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S71" s="19" t="s">
+      <c r="T71" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W71" s="21">
+      <c r="X71" s="21">
         <v>0.371</v>
       </c>
     </row>
-    <row r="72" spans="1:23" s="21" customFormat="1">
+    <row r="72" spans="1:24" s="21" customFormat="1">
       <c r="A72" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="B72" s="21">
+      <c r="B72" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C72" s="21">
         <v>0.152</v>
       </c>
-      <c r="C72" s="20">
+      <c r="D72" s="20">
         <v>-1.6830000000000001</v>
       </c>
-      <c r="D72" s="20">
+      <c r="E72" s="20">
         <v>-0.81572561388224996</v>
       </c>
-      <c r="I72" s="20">
-        <v>0</v>
-      </c>
-      <c r="N72" s="20">
+      <c r="J72" s="20">
+        <v>0</v>
+      </c>
+      <c r="O72" s="20">
         <v>3.81518914277475</v>
       </c>
-      <c r="O72" s="21">
-        <v>-3.855</v>
-      </c>
-      <c r="P72" s="23"/>
-      <c r="Q72" s="19" t="s">
+      <c r="P72" s="21">
+        <v>3.855</v>
+      </c>
+      <c r="Q72" s="23"/>
+      <c r="R72" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S72" s="19" t="s">
+      <c r="T72" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W72" s="21">
+      <c r="X72" s="21">
         <v>0.41899999999999998</v>
       </c>
     </row>
-    <row r="73" spans="1:23" s="21" customFormat="1">
+    <row r="73" spans="1:24" s="21" customFormat="1">
       <c r="A73" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="B73" s="21">
+      <c r="B73" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C73" s="21">
         <v>0.214</v>
       </c>
-      <c r="C73" s="20">
+      <c r="D73" s="20">
         <v>-2.4769999999999999</v>
       </c>
-      <c r="D73" s="20">
+      <c r="E73" s="20">
         <v>-1.22567508688439</v>
       </c>
-      <c r="I73" s="20">
+      <c r="J73" s="20">
         <v>-3.4044364549679102E-12</v>
       </c>
-      <c r="N73" s="20">
+      <c r="O73" s="20">
         <v>5.5949999999999998</v>
       </c>
-      <c r="O73" s="21">
-        <v>-5.4782042149448502</v>
-      </c>
-      <c r="P73" s="23"/>
-      <c r="Q73" s="19" t="s">
+      <c r="P73" s="21">
+        <v>5.4782042149448502</v>
+      </c>
+      <c r="Q73" s="23"/>
+      <c r="R73" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S73" s="19" t="s">
+      <c r="T73" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W73" s="21">
+      <c r="X73" s="21">
         <v>0.32</v>
       </c>
     </row>
-    <row r="74" spans="1:23" s="21" customFormat="1">
+    <row r="74" spans="1:24" s="21" customFormat="1">
       <c r="A74" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B74" s="21">
+      <c r="B74" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C74" s="21">
         <v>0.254</v>
       </c>
-      <c r="C74" s="20">
+      <c r="D74" s="20">
         <v>-2.8620000000000001</v>
       </c>
-      <c r="D74" s="20">
+      <c r="E74" s="20">
         <v>-1.4136198692773401</v>
       </c>
-      <c r="I74" s="20">
+      <c r="J74" s="20">
         <v>7.3805128675275E-12</v>
       </c>
-      <c r="N74" s="20">
+      <c r="O74" s="20">
         <v>6.484</v>
       </c>
-      <c r="O74" s="21">
-        <v>-6.2489999999999997</v>
-      </c>
-      <c r="P74" s="23"/>
-      <c r="Q74" s="19" t="s">
+      <c r="P74" s="21">
+        <v>6.2489999999999997</v>
+      </c>
+      <c r="Q74" s="23"/>
+      <c r="R74" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S74" s="19" t="s">
+      <c r="T74" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W74" s="21">
+      <c r="X74" s="21">
         <v>0.37799999999999995</v>
       </c>
     </row>
-    <row r="75" spans="1:23" s="21" customFormat="1">
+    <row r="75" spans="1:24" s="21" customFormat="1">
       <c r="A75" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B75" s="21">
+      <c r="B75" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C75" s="21">
         <v>0.28399999999999997</v>
       </c>
-      <c r="C75" s="20">
+      <c r="D75" s="20">
         <v>-3.2050000000000001</v>
       </c>
-      <c r="D75" s="20">
+      <c r="E75" s="20">
         <v>-1.47353470842518</v>
       </c>
-      <c r="I75" s="20">
+      <c r="J75" s="20">
         <v>-3.4111879987364099E-12</v>
       </c>
-      <c r="N75" s="20">
+      <c r="O75" s="20">
         <v>8.0890000000000004</v>
       </c>
-      <c r="O75" s="21">
-        <v>-7.9485854277214001</v>
-      </c>
-      <c r="P75" s="23"/>
-      <c r="Q75" s="19" t="s">
+      <c r="P75" s="21">
+        <v>7.9485854277214001</v>
+      </c>
+      <c r="Q75" s="23"/>
+      <c r="R75" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S75" s="19" t="s">
+      <c r="T75" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W75" s="21">
+      <c r="X75" s="21">
         <v>0.39100000000000001</v>
       </c>
     </row>
-    <row r="76" spans="1:23" s="21" customFormat="1">
+    <row r="76" spans="1:24" s="21" customFormat="1">
       <c r="A76" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B76" s="21">
+      <c r="B76" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C76" s="21">
         <v>0.33400000000000002</v>
       </c>
-      <c r="C76" s="20">
+      <c r="D76" s="20">
         <v>-5.2350000000000003</v>
       </c>
-      <c r="D76" s="20">
+      <c r="E76" s="20">
         <v>-1.99253212300414</v>
       </c>
-      <c r="I76" s="20">
+      <c r="J76" s="20">
         <v>2.0830000000081101</v>
       </c>
-      <c r="N76" s="20">
+      <c r="O76" s="20">
         <v>11.872999999999999</v>
       </c>
-      <c r="O76" s="21">
-        <v>-9.6077296533960403</v>
-      </c>
-      <c r="P76" s="23"/>
-      <c r="Q76" s="19" t="s">
+      <c r="P76" s="21">
+        <v>9.6077296533960403</v>
+      </c>
+      <c r="Q76" s="23"/>
+      <c r="R76" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S76" s="19" t="s">
+      <c r="T76" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W76" s="21">
+      <c r="X76" s="21">
         <v>0.41899999999999998</v>
       </c>
     </row>
-    <row r="77" spans="1:23" s="21" customFormat="1">
+    <row r="77" spans="1:24" s="21" customFormat="1">
       <c r="A77" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="B77" s="21">
+      <c r="B77" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C77" s="21">
         <v>0.379</v>
       </c>
-      <c r="C77" s="20">
+      <c r="D77" s="20">
         <v>-6.9569999999999999</v>
       </c>
-      <c r="D77" s="20">
+      <c r="E77" s="20">
         <v>-2.0155334705947299</v>
       </c>
-      <c r="I77" s="20">
+      <c r="J77" s="20">
         <v>5.5389999999999997</v>
       </c>
-      <c r="N77" s="20">
+      <c r="O77" s="20">
         <v>14.304133448972699</v>
       </c>
-      <c r="O77" s="21">
-        <v>-8.8979999999999997</v>
-      </c>
-      <c r="P77" s="23"/>
-      <c r="Q77" s="19" t="s">
+      <c r="P77" s="21">
+        <v>8.8979999999999997</v>
+      </c>
+      <c r="Q77" s="23"/>
+      <c r="R77" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="S77" s="19" t="s">
+      <c r="T77" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="W77" s="21">
+      <c r="X77" s="21">
         <v>0.39100000000000001</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add code for graph
</commit_message>
<xml_diff>
--- a/data/proteomics/physiology_collection.xlsx
+++ b/data/proteomics/physiology_collection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Documents/GitHub/De-nevo-protein-3D-structure-yeast/data/proteomics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5CD058E-38E8-0946-888A-DB788D917361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5066DF8-4453-A044-86EF-EF08044830BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="26880" windowHeight="15220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2780" yWindow="500" windowWidth="32900" windowHeight="21440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -18,6 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$T$1:$T$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Supplementary File 1e vip'!$T$1:$T$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="116">
   <si>
     <t>sample</t>
   </si>
@@ -565,7 +566,7 @@
       <name val="Times Roman"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -775,6 +776,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -951,7 +958,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1018,6 +1025,8 @@
     <xf numFmtId="0" fontId="21" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="38" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4994,1521 +5003,2435 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:V43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="2" max="2" width="17.1640625" customWidth="1"/>
+    <col min="3" max="3" width="21.33203125" customWidth="1"/>
+    <col min="4" max="4" width="23.83203125" customWidth="1"/>
+    <col min="15" max="15" width="20.33203125" customWidth="1"/>
+    <col min="18" max="18" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="30.5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:22">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
+      <c r="Q1" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="R1" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="S1" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="T1" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="U1" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="V1" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="C2">
         <v>0.82299999999999995</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>0.13100000000000001</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>0.13100000000000001</v>
       </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
         <v>7.2308500000000005E-4</v>
       </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
       <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
         <v>4.0285879999999996E-3</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>2.4449999999999998</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>2.3620000000000001</v>
       </c>
-    </row>
-    <row r="3" spans="1:14">
+      <c r="Q2" s="15">
+        <v>0.27251471399999999</v>
+      </c>
+      <c r="R2" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S2" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T2" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U2" s="15">
+        <v>30</v>
+      </c>
+      <c r="V2" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="C3">
         <v>0.70399999999999996</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>8.6999999999999994E-2</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>8.6999999999999994E-2</v>
       </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
         <v>1.6583900000000001E-4</v>
       </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
       <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
         <v>6.6796169999999997E-3</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>2.105</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>2.2759999999999998</v>
       </c>
-    </row>
-    <row r="4" spans="1:14">
+      <c r="Q3" s="15">
+        <v>0.25082010700000001</v>
+      </c>
+      <c r="R3" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S3" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T3" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U3" s="15">
+        <v>30</v>
+      </c>
+      <c r="V3" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="C4">
         <v>0.76800000000000002</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>0.14000000000000001</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>0.14000000000000001</v>
       </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
       <c r="I4">
         <v>0</v>
       </c>
       <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
         <v>3.81541E-4</v>
       </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
       <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
         <v>9.7823159999999992E-3</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>2.383</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>1.6240000000000001</v>
       </c>
-    </row>
-    <row r="5" spans="1:14">
-      <c r="A5">
+      <c r="Q4" s="15">
+        <v>0.26109650000000001</v>
+      </c>
+      <c r="R4" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S4" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T4" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U4" s="15">
+        <v>30</v>
+      </c>
+      <c r="V4" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" s="28" customFormat="1">
+      <c r="A5" s="28">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="29">
+        <v>0.1</v>
+      </c>
+      <c r="C5" s="28">
         <v>1.18</v>
       </c>
-      <c r="C5">
+      <c r="D5" s="28">
         <v>2.2029999999999998</v>
       </c>
-      <c r="G5">
+      <c r="H5" s="28">
         <v>2.2029999999999998</v>
       </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
+      <c r="I5" s="28">
+        <v>0</v>
+      </c>
+      <c r="J5" s="28">
+        <v>0</v>
+      </c>
+      <c r="K5" s="28">
         <v>1.2795499999999999E-4</v>
       </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
+      <c r="L5" s="28">
+        <v>0</v>
+      </c>
+      <c r="M5" s="28">
+        <v>0</v>
+      </c>
+      <c r="N5" s="28">
         <v>1.93</v>
       </c>
-      <c r="N5">
+      <c r="O5" s="28">
         <v>2.44</v>
       </c>
-    </row>
-    <row r="6" spans="1:14">
-      <c r="A6">
+      <c r="Q5" s="29">
+        <v>0.35967375000000001</v>
+      </c>
+      <c r="R5" s="29" t="s">
+        <v>100</v>
+      </c>
+      <c r="S5" s="29">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="T5" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="U5" s="29">
+        <v>3</v>
+      </c>
+      <c r="V5" s="29" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" s="28" customFormat="1">
+      <c r="A6" s="28">
+        <v>5</v>
+      </c>
+      <c r="B6" s="29">
+        <v>0.1</v>
+      </c>
+      <c r="C6" s="28">
         <v>1.127</v>
       </c>
-      <c r="C6">
+      <c r="D6" s="28">
         <v>2.0979999999999999</v>
       </c>
-      <c r="G6">
+      <c r="H6" s="28">
         <v>2.0979999999999999</v>
       </c>
-      <c r="H6">
+      <c r="I6" s="28">
         <v>1.6766474999999999E-2</v>
       </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
+      <c r="J6" s="28">
+        <v>0</v>
+      </c>
+      <c r="K6" s="28">
         <v>1.5726999999999999E-4</v>
       </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
+      <c r="L6" s="28">
+        <v>0</v>
+      </c>
+      <c r="M6" s="28">
+        <v>0</v>
+      </c>
+      <c r="N6" s="28">
         <v>2.0699999999999998</v>
       </c>
-      <c r="N6">
+      <c r="O6" s="28">
         <v>2.39</v>
       </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7">
+      <c r="Q6" s="29">
+        <v>0.377942893</v>
+      </c>
+      <c r="R6" s="29" t="s">
+        <v>100</v>
+      </c>
+      <c r="S6" s="29">
+        <v>5</v>
+      </c>
+      <c r="T6" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="U6" s="29">
+        <v>3</v>
+      </c>
+      <c r="V6" s="29" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" s="28" customFormat="1">
+      <c r="A7" s="28">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="29">
+        <v>0.1</v>
+      </c>
+      <c r="C7" s="28">
         <v>1.0980000000000001</v>
       </c>
-      <c r="C7">
+      <c r="D7" s="28">
         <v>2.0550000000000002</v>
       </c>
-      <c r="G7">
+      <c r="H7" s="28">
         <v>2.0550000000000002</v>
       </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
+      <c r="I7" s="28">
+        <v>0</v>
+      </c>
+      <c r="J7" s="28">
+        <v>0</v>
+      </c>
+      <c r="K7" s="28">
         <v>1.3422099999999999E-4</v>
       </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
+      <c r="L7" s="28">
+        <v>0</v>
+      </c>
+      <c r="M7" s="28">
+        <v>0</v>
+      </c>
+      <c r="N7" s="28">
         <v>1.97</v>
       </c>
-      <c r="N7">
+      <c r="O7" s="28">
         <v>2.1800000000000002</v>
       </c>
-    </row>
-    <row r="8" spans="1:14">
+      <c r="Q7" s="29">
+        <v>0.33645671399999999</v>
+      </c>
+      <c r="R7" s="29" t="s">
+        <v>100</v>
+      </c>
+      <c r="S7" s="29">
+        <v>5</v>
+      </c>
+      <c r="T7" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="U7" s="29">
+        <v>3</v>
+      </c>
+      <c r="V7" s="29" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C8">
         <v>1.51</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>0.308</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>0.308</v>
       </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
       <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
         <v>7.5614127000000003E-2</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>1.7982350000000001E-2</v>
       </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
         <v>3.4660000000000002</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>3.6160000000000001</v>
       </c>
-    </row>
-    <row r="9" spans="1:14">
+      <c r="Q8" s="15">
+        <v>0.209333929</v>
+      </c>
+      <c r="R8" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S8" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T8" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U8" s="15">
+        <v>30</v>
+      </c>
+      <c r="V8" s="15" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C9">
         <v>1.5109999999999999</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <v>0.308</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>0.308</v>
       </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
       <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
         <v>4.9087042999999997E-2</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>1.38432E-2</v>
       </c>
-      <c r="K9">
-        <v>0</v>
-      </c>
       <c r="L9">
         <v>0</v>
       </c>
       <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9">
         <v>3.1360000000000001</v>
       </c>
-      <c r="N9">
+      <c r="O9">
         <v>3.5219999999999998</v>
       </c>
-    </row>
-    <row r="10" spans="1:14">
+      <c r="Q9" s="15">
+        <v>0.22151335699999999</v>
+      </c>
+      <c r="R9" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S9" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T9" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U9" s="15">
+        <v>30</v>
+      </c>
+      <c r="V9" s="15" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C10">
         <v>1.4890000000000001</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <v>0.30399999999999999</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>0.30399999999999999</v>
       </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
       <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
         <v>6.6037847999999996E-2</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>1.602926E-2</v>
       </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
         <v>3.161</v>
       </c>
-      <c r="N10">
+      <c r="O10">
         <v>3.8239999999999998</v>
       </c>
-    </row>
-    <row r="11" spans="1:14">
+      <c r="Q10" s="15">
+        <v>0.24587221400000001</v>
+      </c>
+      <c r="R10" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S10" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T10" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U10" s="15">
+        <v>30</v>
+      </c>
+      <c r="V10" s="15" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="15">
+        <v>0.13</v>
+      </c>
+      <c r="C11">
         <v>2.0190000000000001</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <v>0.41499999999999998</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>0.41499999999999998</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>0.14387805000000001</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>0.23128044</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>2.4418572999999999E-2</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>7.3894399999999995E-4</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <v>4.2122905000000002E-2</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <v>5.51</v>
       </c>
-      <c r="N11">
+      <c r="O11">
         <v>5.2519999999999998</v>
       </c>
-    </row>
-    <row r="12" spans="1:14">
+      <c r="Q11" s="15">
+        <v>0.30372450000000001</v>
+      </c>
+      <c r="R11" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S11" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T11" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U11" s="15">
+        <v>30</v>
+      </c>
+      <c r="V11" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="15">
+        <v>0.13</v>
+      </c>
+      <c r="C12">
         <v>2.0590000000000002</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <v>0.42499999999999999</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>0.42499999999999999</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>0.13916811300000001</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>0.22761730999999999</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>2.5077986E-2</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>2.152588E-3</v>
       </c>
-      <c r="L12">
+      <c r="M12">
         <v>3.3899711999999999E-2</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <v>5.3739999999999997</v>
       </c>
-      <c r="N12">
+      <c r="O12">
         <v>4.5460000000000003</v>
       </c>
-    </row>
-    <row r="13" spans="1:14">
+      <c r="Q12" s="15">
+        <v>0.25690982099999998</v>
+      </c>
+      <c r="R12" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S12" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T12" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U12" s="15">
+        <v>30</v>
+      </c>
+      <c r="V12" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="15">
+        <v>0.13</v>
+      </c>
+      <c r="C13">
         <v>2.1349999999999998</v>
       </c>
-      <c r="C13">
+      <c r="D13">
         <v>0.438</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <v>0.438</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>0.13267562499999999</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>0.25727792100000002</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>2.6121129999999999E-2</v>
       </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
       <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
         <v>4.1071206999999998E-2</v>
       </c>
-      <c r="M13">
+      <c r="N13">
         <v>5.3019999999999996</v>
       </c>
-      <c r="N13">
+      <c r="O13">
         <v>5.07</v>
       </c>
-    </row>
-    <row r="14" spans="1:14">
+      <c r="Q13" s="15">
+        <v>0.26642500000000002</v>
+      </c>
+      <c r="R13" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S13" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T13" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U13" s="15">
+        <v>30</v>
+      </c>
+      <c r="V13" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22">
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="15">
+        <v>0.18</v>
+      </c>
+      <c r="C14">
         <v>3.266</v>
       </c>
-      <c r="C14">
+      <c r="D14">
         <v>0.66900000000000004</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>0.66900000000000004</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>1.2813869950000001</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>0.18048138799999999</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>3.2745818000000003E-2</v>
       </c>
-      <c r="K14">
-        <v>0</v>
-      </c>
       <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
         <v>5.6452840000000004E-3</v>
       </c>
-      <c r="M14">
+      <c r="N14">
         <v>7.2619999999999996</v>
       </c>
-      <c r="N14">
+      <c r="O14">
         <v>5.42</v>
       </c>
-    </row>
-    <row r="15" spans="1:14">
+      <c r="Q14" s="15">
+        <v>0.28926142900000001</v>
+      </c>
+      <c r="R14" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S14" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T14" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U14" s="15">
+        <v>30</v>
+      </c>
+      <c r="V14" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22">
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="15">
+        <v>0.18</v>
+      </c>
+      <c r="C15">
         <v>3.202</v>
       </c>
-      <c r="C15">
+      <c r="D15">
         <v>0.65900000000000003</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>0.65900000000000003</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <v>1.4870797280000001</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <v>0.41515672300000001</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>3.1272250000000001E-2</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <v>2.6969479999999998E-3</v>
       </c>
-      <c r="L15">
+      <c r="M15">
         <v>1.6418242E-2</v>
       </c>
-      <c r="M15">
+      <c r="N15">
         <v>7.3049999999999997</v>
       </c>
-      <c r="N15">
+      <c r="O15">
         <v>6.0170000000000003</v>
       </c>
-    </row>
-    <row r="16" spans="1:14">
+      <c r="Q15" s="15">
+        <v>0.28202989299999998</v>
+      </c>
+      <c r="R15" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S15" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T15" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U15" s="15">
+        <v>30</v>
+      </c>
+      <c r="V15" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22">
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="15">
+        <v>0.18</v>
+      </c>
+      <c r="C16">
         <v>2.83</v>
       </c>
-      <c r="C16">
+      <c r="D16">
         <v>0.58099999999999996</v>
       </c>
-      <c r="G16">
+      <c r="H16">
         <v>0.58099999999999996</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>1.069367508</v>
       </c>
-      <c r="I16">
+      <c r="J16">
         <v>0.18424942899999999</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>2.652065E-2</v>
       </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
       <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
         <v>1.5674206999999999E-2</v>
       </c>
-      <c r="M16">
+      <c r="N16">
         <v>6.2510000000000003</v>
       </c>
-      <c r="N16">
+      <c r="O16">
         <v>5.2640000000000002</v>
       </c>
-    </row>
-    <row r="17" spans="1:14">
+      <c r="Q16" s="15">
+        <v>0.288119607</v>
+      </c>
+      <c r="R16" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S16" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T16" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U16" s="15">
+        <v>30</v>
+      </c>
+      <c r="V16" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22">
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="15">
+        <v>0.3</v>
+      </c>
+      <c r="C17">
         <v>7.9909999999999997</v>
       </c>
-      <c r="C17">
+      <c r="D17">
         <v>1.6479999999999999</v>
       </c>
-      <c r="G17">
+      <c r="H17">
         <v>1.6479999999999999</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <v>7.0441347099999998</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <v>0.31251037799999998</v>
       </c>
-      <c r="J17">
+      <c r="K17">
         <v>5.1692219999999997E-2</v>
       </c>
-      <c r="K17">
+      <c r="L17">
         <v>1.1339925000000001E-2</v>
       </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
       <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17">
         <v>14.086</v>
       </c>
-      <c r="N17">
+      <c r="O17">
         <v>8.3010000000000002</v>
       </c>
-    </row>
-    <row r="18" spans="1:14">
+      <c r="Q17" s="15">
+        <v>0.42247392900000003</v>
+      </c>
+      <c r="R17" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S17" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T17" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U17" s="15">
+        <v>30</v>
+      </c>
+      <c r="V17" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22">
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="15">
+        <v>0.3</v>
+      </c>
+      <c r="C18">
         <v>8.2759999999999998</v>
       </c>
-      <c r="C18">
+      <c r="D18">
         <v>1.6950000000000001</v>
       </c>
-      <c r="G18">
+      <c r="H18">
         <v>1.6950000000000001</v>
       </c>
-      <c r="H18">
+      <c r="I18">
         <v>6.6847254490000001</v>
       </c>
-      <c r="I18">
+      <c r="J18">
         <v>0.27229536399999998</v>
       </c>
-      <c r="J18">
+      <c r="K18">
         <v>4.4478275999999997E-2</v>
       </c>
-      <c r="K18">
+      <c r="L18">
         <v>3.4668667E-2</v>
       </c>
-      <c r="L18">
-        <v>0</v>
-      </c>
       <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18">
         <v>15.111000000000001</v>
       </c>
-      <c r="N18">
+      <c r="O18">
         <v>8.3870000000000005</v>
       </c>
-    </row>
-    <row r="19" spans="1:14">
+      <c r="Q18" s="15">
+        <v>0.42133210700000001</v>
+      </c>
+      <c r="R18" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S18" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T18" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U18" s="15">
+        <v>30</v>
+      </c>
+      <c r="V18" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22">
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="15">
+        <v>0.3</v>
+      </c>
+      <c r="C19">
         <v>8.9320000000000004</v>
       </c>
-      <c r="C19">
+      <c r="D19">
         <v>1.8660000000000001</v>
       </c>
-      <c r="G19">
+      <c r="H19">
         <v>1.8660000000000001</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <v>8.2124218889999998</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <v>0.61718923199999998</v>
       </c>
-      <c r="J19">
+      <c r="K19">
         <v>6.4337543999999997E-2</v>
       </c>
-      <c r="K19">
+      <c r="L19">
         <v>2.9481279999999999E-2</v>
       </c>
-      <c r="L19">
-        <v>0</v>
-      </c>
       <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19">
         <v>16.956</v>
       </c>
-      <c r="N19">
+      <c r="O19">
         <v>9.34</v>
       </c>
-    </row>
-    <row r="20" spans="1:14">
+      <c r="Q19" s="15">
+        <v>0.39963749999999998</v>
+      </c>
+      <c r="R19" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S19" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T19" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U19" s="15">
+        <v>30</v>
+      </c>
+      <c r="V19" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22">
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="15">
+        <v>0.35</v>
+      </c>
+      <c r="C20">
         <v>12.936999999999999</v>
       </c>
-      <c r="C20">
+      <c r="D20">
         <v>2.7120000000000002</v>
       </c>
-      <c r="G20">
+      <c r="H20">
         <v>2.7120000000000002</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <v>11.927306959999999</v>
       </c>
-      <c r="I20">
+      <c r="J20">
         <v>0.47269426599999997</v>
       </c>
-      <c r="J20">
+      <c r="K20">
         <v>8.9757966999999994E-2</v>
       </c>
-      <c r="K20">
+      <c r="L20">
         <v>3.5944587E-2</v>
       </c>
-      <c r="L20">
-        <v>0</v>
-      </c>
       <c r="M20">
+        <v>0</v>
+      </c>
+      <c r="N20">
         <v>20.902000000000001</v>
       </c>
-      <c r="N20">
+      <c r="O20">
         <v>12.682</v>
       </c>
-    </row>
-    <row r="21" spans="1:14">
+      <c r="Q20" s="15">
+        <v>0.48415467400000001</v>
+      </c>
+      <c r="R20" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S20" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T20" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U20" s="15">
+        <v>30</v>
+      </c>
+      <c r="V20" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22">
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="15">
+        <v>0.35</v>
+      </c>
+      <c r="C21">
         <v>13.23</v>
       </c>
-      <c r="C21">
+      <c r="D21">
         <v>2.786</v>
       </c>
-      <c r="G21">
+      <c r="H21">
         <v>2.786</v>
       </c>
-      <c r="H21">
+      <c r="I21">
         <v>12.12470377</v>
       </c>
-      <c r="I21">
+      <c r="J21">
         <v>0.63692599999999999</v>
       </c>
-      <c r="J21">
+      <c r="K21">
         <v>0.104193063</v>
       </c>
-      <c r="K21">
+      <c r="L21">
         <v>3.3770889999999998E-2</v>
       </c>
-      <c r="L21">
-        <v>0</v>
-      </c>
       <c r="M21">
+        <v>0</v>
+      </c>
+      <c r="N21">
         <v>21.082999999999998</v>
       </c>
-      <c r="N21">
+      <c r="O21">
         <v>12.353999999999999</v>
       </c>
-    </row>
-    <row r="22" spans="1:14">
+      <c r="Q21" s="15">
+        <v>0.48992198300000001</v>
+      </c>
+      <c r="R21" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S21" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T21" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U21" s="15">
+        <v>30</v>
+      </c>
+      <c r="V21" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22">
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="15">
+        <v>0.35</v>
+      </c>
+      <c r="C22">
         <v>13.096</v>
       </c>
-      <c r="C22">
+      <c r="D22">
         <v>2.742</v>
       </c>
-      <c r="G22">
+      <c r="H22">
         <v>2.742</v>
       </c>
-      <c r="H22">
+      <c r="I22">
         <v>11.84780602</v>
       </c>
-      <c r="I22">
+      <c r="J22">
         <v>0.47734259699999998</v>
       </c>
-      <c r="J22">
+      <c r="K22">
         <v>9.1823417000000004E-2</v>
       </c>
-      <c r="K22">
-        <v>0</v>
-      </c>
       <c r="L22">
         <v>0</v>
       </c>
       <c r="M22">
+        <v>0</v>
+      </c>
+      <c r="N22">
         <v>21.097999999999999</v>
       </c>
-      <c r="N22">
+      <c r="O22">
         <v>12.977</v>
       </c>
-    </row>
-    <row r="23" spans="1:14">
+      <c r="Q22" s="15">
+        <v>0.50886425499999999</v>
+      </c>
+      <c r="R22" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="S22" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="T22" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U22" s="15">
+        <v>30</v>
+      </c>
+      <c r="V22" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22">
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C23">
         <v>0.82699999999999996</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>0.747</v>
       </c>
-      <c r="G23">
+      <c r="H23">
         <v>1.4930000000000001</v>
       </c>
-      <c r="H23">
-        <v>0</v>
-      </c>
       <c r="I23">
         <v>0</v>
       </c>
       <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
         <v>8.7561730000000008E-3</v>
       </c>
-      <c r="K23">
-        <v>0</v>
-      </c>
       <c r="L23">
         <v>0</v>
       </c>
       <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="N23">
         <v>2.7690000000000001</v>
       </c>
-      <c r="N23">
+      <c r="O23">
         <v>2.4500000000000002</v>
       </c>
-    </row>
-    <row r="24" spans="1:14">
+      <c r="Q23" s="15">
+        <v>0.49783414300000001</v>
+      </c>
+      <c r="R23" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="S23" s="15">
+        <v>5.53</v>
+      </c>
+      <c r="T23" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="U23" s="15">
+        <v>5</v>
+      </c>
+      <c r="V23" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22">
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C24">
         <v>0.78800000000000003</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>0.71199999999999997</v>
       </c>
-      <c r="G24">
+      <c r="H24">
         <v>1.423</v>
       </c>
-      <c r="H24">
-        <v>0</v>
-      </c>
       <c r="I24">
         <v>0</v>
       </c>
       <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
         <v>5.5182690000000001E-3</v>
       </c>
-      <c r="K24">
-        <v>0</v>
-      </c>
       <c r="L24">
         <v>0</v>
       </c>
       <c r="M24">
+        <v>0</v>
+      </c>
+      <c r="N24">
         <v>2.7170000000000001</v>
       </c>
-      <c r="N24">
+      <c r="O24">
         <v>2.3530000000000002</v>
       </c>
-    </row>
-    <row r="25" spans="1:14">
+      <c r="Q24" s="15">
+        <v>0.58385135700000002</v>
+      </c>
+      <c r="R24" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="S24" s="15">
+        <v>5.53</v>
+      </c>
+      <c r="T24" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="U24" s="15">
+        <v>5</v>
+      </c>
+      <c r="V24" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22">
       <c r="A25">
         <v>24</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C25">
         <v>0.76700000000000002</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>0.69099999999999995</v>
       </c>
-      <c r="G25">
+      <c r="H25">
         <v>1.3819999999999999</v>
       </c>
-      <c r="H25">
-        <v>0</v>
-      </c>
       <c r="I25">
         <v>0</v>
       </c>
       <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
         <v>1.9902549999999998E-3</v>
       </c>
-      <c r="K25">
-        <v>0</v>
-      </c>
       <c r="L25">
         <v>0</v>
       </c>
       <c r="M25">
+        <v>0</v>
+      </c>
+      <c r="N25">
         <v>2.5739999999999998</v>
       </c>
-      <c r="N25">
+      <c r="O25">
         <v>2.25</v>
       </c>
-    </row>
-    <row r="26" spans="1:14">
+      <c r="Q25" s="15">
+        <v>0.59412774999999995</v>
+      </c>
+      <c r="R25" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="S25" s="15">
+        <v>5.53</v>
+      </c>
+      <c r="T25" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="U25" s="15">
+        <v>5</v>
+      </c>
+      <c r="V25" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22">
       <c r="A26">
         <v>25</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C26">
         <v>0.80700000000000005</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <v>4.92</v>
       </c>
-      <c r="G26">
+      <c r="H26">
         <v>9.8390000000000004</v>
       </c>
-      <c r="H26">
-        <v>0</v>
-      </c>
       <c r="I26">
         <v>0</v>
       </c>
       <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
         <v>3.9436786000000001E-2</v>
       </c>
-      <c r="K26">
-        <v>0</v>
-      </c>
       <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="M26">
         <v>1.3630471999999999E-2</v>
       </c>
-      <c r="M26">
+      <c r="N26">
         <v>3.032</v>
       </c>
-      <c r="N26">
+      <c r="O26">
         <v>1.7749999999999999</v>
       </c>
-    </row>
-    <row r="27" spans="1:14">
+      <c r="Q26" s="15">
+        <v>0.510013571</v>
+      </c>
+      <c r="R26" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="S26" s="15">
+        <v>5.53</v>
+      </c>
+      <c r="T26" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="U26" s="15">
+        <v>3</v>
+      </c>
+      <c r="V26" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22">
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C27">
         <v>0.64900000000000002</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <v>3.9620000000000002</v>
       </c>
-      <c r="G27">
+      <c r="H27">
         <v>7.9240000000000004</v>
       </c>
-      <c r="H27">
-        <v>0</v>
-      </c>
       <c r="I27">
         <v>0</v>
       </c>
       <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
         <v>3.0460814999999999E-2</v>
       </c>
-      <c r="K27">
-        <v>0</v>
-      </c>
       <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27">
         <v>9.5061450000000006E-3</v>
       </c>
-      <c r="M27">
+      <c r="N27">
         <v>1.9590000000000001</v>
       </c>
-      <c r="N27">
+      <c r="O27">
         <v>1.623</v>
       </c>
-    </row>
-    <row r="28" spans="1:14">
+      <c r="Q27" s="15">
+        <v>0.29420932100000002</v>
+      </c>
+      <c r="R27" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="S27" s="15">
+        <v>5.53</v>
+      </c>
+      <c r="T27" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="U27" s="15">
+        <v>3</v>
+      </c>
+      <c r="V27" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22">
       <c r="A28">
         <v>27</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C28">
         <v>0.76500000000000001</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <v>4.6159999999999997</v>
       </c>
-      <c r="G28">
+      <c r="H28">
         <v>9.2319999999999993</v>
       </c>
-      <c r="H28">
-        <v>0</v>
-      </c>
       <c r="I28">
         <v>0</v>
       </c>
       <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
         <v>2.5119712999999998E-2</v>
       </c>
-      <c r="K28">
-        <v>0</v>
-      </c>
       <c r="L28">
         <v>0</v>
       </c>
       <c r="M28">
+        <v>0</v>
+      </c>
+      <c r="N28">
         <v>2.569</v>
       </c>
-      <c r="N28">
+      <c r="O28">
         <v>1.2909999999999999</v>
       </c>
-    </row>
-    <row r="29" spans="1:14">
+      <c r="Q28" s="15">
+        <v>0.358912536</v>
+      </c>
+      <c r="R28" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="S28" s="15">
+        <v>5.53</v>
+      </c>
+      <c r="T28" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="U28" s="15">
+        <v>3</v>
+      </c>
+      <c r="V28" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22">
       <c r="A29">
         <v>28</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C29">
         <v>1.381</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <v>0.158</v>
       </c>
-      <c r="G29">
+      <c r="H29">
         <v>0.317</v>
       </c>
-      <c r="H29">
+      <c r="I29">
         <v>1.8073279000000001E-2</v>
       </c>
-      <c r="I29">
+      <c r="J29">
         <v>7.8381013999999999E-2</v>
       </c>
-      <c r="J29">
+      <c r="K29">
         <v>0.86713414300000002</v>
       </c>
-      <c r="K29">
+      <c r="L29">
         <v>5.4564440000000004E-3</v>
       </c>
-      <c r="L29">
+      <c r="M29">
         <v>4.6616212999999997E-2</v>
       </c>
-      <c r="M29">
+      <c r="N29">
         <v>4.3209999999999997</v>
       </c>
-      <c r="N29">
+      <c r="O29">
         <v>3.883</v>
       </c>
-    </row>
-    <row r="30" spans="1:14">
+      <c r="Q29" s="15">
+        <v>0.20552785700000001</v>
+      </c>
+      <c r="R29" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="S29" s="15">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="T29" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U29" s="15">
+        <v>30</v>
+      </c>
+      <c r="V29" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22">
       <c r="A30">
         <v>29</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C30">
         <v>1.2589999999999999</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <v>0.14199999999999999</v>
       </c>
-      <c r="G30">
+      <c r="H30">
         <v>0.28399999999999997</v>
       </c>
-      <c r="H30">
-        <v>0</v>
-      </c>
       <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
         <v>3.4333113999999998E-2</v>
       </c>
-      <c r="J30">
+      <c r="K30">
         <v>0.69158415699999998</v>
       </c>
-      <c r="K30">
-        <v>0</v>
-      </c>
       <c r="L30">
+        <v>0</v>
+      </c>
+      <c r="M30">
         <v>4.5041784000000001E-2</v>
       </c>
-      <c r="M30">
+      <c r="N30">
         <v>3.93</v>
       </c>
-      <c r="N30">
+      <c r="O30">
         <v>3.3959999999999999</v>
       </c>
-    </row>
-    <row r="31" spans="1:14">
+      <c r="Q30" s="15">
+        <v>0.35282282100000001</v>
+      </c>
+      <c r="R30" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="S30" s="15">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="T30" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U30" s="15">
+        <v>30</v>
+      </c>
+      <c r="V30" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22">
       <c r="A31">
         <v>30</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C31">
         <v>1.3</v>
       </c>
-      <c r="D31">
+      <c r="E31">
         <v>0.14899999999999999</v>
       </c>
-      <c r="G31">
+      <c r="H31">
         <v>0.29799999999999999</v>
       </c>
-      <c r="H31">
-        <v>0</v>
-      </c>
       <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
         <v>7.6426068999999999E-2</v>
       </c>
-      <c r="J31">
+      <c r="K31">
         <v>0.84262339500000005</v>
       </c>
-      <c r="K31">
+      <c r="L31">
         <v>5.663179E-3</v>
       </c>
-      <c r="L31">
+      <c r="M31">
         <v>4.1991897E-2</v>
       </c>
-      <c r="M31">
+      <c r="N31">
         <v>4.077</v>
       </c>
-      <c r="N31">
+      <c r="O31">
         <v>3.3340000000000001</v>
       </c>
-    </row>
-    <row r="32" spans="1:14">
+      <c r="Q31" s="15">
+        <v>0.36195739300000002</v>
+      </c>
+      <c r="R31" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="S31" s="15">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="T31" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U31" s="15">
+        <v>30</v>
+      </c>
+      <c r="V31" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22">
       <c r="A32">
         <v>31</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C32">
         <v>1.4850000000000001</v>
       </c>
-      <c r="E32">
+      <c r="F32">
         <v>2.8620000000000001</v>
       </c>
-      <c r="G32">
+      <c r="H32">
         <v>2.8620000000000001</v>
       </c>
-      <c r="H32">
-        <v>0</v>
-      </c>
       <c r="I32">
         <v>0</v>
       </c>
       <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32">
         <v>6.3162172000000003E-2</v>
       </c>
-      <c r="K32">
-        <v>0</v>
-      </c>
       <c r="L32">
         <v>0</v>
       </c>
       <c r="M32">
+        <v>0</v>
+      </c>
+      <c r="N32">
         <v>5.7110000000000003</v>
       </c>
-      <c r="N32">
+      <c r="O32">
         <v>5.6040000000000001</v>
       </c>
-    </row>
-    <row r="33" spans="1:14">
+      <c r="Q32" s="15">
+        <v>0.425138179</v>
+      </c>
+      <c r="R32" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="S32" s="15">
+        <v>12.35</v>
+      </c>
+      <c r="T32" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="U32" s="15">
+        <v>3</v>
+      </c>
+      <c r="V32" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22">
       <c r="A33">
         <v>32</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C33">
         <v>1.6</v>
       </c>
-      <c r="E33">
+      <c r="F33">
         <v>3.0840000000000001</v>
       </c>
-      <c r="G33">
+      <c r="H33">
         <v>3.0840000000000001</v>
       </c>
-      <c r="H33">
-        <v>0</v>
-      </c>
       <c r="I33">
         <v>0</v>
       </c>
       <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
         <v>7.4209667000000007E-2</v>
       </c>
-      <c r="K33">
-        <v>0</v>
-      </c>
       <c r="L33">
         <v>0</v>
       </c>
       <c r="M33">
+        <v>0</v>
+      </c>
+      <c r="N33">
         <v>6.0389999999999997</v>
       </c>
-      <c r="N33">
+      <c r="O33">
         <v>5.8689999999999998</v>
       </c>
-    </row>
-    <row r="34" spans="1:14">
+      <c r="Q33" s="15">
+        <v>0.52028996400000005</v>
+      </c>
+      <c r="R33" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="S33" s="15">
+        <v>12.35</v>
+      </c>
+      <c r="T33" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="U33" s="15">
+        <v>3</v>
+      </c>
+      <c r="V33" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22">
       <c r="A34">
         <v>33</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C34">
         <v>1.4350000000000001</v>
       </c>
-      <c r="E34">
+      <c r="F34">
         <v>2.7629999999999999</v>
       </c>
-      <c r="G34">
+      <c r="H34">
         <v>2.7629999999999999</v>
       </c>
-      <c r="H34">
-        <v>0</v>
-      </c>
       <c r="I34">
         <v>0</v>
       </c>
       <c r="J34">
+        <v>0</v>
+      </c>
+      <c r="K34">
         <v>7.4921513999999995E-2</v>
       </c>
-      <c r="K34">
-        <v>0</v>
-      </c>
       <c r="L34">
         <v>0</v>
       </c>
       <c r="M34">
+        <v>0</v>
+      </c>
+      <c r="N34">
         <v>5.32</v>
       </c>
-      <c r="N34">
+      <c r="O34">
         <v>5.0789999999999997</v>
       </c>
-    </row>
-    <row r="35" spans="1:14">
+      <c r="Q34" s="15">
+        <v>0.452161286</v>
+      </c>
+      <c r="R34" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="S34" s="15">
+        <v>12.35</v>
+      </c>
+      <c r="T34" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="U34" s="15">
+        <v>3</v>
+      </c>
+      <c r="V34" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22">
       <c r="A35">
         <v>34</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C35">
         <v>1.6779999999999999</v>
       </c>
-      <c r="E35">
+      <c r="F35">
         <v>0.33400000000000002</v>
       </c>
-      <c r="G35">
+      <c r="H35">
         <v>0.33400000000000002</v>
       </c>
-      <c r="H35">
-        <v>0</v>
-      </c>
       <c r="I35">
         <v>0</v>
       </c>
       <c r="J35">
+        <v>0</v>
+      </c>
+      <c r="K35">
         <v>0.27117874199999997</v>
       </c>
-      <c r="K35">
-        <v>0</v>
-      </c>
       <c r="L35">
         <v>0</v>
       </c>
       <c r="M35">
+        <v>0</v>
+      </c>
+      <c r="N35">
         <v>5.7240000000000002</v>
       </c>
-      <c r="N35">
+      <c r="O35">
         <v>5.9080000000000004</v>
       </c>
-    </row>
-    <row r="36" spans="1:14">
+      <c r="Q35" s="15">
+        <v>0.41790664300000002</v>
+      </c>
+      <c r="R35" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="S35" s="15">
+        <v>1.24</v>
+      </c>
+      <c r="T35" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U35" s="15">
+        <v>30</v>
+      </c>
+      <c r="V35" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22">
       <c r="A36">
         <v>35</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C36">
         <v>1.6930000000000001</v>
       </c>
-      <c r="E36">
+      <c r="F36">
         <v>0.33700000000000002</v>
       </c>
-      <c r="G36">
+      <c r="H36">
         <v>0.33700000000000002</v>
       </c>
-      <c r="H36">
-        <v>0</v>
-      </c>
       <c r="I36">
         <v>0</v>
       </c>
       <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
         <v>0.30716928599999999</v>
       </c>
-      <c r="K36">
-        <v>0</v>
-      </c>
       <c r="L36">
         <v>0</v>
       </c>
       <c r="M36">
+        <v>0</v>
+      </c>
+      <c r="N36">
         <v>5.9720000000000004</v>
       </c>
-      <c r="N36">
+      <c r="O36">
         <v>5.29</v>
       </c>
-    </row>
-    <row r="37" spans="1:14">
+      <c r="Q36" s="15">
+        <v>0.37870410700000001</v>
+      </c>
+      <c r="R36" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="S36" s="15">
+        <v>1.24</v>
+      </c>
+      <c r="T36" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U36" s="15">
+        <v>30</v>
+      </c>
+      <c r="V36" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22">
       <c r="A37">
         <v>36</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C37">
         <v>1.647</v>
       </c>
-      <c r="E37">
+      <c r="F37">
         <v>0.32700000000000001</v>
       </c>
-      <c r="G37">
+      <c r="H37">
         <v>0.32700000000000001</v>
       </c>
-      <c r="H37">
-        <v>0</v>
-      </c>
       <c r="I37">
         <v>0</v>
       </c>
       <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
         <v>0.20397084300000001</v>
       </c>
-      <c r="K37">
-        <v>0</v>
-      </c>
       <c r="L37">
         <v>0</v>
       </c>
       <c r="M37">
+        <v>0</v>
+      </c>
+      <c r="N37">
         <v>6.1310000000000002</v>
       </c>
-      <c r="N37">
+      <c r="O37">
         <v>5.69</v>
       </c>
-    </row>
-    <row r="38" spans="1:14">
+      <c r="Q37" s="15">
+        <v>0.39887628600000002</v>
+      </c>
+      <c r="R37" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="S37" s="15">
+        <v>1.24</v>
+      </c>
+      <c r="T37" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U37" s="15">
+        <v>30</v>
+      </c>
+      <c r="V37" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22">
       <c r="A38">
         <v>37</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C38">
         <v>1.4790000000000001</v>
-      </c>
-      <c r="F38">
-        <v>2.919</v>
       </c>
       <c r="G38">
         <v>2.919</v>
       </c>
       <c r="H38">
+        <v>2.919</v>
+      </c>
+      <c r="I38">
         <v>6.4434642E-2</v>
       </c>
-      <c r="I38">
-        <v>0</v>
-      </c>
       <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
         <v>0.16559933199999999</v>
       </c>
-      <c r="K38">
-        <v>0</v>
-      </c>
       <c r="L38">
+        <v>0</v>
+      </c>
+      <c r="M38">
         <v>4.8736990000000004E-3</v>
       </c>
-      <c r="M38">
+      <c r="N38">
         <v>4.7869999999999999</v>
       </c>
-      <c r="N38">
+      <c r="O38">
         <v>4.5609999999999999</v>
       </c>
-    </row>
-    <row r="39" spans="1:14">
+      <c r="Q38" s="15">
+        <v>0.32085182099999998</v>
+      </c>
+      <c r="R38" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="S38" s="15">
+        <v>9.81</v>
+      </c>
+      <c r="T38" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="U38" s="15">
+        <v>3</v>
+      </c>
+      <c r="V38" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22">
       <c r="A39">
         <v>38</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C39">
         <v>1.633</v>
-      </c>
-      <c r="F39">
-        <v>3.2</v>
       </c>
       <c r="G39">
         <v>3.2</v>
       </c>
       <c r="H39">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="I39">
         <v>0</v>
       </c>
       <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
         <v>0.156217087</v>
       </c>
-      <c r="K39">
-        <v>0</v>
-      </c>
       <c r="L39">
         <v>0</v>
       </c>
       <c r="M39">
+        <v>0</v>
+      </c>
+      <c r="N39">
         <v>5.1379999999999999</v>
       </c>
-      <c r="N39">
+      <c r="O39">
         <v>4.9089999999999998</v>
       </c>
-    </row>
-    <row r="40" spans="1:14">
+      <c r="Q39" s="15">
+        <v>0.41866785699999998</v>
+      </c>
+      <c r="R39" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="S39" s="15">
+        <v>9.81</v>
+      </c>
+      <c r="T39" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="U39" s="15">
+        <v>3</v>
+      </c>
+      <c r="V39" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22">
       <c r="A40">
         <v>39</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C40">
         <v>1.571</v>
-      </c>
-      <c r="F40">
-        <v>3.0830000000000002</v>
       </c>
       <c r="G40">
         <v>3.0830000000000002</v>
       </c>
       <c r="H40">
+        <v>3.0830000000000002</v>
+      </c>
+      <c r="I40">
         <v>6.4504826000000001E-2</v>
       </c>
-      <c r="I40">
-        <v>0</v>
-      </c>
       <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
         <v>0.15037355499999999</v>
       </c>
-      <c r="K40">
-        <v>0</v>
-      </c>
       <c r="L40">
+        <v>0</v>
+      </c>
+      <c r="M40">
         <v>5.596462E-3</v>
       </c>
-      <c r="M40">
+      <c r="N40">
         <v>4.9610000000000003</v>
       </c>
-      <c r="N40">
+      <c r="O40">
         <v>4.5490000000000004</v>
       </c>
-    </row>
-    <row r="41" spans="1:14">
+      <c r="Q40" s="15">
+        <v>0.33150882100000001</v>
+      </c>
+      <c r="R40" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="S40" s="15">
+        <v>9.81</v>
+      </c>
+      <c r="T40" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="U40" s="15">
+        <v>3</v>
+      </c>
+      <c r="V40" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22">
       <c r="A41">
         <v>40</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C41">
         <v>1.4510000000000001</v>
-      </c>
-      <c r="F41">
-        <v>0.29199999999999998</v>
       </c>
       <c r="G41">
         <v>0.29199999999999998</v>
       </c>
       <c r="H41">
+        <v>0.29199999999999998</v>
+      </c>
+      <c r="I41">
         <v>0.16597783599999999</v>
       </c>
-      <c r="I41">
+      <c r="J41">
         <v>6.6479359000000002E-2</v>
       </c>
-      <c r="J41">
+      <c r="K41">
         <v>0.60819290000000004</v>
       </c>
-      <c r="K41">
-        <v>0</v>
-      </c>
       <c r="L41">
+        <v>0</v>
+      </c>
+      <c r="M41">
         <v>2.5725250000000002E-2</v>
       </c>
-      <c r="M41">
+      <c r="N41">
         <v>4.18</v>
       </c>
-      <c r="N41">
+      <c r="O41">
         <v>4.0129999999999999</v>
       </c>
-    </row>
-    <row r="42" spans="1:14">
+      <c r="Q41" s="15">
+        <v>0.43998185699999998</v>
+      </c>
+      <c r="R41" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="S41" s="15">
+        <v>0.98</v>
+      </c>
+      <c r="T41" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U41" s="15">
+        <v>30</v>
+      </c>
+      <c r="V41" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22">
       <c r="A42">
         <v>41</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C42">
         <v>1.7090000000000001</v>
-      </c>
-      <c r="F42">
-        <v>0.33900000000000002</v>
       </c>
       <c r="G42">
         <v>0.33900000000000002</v>
       </c>
       <c r="H42">
+        <v>0.33900000000000002</v>
+      </c>
+      <c r="I42">
         <v>6.0174350000000001E-2</v>
       </c>
-      <c r="I42">
+      <c r="J42">
         <v>7.8079274000000004E-2</v>
       </c>
-      <c r="J42">
+      <c r="K42">
         <v>0.66867871400000001</v>
       </c>
-      <c r="K42">
-        <v>0</v>
-      </c>
       <c r="L42">
+        <v>0</v>
+      </c>
+      <c r="M42">
         <v>3.5868012999999997E-2</v>
       </c>
-      <c r="M42">
+      <c r="N42">
         <v>4.9020000000000001</v>
       </c>
-      <c r="N42">
+      <c r="O42">
         <v>4.45</v>
       </c>
-    </row>
-    <row r="43" spans="1:14">
+      <c r="Q42" s="15">
+        <v>0.448355214</v>
+      </c>
+      <c r="R42" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="S42" s="15">
+        <v>0.98</v>
+      </c>
+      <c r="T42" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U42" s="15">
+        <v>30</v>
+      </c>
+      <c r="V42" s="15" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22">
       <c r="A43">
         <v>42</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="C43">
         <v>1.6220000000000001</v>
-      </c>
-      <c r="F43">
-        <v>0.32900000000000001</v>
       </c>
       <c r="G43">
         <v>0.32900000000000001</v>
       </c>
       <c r="H43">
+        <v>0.32900000000000001</v>
+      </c>
+      <c r="I43">
         <v>0.18362290100000001</v>
       </c>
-      <c r="I43">
+      <c r="J43">
         <v>0.16825845</v>
       </c>
-      <c r="J43">
+      <c r="K43">
         <v>0.92271634599999997</v>
       </c>
-      <c r="K43">
-        <v>0</v>
-      </c>
       <c r="L43">
+        <v>0</v>
+      </c>
+      <c r="M43">
         <v>4.8272586999999999E-2</v>
       </c>
-      <c r="M43">
+      <c r="N43">
         <v>4.5620000000000003</v>
       </c>
-      <c r="N43">
+      <c r="O43">
         <v>4.2300000000000004</v>
+      </c>
+      <c r="Q43" s="15">
+        <v>0.42361575000000001</v>
+      </c>
+      <c r="R43" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="S43" s="15">
+        <v>0.98</v>
+      </c>
+      <c r="T43" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U43" s="15">
+        <v>30</v>
+      </c>
+      <c r="V43" s="15" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: add more analysis
</commit_message>
<xml_diff>
--- a/data/proteomics/physiology_collection.xlsx
+++ b/data/proteomics/physiology_collection.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10313"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Documents/GitHub/De-nevo-protein-3D-structure-yeast/data/proteomics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5066DF8-4453-A044-86EF-EF08044830BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13969006-75B9-A247-900C-F5202197DEF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2780" yWindow="500" windowWidth="32900" windowHeight="21440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1440" windowWidth="26880" windowHeight="15220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$T$1:$T$77</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Supplementary File 1e vip'!$T$1:$T$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Supplementary File 1e vip'!$B$1:$B$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -5003,6 +5003,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:V43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
@@ -5082,7 +5083,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:22">
+    <row r="2" spans="1:22" hidden="1">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5138,7 +5139,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="3" spans="1:22">
+    <row r="3" spans="1:22" hidden="1">
       <c r="A3">
         <v>2</v>
       </c>
@@ -5194,7 +5195,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:22">
+    <row r="4" spans="1:22" hidden="1">
       <c r="A4">
         <v>3</v>
       </c>
@@ -5586,7 +5587,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="11" spans="1:22">
+    <row r="11" spans="1:22" hidden="1">
       <c r="A11">
         <v>10</v>
       </c>
@@ -5642,7 +5643,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="12" spans="1:22">
+    <row r="12" spans="1:22" hidden="1">
       <c r="A12">
         <v>11</v>
       </c>
@@ -5698,7 +5699,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:22">
+    <row r="13" spans="1:22" hidden="1">
       <c r="A13">
         <v>12</v>
       </c>
@@ -5754,7 +5755,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="14" spans="1:22">
+    <row r="14" spans="1:22" hidden="1">
       <c r="A14">
         <v>13</v>
       </c>
@@ -5810,7 +5811,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="15" spans="1:22">
+    <row r="15" spans="1:22" hidden="1">
       <c r="A15">
         <v>14</v>
       </c>
@@ -5866,7 +5867,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="16" spans="1:22">
+    <row r="16" spans="1:22" hidden="1">
       <c r="A16">
         <v>15</v>
       </c>
@@ -5922,7 +5923,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="17" spans="1:22">
+    <row r="17" spans="1:22" hidden="1">
       <c r="A17">
         <v>16</v>
       </c>
@@ -5978,7 +5979,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="18" spans="1:22">
+    <row r="18" spans="1:22" hidden="1">
       <c r="A18">
         <v>17</v>
       </c>
@@ -6034,7 +6035,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="19" spans="1:22">
+    <row r="19" spans="1:22" hidden="1">
       <c r="A19">
         <v>18</v>
       </c>
@@ -6090,7 +6091,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="20" spans="1:22">
+    <row r="20" spans="1:22" hidden="1">
       <c r="A20">
         <v>19</v>
       </c>
@@ -6146,7 +6147,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="21" spans="1:22">
+    <row r="21" spans="1:22" hidden="1">
       <c r="A21">
         <v>20</v>
       </c>
@@ -6202,7 +6203,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="22" spans="1:22">
+    <row r="22" spans="1:22" hidden="1">
       <c r="A22">
         <v>21</v>
       </c>
@@ -7435,6 +7436,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B1:B43" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="0.1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: refine the repo
</commit_message>
<xml_diff>
--- a/data/proteomics/physiology_collection.xlsx
+++ b/data/proteomics/physiology_collection.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10313"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Documents/GitHub/De-nevo-protein-3D-structure-yeast/data/proteomics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13969006-75B9-A247-900C-F5202197DEF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFD3D75D-BE95-5540-8EF8-954FC8521231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1440" windowWidth="26880" windowHeight="15220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1440" windowWidth="26060" windowHeight="15220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -958,7 +958,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1006,11 +1006,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1027,6 +1022,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="38" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4429,17 +4427,17 @@
         <v>0.42361575000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:24" s="26" customFormat="1">
-      <c r="A48" s="24" t="s">
+    <row r="48" spans="1:24" s="23" customFormat="1">
+      <c r="A48" s="21" t="s">
         <v>61</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C48" s="25">
+      <c r="C48" s="22">
         <v>0.1</v>
       </c>
-      <c r="Q48" s="27"/>
+      <c r="Q48" s="24"/>
     </row>
     <row r="49" spans="1:17" s="7" customFormat="1">
       <c r="A49" s="4" t="s">
@@ -4682,22 +4680,21 @@
       <c r="C69" s="19">
         <v>2.7E-2</v>
       </c>
-      <c r="D69" s="20">
+      <c r="D69" s="27">
         <v>-0.33700000000000002</v>
       </c>
-      <c r="E69" s="20">
+      <c r="E69" s="27">
         <v>-0.151308114750691</v>
       </c>
-      <c r="J69" s="20">
-        <v>0</v>
-      </c>
-      <c r="O69" s="20">
+      <c r="J69" s="27">
+        <v>0</v>
+      </c>
+      <c r="O69" s="27">
         <v>0.878</v>
       </c>
-      <c r="P69" s="21">
+      <c r="P69" s="20">
         <v>0.86358170086251695</v>
       </c>
-      <c r="Q69" s="22"/>
       <c r="R69" s="19" t="s">
         <v>100</v>
       </c>
@@ -4708,291 +4705,283 @@
         <v>0.29899999999999999</v>
       </c>
     </row>
-    <row r="70" spans="1:24" s="21" customFormat="1">
+    <row r="70" spans="1:24" s="20" customFormat="1">
       <c r="A70" s="9" t="s">
         <v>82</v>
       </c>
       <c r="B70" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C70" s="21">
+      <c r="C70" s="20">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="D70" s="20">
+      <c r="D70" s="27">
         <v>-0.52300000000000002</v>
       </c>
-      <c r="E70" s="20">
+      <c r="E70" s="27">
         <v>-0.22220072795676099</v>
       </c>
-      <c r="J70" s="20">
-        <v>0</v>
-      </c>
-      <c r="O70" s="20">
+      <c r="J70" s="27">
+        <v>0</v>
+      </c>
+      <c r="O70" s="27">
         <v>1.458</v>
       </c>
-      <c r="P70" s="21">
+      <c r="P70" s="20">
         <v>1.4368262739973601</v>
       </c>
-      <c r="Q70" s="23"/>
       <c r="R70" s="19" t="s">
         <v>100</v>
       </c>
       <c r="T70" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="X70" s="21">
+      <c r="X70" s="20">
         <v>0.312</v>
       </c>
     </row>
-    <row r="71" spans="1:24" s="21" customFormat="1">
+    <row r="71" spans="1:24" s="20" customFormat="1">
       <c r="A71" s="9" t="s">
         <v>83</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C71" s="21">
+      <c r="C71" s="20">
         <v>0.10199999999999999</v>
       </c>
-      <c r="D71" s="20">
+      <c r="D71" s="27">
         <v>-1.171</v>
       </c>
-      <c r="E71" s="20">
+      <c r="E71" s="27">
         <v>-0.59240301221006997</v>
       </c>
-      <c r="J71" s="20">
-        <v>0</v>
-      </c>
-      <c r="O71" s="20">
+      <c r="J71" s="27">
+        <v>0</v>
+      </c>
+      <c r="O71" s="27">
         <v>2.5470000000000002</v>
       </c>
-      <c r="P71" s="21">
+      <c r="P71" s="20">
         <v>2.4905493340587901</v>
       </c>
-      <c r="Q71" s="23"/>
       <c r="R71" s="19" t="s">
         <v>100</v>
       </c>
       <c r="T71" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="X71" s="21">
+      <c r="X71" s="20">
         <v>0.371</v>
       </c>
     </row>
-    <row r="72" spans="1:24" s="21" customFormat="1">
+    <row r="72" spans="1:24" s="20" customFormat="1">
       <c r="A72" s="9" t="s">
         <v>84</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C72" s="21">
+      <c r="C72" s="20">
         <v>0.152</v>
       </c>
-      <c r="D72" s="20">
+      <c r="D72" s="27">
         <v>-1.6830000000000001</v>
       </c>
-      <c r="E72" s="20">
+      <c r="E72" s="27">
         <v>-0.81572561388224996</v>
       </c>
-      <c r="J72" s="20">
-        <v>0</v>
-      </c>
-      <c r="O72" s="20">
+      <c r="J72" s="27">
+        <v>0</v>
+      </c>
+      <c r="O72" s="27">
         <v>3.81518914277475</v>
       </c>
-      <c r="P72" s="21">
+      <c r="P72" s="20">
         <v>3.855</v>
       </c>
-      <c r="Q72" s="23"/>
       <c r="R72" s="19" t="s">
         <v>100</v>
       </c>
       <c r="T72" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="X72" s="21">
+      <c r="X72" s="20">
         <v>0.41899999999999998</v>
       </c>
     </row>
-    <row r="73" spans="1:24" s="21" customFormat="1">
+    <row r="73" spans="1:24" s="20" customFormat="1">
       <c r="A73" s="9" t="s">
         <v>85</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C73" s="21">
+      <c r="C73" s="20">
         <v>0.214</v>
       </c>
-      <c r="D73" s="20">
+      <c r="D73" s="27">
         <v>-2.4769999999999999</v>
       </c>
-      <c r="E73" s="20">
+      <c r="E73" s="27">
         <v>-1.22567508688439</v>
       </c>
-      <c r="J73" s="20">
+      <c r="J73" s="27">
         <v>-3.4044364549679102E-12</v>
       </c>
-      <c r="O73" s="20">
+      <c r="O73" s="27">
         <v>5.5949999999999998</v>
       </c>
-      <c r="P73" s="21">
+      <c r="P73" s="20">
         <v>5.4782042149448502</v>
       </c>
-      <c r="Q73" s="23"/>
       <c r="R73" s="19" t="s">
         <v>100</v>
       </c>
       <c r="T73" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="X73" s="21">
+      <c r="X73" s="20">
         <v>0.32</v>
       </c>
     </row>
-    <row r="74" spans="1:24" s="21" customFormat="1">
+    <row r="74" spans="1:24" s="20" customFormat="1">
       <c r="A74" s="9" t="s">
         <v>86</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C74" s="21">
+      <c r="C74" s="20">
         <v>0.254</v>
       </c>
-      <c r="D74" s="20">
+      <c r="D74" s="27">
         <v>-2.8620000000000001</v>
       </c>
-      <c r="E74" s="20">
+      <c r="E74" s="27">
         <v>-1.4136198692773401</v>
       </c>
-      <c r="J74" s="20">
+      <c r="J74" s="27">
         <v>7.3805128675275E-12</v>
       </c>
-      <c r="O74" s="20">
+      <c r="O74" s="27">
         <v>6.484</v>
       </c>
-      <c r="P74" s="21">
+      <c r="P74" s="20">
         <v>6.2489999999999997</v>
       </c>
-      <c r="Q74" s="23"/>
       <c r="R74" s="19" t="s">
         <v>100</v>
       </c>
       <c r="T74" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="X74" s="21">
+      <c r="X74" s="20">
         <v>0.37799999999999995</v>
       </c>
     </row>
-    <row r="75" spans="1:24" s="21" customFormat="1">
+    <row r="75" spans="1:24" s="20" customFormat="1">
       <c r="A75" s="9" t="s">
         <v>87</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C75" s="21">
+      <c r="C75" s="20">
         <v>0.28399999999999997</v>
       </c>
-      <c r="D75" s="20">
+      <c r="D75" s="27">
         <v>-3.2050000000000001</v>
       </c>
-      <c r="E75" s="20">
+      <c r="E75" s="27">
         <v>-1.47353470842518</v>
       </c>
-      <c r="J75" s="20">
+      <c r="J75" s="27">
         <v>-3.4111879987364099E-12</v>
       </c>
-      <c r="O75" s="20">
+      <c r="O75" s="27">
         <v>8.0890000000000004</v>
       </c>
-      <c r="P75" s="21">
+      <c r="P75" s="20">
         <v>7.9485854277214001</v>
       </c>
-      <c r="Q75" s="23"/>
       <c r="R75" s="19" t="s">
         <v>100</v>
       </c>
       <c r="T75" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="X75" s="21">
+      <c r="X75" s="20">
         <v>0.39100000000000001</v>
       </c>
     </row>
-    <row r="76" spans="1:24" s="21" customFormat="1">
+    <row r="76" spans="1:24" s="20" customFormat="1">
       <c r="A76" s="9" t="s">
         <v>88</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C76" s="21">
+      <c r="C76" s="20">
         <v>0.33400000000000002</v>
       </c>
-      <c r="D76" s="20">
+      <c r="D76" s="27">
         <v>-5.2350000000000003</v>
       </c>
-      <c r="E76" s="20">
+      <c r="E76" s="27">
         <v>-1.99253212300414</v>
       </c>
-      <c r="J76" s="20">
+      <c r="J76" s="27">
         <v>2.0830000000081101</v>
       </c>
-      <c r="O76" s="20">
+      <c r="O76" s="27">
         <v>11.872999999999999</v>
       </c>
-      <c r="P76" s="21">
+      <c r="P76" s="20">
         <v>9.6077296533960403</v>
       </c>
-      <c r="Q76" s="23"/>
       <c r="R76" s="19" t="s">
         <v>100</v>
       </c>
       <c r="T76" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="X76" s="21">
+      <c r="X76" s="20">
         <v>0.41899999999999998</v>
       </c>
     </row>
-    <row r="77" spans="1:24" s="21" customFormat="1">
+    <row r="77" spans="1:24" s="20" customFormat="1">
       <c r="A77" s="9" t="s">
         <v>89</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C77" s="21">
+      <c r="C77" s="20">
         <v>0.379</v>
       </c>
-      <c r="D77" s="20">
+      <c r="D77" s="27">
         <v>-6.9569999999999999</v>
       </c>
-      <c r="E77" s="20">
+      <c r="E77" s="27">
         <v>-2.0155334705947299</v>
       </c>
-      <c r="J77" s="20">
+      <c r="J77" s="27">
         <v>5.5389999999999997</v>
       </c>
-      <c r="O77" s="20">
+      <c r="O77" s="27">
         <v>14.304133448972699</v>
       </c>
-      <c r="P77" s="21">
+      <c r="P77" s="20">
         <v>8.8979999999999997</v>
       </c>
-      <c r="Q77" s="23"/>
       <c r="R77" s="19" t="s">
         <v>100</v>
       </c>
       <c r="T77" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="X77" s="21">
+      <c r="X77" s="20">
         <v>0.39100000000000001</v>
       </c>
     </row>
@@ -5251,171 +5240,171 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:22" s="28" customFormat="1">
-      <c r="A5" s="28">
+    <row r="5" spans="1:22" s="25" customFormat="1">
+      <c r="A5" s="25">
         <v>4</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="26">
         <v>0.1</v>
       </c>
-      <c r="C5" s="28">
+      <c r="C5" s="25">
         <v>1.18</v>
       </c>
-      <c r="D5" s="28">
+      <c r="D5" s="25">
         <v>2.2029999999999998</v>
       </c>
-      <c r="H5" s="28">
+      <c r="H5" s="25">
         <v>2.2029999999999998</v>
       </c>
-      <c r="I5" s="28">
-        <v>0</v>
-      </c>
-      <c r="J5" s="28">
-        <v>0</v>
-      </c>
-      <c r="K5" s="28">
+      <c r="I5" s="25">
+        <v>0</v>
+      </c>
+      <c r="J5" s="25">
+        <v>0</v>
+      </c>
+      <c r="K5" s="25">
         <v>1.2795499999999999E-4</v>
       </c>
-      <c r="L5" s="28">
-        <v>0</v>
-      </c>
-      <c r="M5" s="28">
-        <v>0</v>
-      </c>
-      <c r="N5" s="28">
+      <c r="L5" s="25">
+        <v>0</v>
+      </c>
+      <c r="M5" s="25">
+        <v>0</v>
+      </c>
+      <c r="N5" s="25">
         <v>1.93</v>
       </c>
-      <c r="O5" s="28">
+      <c r="O5" s="25">
         <v>2.44</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="26">
         <v>0.35967375000000001</v>
       </c>
-      <c r="R5" s="29" t="s">
+      <c r="R5" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="S5" s="29">
+      <c r="S5" s="26">
         <v>5</v>
       </c>
-      <c r="T5" s="29" t="s">
+      <c r="T5" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="U5" s="29">
+      <c r="U5" s="26">
         <v>3</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V5" s="26" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:22" s="28" customFormat="1">
-      <c r="A6" s="28">
+    <row r="6" spans="1:22" s="25" customFormat="1">
+      <c r="A6" s="25">
         <v>5</v>
       </c>
-      <c r="B6" s="29">
+      <c r="B6" s="26">
         <v>0.1</v>
       </c>
-      <c r="C6" s="28">
+      <c r="C6" s="25">
         <v>1.127</v>
       </c>
-      <c r="D6" s="28">
+      <c r="D6" s="25">
         <v>2.0979999999999999</v>
       </c>
-      <c r="H6" s="28">
+      <c r="H6" s="25">
         <v>2.0979999999999999</v>
       </c>
-      <c r="I6" s="28">
+      <c r="I6" s="25">
         <v>1.6766474999999999E-2</v>
       </c>
-      <c r="J6" s="28">
-        <v>0</v>
-      </c>
-      <c r="K6" s="28">
+      <c r="J6" s="25">
+        <v>0</v>
+      </c>
+      <c r="K6" s="25">
         <v>1.5726999999999999E-4</v>
       </c>
-      <c r="L6" s="28">
-        <v>0</v>
-      </c>
-      <c r="M6" s="28">
-        <v>0</v>
-      </c>
-      <c r="N6" s="28">
+      <c r="L6" s="25">
+        <v>0</v>
+      </c>
+      <c r="M6" s="25">
+        <v>0</v>
+      </c>
+      <c r="N6" s="25">
         <v>2.0699999999999998</v>
       </c>
-      <c r="O6" s="28">
+      <c r="O6" s="25">
         <v>2.39</v>
       </c>
-      <c r="Q6" s="29">
+      <c r="Q6" s="26">
         <v>0.377942893</v>
       </c>
-      <c r="R6" s="29" t="s">
+      <c r="R6" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="S6" s="29">
+      <c r="S6" s="26">
         <v>5</v>
       </c>
-      <c r="T6" s="29" t="s">
+      <c r="T6" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="U6" s="29">
+      <c r="U6" s="26">
         <v>3</v>
       </c>
-      <c r="V6" s="29" t="s">
+      <c r="V6" s="26" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:22" s="28" customFormat="1">
-      <c r="A7" s="28">
+    <row r="7" spans="1:22" s="25" customFormat="1">
+      <c r="A7" s="25">
         <v>6</v>
       </c>
-      <c r="B7" s="29">
+      <c r="B7" s="26">
         <v>0.1</v>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="25">
         <v>1.0980000000000001</v>
       </c>
-      <c r="D7" s="28">
+      <c r="D7" s="25">
         <v>2.0550000000000002</v>
       </c>
-      <c r="H7" s="28">
+      <c r="H7" s="25">
         <v>2.0550000000000002</v>
       </c>
-      <c r="I7" s="28">
-        <v>0</v>
-      </c>
-      <c r="J7" s="28">
-        <v>0</v>
-      </c>
-      <c r="K7" s="28">
+      <c r="I7" s="25">
+        <v>0</v>
+      </c>
+      <c r="J7" s="25">
+        <v>0</v>
+      </c>
+      <c r="K7" s="25">
         <v>1.3422099999999999E-4</v>
       </c>
-      <c r="L7" s="28">
-        <v>0</v>
-      </c>
-      <c r="M7" s="28">
-        <v>0</v>
-      </c>
-      <c r="N7" s="28">
+      <c r="L7" s="25">
+        <v>0</v>
+      </c>
+      <c r="M7" s="25">
+        <v>0</v>
+      </c>
+      <c r="N7" s="25">
         <v>1.97</v>
       </c>
-      <c r="O7" s="28">
+      <c r="O7" s="25">
         <v>2.1800000000000002</v>
       </c>
-      <c r="Q7" s="29">
+      <c r="Q7" s="26">
         <v>0.33645671399999999</v>
       </c>
-      <c r="R7" s="29" t="s">
+      <c r="R7" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="S7" s="29">
+      <c r="S7" s="26">
         <v>5</v>
       </c>
-      <c r="T7" s="29" t="s">
+      <c r="T7" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="U7" s="29">
+      <c r="U7" s="26">
         <v>3</v>
       </c>
-      <c r="V7" s="29" t="s">
+      <c r="V7" s="26" t="s">
         <v>104</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add more code to analyse organelle mass fraction
</commit_message>
<xml_diff>
--- a/data/proteomics/physiology_collection.xlsx
+++ b/data/proteomics/physiology_collection.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11211"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Documents/GitHub/De-nevo-protein-3D-structure-yeast/data/proteomics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFD3D75D-BE95-5540-8EF8-954FC8521231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204D9642-9ED2-5146-9F94-D51ED0E73C7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1440" windowWidth="26060" windowHeight="15220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11440" yWindow="2440" windowWidth="34960" windowHeight="18520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
     <sheet name="Supplementary File 1e vip" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$T$1:$T$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$Q$1:$Q$87</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Supplementary File 1e vip'!$B$1:$B$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="126">
   <si>
     <t>sample</t>
   </si>
@@ -382,6 +382,36 @@
   </si>
   <si>
     <t>other_lab</t>
+  </si>
+  <si>
+    <t>REF</t>
+  </si>
+  <si>
+    <t>EtOH  20g/L</t>
+  </si>
+  <si>
+    <t>EtOH  40g/L</t>
+  </si>
+  <si>
+    <t>EtOH  60g/L</t>
+  </si>
+  <si>
+    <t>Osmo 0.2 M (NaCl)</t>
+  </si>
+  <si>
+    <t>Osmo 0.4 M (NaCl)</t>
+  </si>
+  <si>
+    <t>Osmo 0.6 M (NaCl)</t>
+  </si>
+  <si>
+    <t>Temp 33C</t>
+  </si>
+  <si>
+    <t>Temp 36C</t>
+  </si>
+  <si>
+    <t>Temp 38C</t>
   </si>
 </sst>
 </file>
@@ -958,7 +988,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1015,7 +1045,6 @@
     <xf numFmtId="0" fontId="18" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1024,6 +1053,24 @@
     <xf numFmtId="0" fontId="21" fillId="38" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1084,7 +1131,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2013 - 2022">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1372,7 +1419,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1380,12 +1427,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E8F22EE-2E06-6741-B451-D4EA064EAB2E}">
-  <dimension ref="A1:Z77"/>
+  <dimension ref="A1:Z87"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="37.6640625" style="2" customWidth="1"/>
     <col min="2" max="2" width="32.1640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="21.6640625" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" style="32" customWidth="1"/>
     <col min="4" max="4" width="22" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.1640625" bestFit="1" customWidth="1"/>
@@ -1417,7 +1464,7 @@
       <c r="B1" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="18" t="s">
         <v>91</v>
       </c>
       <c r="D1" s="12" t="s">
@@ -1497,6 +1544,7 @@
       <c r="B2" s="1" t="s">
         <v>114</v>
       </c>
+      <c r="C2" s="18"/>
       <c r="Q2" s="11"/>
     </row>
     <row r="3" spans="1:26" s="12" customFormat="1">
@@ -1506,6 +1554,7 @@
       <c r="B3" s="1" t="s">
         <v>114</v>
       </c>
+      <c r="C3" s="18"/>
       <c r="Q3" s="11"/>
     </row>
     <row r="4" spans="1:26" s="12" customFormat="1">
@@ -1515,6 +1564,7 @@
       <c r="B4" s="1" t="s">
         <v>114</v>
       </c>
+      <c r="C4" s="18"/>
       <c r="Q4" s="11"/>
     </row>
     <row r="5" spans="1:26" s="13" customFormat="1">
@@ -1524,7 +1574,7 @@
       <c r="B5" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="27">
         <v>0.42399999999999999</v>
       </c>
       <c r="D5" s="13">
@@ -1560,7 +1610,7 @@
       <c r="B6" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="28">
         <v>0.05</v>
       </c>
       <c r="D6" s="16">
@@ -1628,7 +1678,7 @@
       <c r="B7" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="28">
         <v>0.05</v>
       </c>
       <c r="D7" s="16">
@@ -1696,7 +1746,7 @@
       <c r="B8" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="28">
         <v>0.05</v>
       </c>
       <c r="D8" s="16">
@@ -1764,7 +1814,7 @@
       <c r="B9" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="28">
         <v>0.1</v>
       </c>
       <c r="D9" s="16">
@@ -1832,7 +1882,7 @@
       <c r="B10" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="28">
         <v>0.1</v>
       </c>
       <c r="D10" s="16">
@@ -1900,7 +1950,7 @@
       <c r="B11" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="28">
         <v>0.1</v>
       </c>
       <c r="D11" s="16">
@@ -1968,7 +2018,7 @@
       <c r="B12" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="28">
         <v>0.1</v>
       </c>
       <c r="D12" s="16">
@@ -2036,7 +2086,7 @@
       <c r="B13" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C13" s="15">
+      <c r="C13" s="28">
         <v>0.1</v>
       </c>
       <c r="D13" s="16">
@@ -2104,7 +2154,7 @@
       <c r="B14" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="28">
         <v>0.1</v>
       </c>
       <c r="D14" s="16">
@@ -2172,7 +2222,7 @@
       <c r="B15" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="28">
         <v>0.13</v>
       </c>
       <c r="D15" s="16">
@@ -2240,7 +2290,7 @@
       <c r="B16" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="28">
         <v>0.13</v>
       </c>
       <c r="D16" s="16">
@@ -2308,7 +2358,7 @@
       <c r="B17" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="28">
         <v>0.13</v>
       </c>
       <c r="D17" s="16">
@@ -2376,7 +2426,7 @@
       <c r="B18" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C18" s="15">
+      <c r="C18" s="28">
         <v>0.18</v>
       </c>
       <c r="D18" s="16">
@@ -2444,7 +2494,7 @@
       <c r="B19" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="15">
+      <c r="C19" s="28">
         <v>0.18</v>
       </c>
       <c r="D19" s="16">
@@ -2512,7 +2562,7 @@
       <c r="B20" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C20" s="15">
+      <c r="C20" s="28">
         <v>0.18</v>
       </c>
       <c r="D20" s="16">
@@ -2580,7 +2630,7 @@
       <c r="B21" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C21" s="15">
+      <c r="C21" s="28">
         <v>0.3</v>
       </c>
       <c r="D21" s="16">
@@ -2648,7 +2698,7 @@
       <c r="B22" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="28">
         <v>0.3</v>
       </c>
       <c r="D22" s="16">
@@ -2716,7 +2766,7 @@
       <c r="B23" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="28">
         <v>0.3</v>
       </c>
       <c r="D23" s="16">
@@ -2784,7 +2834,7 @@
       <c r="B24" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="28">
         <v>0.35</v>
       </c>
       <c r="D24" s="16">
@@ -2852,7 +2902,7 @@
       <c r="B25" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C25" s="15">
+      <c r="C25" s="28">
         <v>0.35</v>
       </c>
       <c r="D25" s="16">
@@ -2920,7 +2970,7 @@
       <c r="B26" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C26" s="15">
+      <c r="C26" s="28">
         <v>0.35</v>
       </c>
       <c r="D26" s="16">
@@ -2988,7 +3038,7 @@
       <c r="B27" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C27" s="15">
+      <c r="C27" s="28">
         <v>0.1</v>
       </c>
       <c r="D27" s="16">
@@ -3059,7 +3109,7 @@
       <c r="B28" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C28" s="15">
+      <c r="C28" s="28">
         <v>0.1</v>
       </c>
       <c r="D28" s="16">
@@ -3130,7 +3180,7 @@
       <c r="B29" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C29" s="15">
+      <c r="C29" s="28">
         <v>0.1</v>
       </c>
       <c r="D29" s="16">
@@ -3201,7 +3251,7 @@
       <c r="B30" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C30" s="15">
+      <c r="C30" s="28">
         <v>0.1</v>
       </c>
       <c r="D30" s="16">
@@ -3272,7 +3322,7 @@
       <c r="B31" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C31" s="15">
+      <c r="C31" s="28">
         <v>0.1</v>
       </c>
       <c r="D31" s="16">
@@ -3343,7 +3393,7 @@
       <c r="B32" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C32" s="15">
+      <c r="C32" s="28">
         <v>0.1</v>
       </c>
       <c r="D32" s="16">
@@ -3414,7 +3464,7 @@
       <c r="B33" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C33" s="15">
+      <c r="C33" s="28">
         <v>0.1</v>
       </c>
       <c r="D33" s="16">
@@ -3482,7 +3532,7 @@
       <c r="B34" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C34" s="15">
+      <c r="C34" s="28">
         <v>0.1</v>
       </c>
       <c r="D34" s="16">
@@ -3550,7 +3600,7 @@
       <c r="B35" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C35" s="15">
+      <c r="C35" s="28">
         <v>0.1</v>
       </c>
       <c r="D35" s="16">
@@ -3618,7 +3668,7 @@
       <c r="B36" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C36" s="15">
+      <c r="C36" s="28">
         <v>0.1</v>
       </c>
       <c r="D36" s="16">
@@ -3686,7 +3736,7 @@
       <c r="B37" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C37" s="15">
+      <c r="C37" s="28">
         <v>0.1</v>
       </c>
       <c r="D37" s="16">
@@ -3754,7 +3804,7 @@
       <c r="B38" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C38" s="15">
+      <c r="C38" s="28">
         <v>0.1</v>
       </c>
       <c r="D38" s="16">
@@ -3822,7 +3872,7 @@
       <c r="B39" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C39" s="15">
+      <c r="C39" s="28">
         <v>0.1</v>
       </c>
       <c r="D39" s="16">
@@ -3890,7 +3940,7 @@
       <c r="B40" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C40" s="15">
+      <c r="C40" s="28">
         <v>0.1</v>
       </c>
       <c r="D40" s="16">
@@ -3958,7 +4008,7 @@
       <c r="B41" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C41" s="15">
+      <c r="C41" s="28">
         <v>0.1</v>
       </c>
       <c r="D41" s="16">
@@ -4026,7 +4076,7 @@
       <c r="B42" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C42" s="15">
+      <c r="C42" s="28">
         <v>0.1</v>
       </c>
       <c r="D42" s="16">
@@ -4094,7 +4144,7 @@
       <c r="B43" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C43" s="15">
+      <c r="C43" s="28">
         <v>0.1</v>
       </c>
       <c r="D43" s="16">
@@ -4162,7 +4212,7 @@
       <c r="B44" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C44" s="15">
+      <c r="C44" s="28">
         <v>0.1</v>
       </c>
       <c r="D44" s="16">
@@ -4230,7 +4280,7 @@
       <c r="B45" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C45" s="15">
+      <c r="C45" s="28">
         <v>0.1</v>
       </c>
       <c r="D45" s="16">
@@ -4298,7 +4348,7 @@
       <c r="B46" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C46" s="15">
+      <c r="C46" s="28">
         <v>0.1</v>
       </c>
       <c r="D46" s="16">
@@ -4366,7 +4416,7 @@
       <c r="B47" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C47" s="15">
+      <c r="C47" s="28">
         <v>0.1</v>
       </c>
       <c r="D47" s="16">
@@ -4427,17 +4477,17 @@
         <v>0.42361575000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:24" s="23" customFormat="1">
+    <row r="48" spans="1:24" s="22" customFormat="1">
       <c r="A48" s="21" t="s">
         <v>61</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C48" s="22">
+      <c r="C48" s="29">
         <v>0.1</v>
       </c>
-      <c r="Q48" s="24"/>
+      <c r="Q48" s="23"/>
     </row>
     <row r="49" spans="1:17" s="7" customFormat="1">
       <c r="A49" s="4" t="s">
@@ -4520,7 +4570,7 @@
       <c r="B53" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C53" s="12">
+      <c r="C53" s="18">
         <v>0.1</v>
       </c>
       <c r="Q53" s="11"/>
@@ -4532,7 +4582,7 @@
       <c r="B54" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C54" s="12">
+      <c r="C54" s="18">
         <v>0.1</v>
       </c>
       <c r="E54" s="18"/>
@@ -4545,7 +4595,7 @@
       <c r="B55" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C55" s="12">
+      <c r="C55" s="18">
         <v>0.1</v>
       </c>
       <c r="Q55" s="11"/>
@@ -4557,7 +4607,7 @@
       <c r="B56" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C56" s="12">
+      <c r="C56" s="18">
         <v>0.1</v>
       </c>
       <c r="Q56" s="11"/>
@@ -4569,6 +4619,7 @@
       <c r="B57" s="1" t="s">
         <v>115</v>
       </c>
+      <c r="C57" s="18"/>
       <c r="Q57" s="11"/>
     </row>
     <row r="58" spans="1:17" s="12" customFormat="1">
@@ -4578,6 +4629,7 @@
       <c r="B58" s="1" t="s">
         <v>115</v>
       </c>
+      <c r="C58" s="18"/>
       <c r="Q58" s="11"/>
     </row>
     <row r="59" spans="1:17" s="12" customFormat="1">
@@ -4587,6 +4639,7 @@
       <c r="B59" s="1" t="s">
         <v>115</v>
       </c>
+      <c r="C59" s="18"/>
       <c r="Q59" s="11"/>
     </row>
     <row r="60" spans="1:17" s="12" customFormat="1">
@@ -4596,6 +4649,7 @@
       <c r="B60" s="1" t="s">
         <v>115</v>
       </c>
+      <c r="C60" s="18"/>
       <c r="Q60" s="11"/>
     </row>
     <row r="61" spans="1:17" s="12" customFormat="1">
@@ -4605,6 +4659,7 @@
       <c r="B61" s="1" t="s">
         <v>115</v>
       </c>
+      <c r="C61" s="18"/>
       <c r="Q61" s="11"/>
     </row>
     <row r="62" spans="1:17" s="12" customFormat="1">
@@ -4614,6 +4669,7 @@
       <c r="B62" s="1" t="s">
         <v>115</v>
       </c>
+      <c r="C62" s="18"/>
       <c r="Q62" s="11"/>
     </row>
     <row r="63" spans="1:17" s="12" customFormat="1">
@@ -4623,6 +4679,7 @@
       <c r="B63" s="1" t="s">
         <v>115</v>
       </c>
+      <c r="C63" s="18"/>
       <c r="Q63" s="11"/>
     </row>
     <row r="64" spans="1:17" s="12" customFormat="1">
@@ -4632,6 +4689,7 @@
       <c r="B64" s="1" t="s">
         <v>115</v>
       </c>
+      <c r="C64" s="18"/>
       <c r="Q64" s="11"/>
     </row>
     <row r="65" spans="1:24" s="12" customFormat="1">
@@ -4641,6 +4699,7 @@
       <c r="B65" s="1" t="s">
         <v>115</v>
       </c>
+      <c r="C65" s="18"/>
       <c r="Q65" s="11"/>
     </row>
     <row r="66" spans="1:24" s="12" customFormat="1">
@@ -4650,6 +4709,7 @@
       <c r="B66" s="1" t="s">
         <v>115</v>
       </c>
+      <c r="C66" s="18"/>
       <c r="Q66" s="11"/>
     </row>
     <row r="67" spans="1:24" s="12" customFormat="1">
@@ -4659,6 +4719,7 @@
       <c r="B67" s="1" t="s">
         <v>115</v>
       </c>
+      <c r="C67" s="18"/>
       <c r="Q67" s="11"/>
     </row>
     <row r="68" spans="1:24" s="12" customFormat="1">
@@ -4668,6 +4729,7 @@
       <c r="B68" s="1" t="s">
         <v>115</v>
       </c>
+      <c r="C68" s="18"/>
       <c r="Q68" s="11"/>
     </row>
     <row r="69" spans="1:24" s="19" customFormat="1">
@@ -4677,19 +4739,19 @@
       <c r="B69" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C69" s="19">
+      <c r="C69" s="30">
         <v>2.7E-2</v>
       </c>
-      <c r="D69" s="27">
+      <c r="D69" s="26">
         <v>-0.33700000000000002</v>
       </c>
-      <c r="E69" s="27">
+      <c r="E69" s="26">
         <v>-0.151308114750691</v>
       </c>
-      <c r="J69" s="27">
-        <v>0</v>
-      </c>
-      <c r="O69" s="27">
+      <c r="J69" s="26">
+        <v>0</v>
+      </c>
+      <c r="O69" s="26">
         <v>0.878</v>
       </c>
       <c r="P69" s="20">
@@ -4712,19 +4774,19 @@
       <c r="B70" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C70" s="20">
+      <c r="C70" s="31">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="D70" s="27">
+      <c r="D70" s="26">
         <v>-0.52300000000000002</v>
       </c>
-      <c r="E70" s="27">
+      <c r="E70" s="26">
         <v>-0.22220072795676099</v>
       </c>
-      <c r="J70" s="27">
-        <v>0</v>
-      </c>
-      <c r="O70" s="27">
+      <c r="J70" s="26">
+        <v>0</v>
+      </c>
+      <c r="O70" s="26">
         <v>1.458</v>
       </c>
       <c r="P70" s="20">
@@ -4747,19 +4809,19 @@
       <c r="B71" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C71" s="20">
+      <c r="C71" s="31">
         <v>0.10199999999999999</v>
       </c>
-      <c r="D71" s="27">
+      <c r="D71" s="26">
         <v>-1.171</v>
       </c>
-      <c r="E71" s="27">
+      <c r="E71" s="26">
         <v>-0.59240301221006997</v>
       </c>
-      <c r="J71" s="27">
-        <v>0</v>
-      </c>
-      <c r="O71" s="27">
+      <c r="J71" s="26">
+        <v>0</v>
+      </c>
+      <c r="O71" s="26">
         <v>2.5470000000000002</v>
       </c>
       <c r="P71" s="20">
@@ -4782,19 +4844,19 @@
       <c r="B72" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C72" s="20">
+      <c r="C72" s="31">
         <v>0.152</v>
       </c>
-      <c r="D72" s="27">
+      <c r="D72" s="26">
         <v>-1.6830000000000001</v>
       </c>
-      <c r="E72" s="27">
+      <c r="E72" s="26">
         <v>-0.81572561388224996</v>
       </c>
-      <c r="J72" s="27">
-        <v>0</v>
-      </c>
-      <c r="O72" s="27">
+      <c r="J72" s="26">
+        <v>0</v>
+      </c>
+      <c r="O72" s="26">
         <v>3.81518914277475</v>
       </c>
       <c r="P72" s="20">
@@ -4817,19 +4879,19 @@
       <c r="B73" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C73" s="20">
+      <c r="C73" s="31">
         <v>0.214</v>
       </c>
-      <c r="D73" s="27">
+      <c r="D73" s="26">
         <v>-2.4769999999999999</v>
       </c>
-      <c r="E73" s="27">
+      <c r="E73" s="26">
         <v>-1.22567508688439</v>
       </c>
-      <c r="J73" s="27">
+      <c r="J73" s="26">
         <v>-3.4044364549679102E-12</v>
       </c>
-      <c r="O73" s="27">
+      <c r="O73" s="26">
         <v>5.5949999999999998</v>
       </c>
       <c r="P73" s="20">
@@ -4852,19 +4914,19 @@
       <c r="B74" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C74" s="20">
+      <c r="C74" s="31">
         <v>0.254</v>
       </c>
-      <c r="D74" s="27">
+      <c r="D74" s="26">
         <v>-2.8620000000000001</v>
       </c>
-      <c r="E74" s="27">
+      <c r="E74" s="26">
         <v>-1.4136198692773401</v>
       </c>
-      <c r="J74" s="27">
+      <c r="J74" s="26">
         <v>7.3805128675275E-12</v>
       </c>
-      <c r="O74" s="27">
+      <c r="O74" s="26">
         <v>6.484</v>
       </c>
       <c r="P74" s="20">
@@ -4887,19 +4949,19 @@
       <c r="B75" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C75" s="20">
+      <c r="C75" s="31">
         <v>0.28399999999999997</v>
       </c>
-      <c r="D75" s="27">
+      <c r="D75" s="26">
         <v>-3.2050000000000001</v>
       </c>
-      <c r="E75" s="27">
+      <c r="E75" s="26">
         <v>-1.47353470842518</v>
       </c>
-      <c r="J75" s="27">
+      <c r="J75" s="26">
         <v>-3.4111879987364099E-12</v>
       </c>
-      <c r="O75" s="27">
+      <c r="O75" s="26">
         <v>8.0890000000000004</v>
       </c>
       <c r="P75" s="20">
@@ -4922,19 +4984,19 @@
       <c r="B76" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C76" s="20">
+      <c r="C76" s="31">
         <v>0.33400000000000002</v>
       </c>
-      <c r="D76" s="27">
+      <c r="D76" s="26">
         <v>-5.2350000000000003</v>
       </c>
-      <c r="E76" s="27">
+      <c r="E76" s="26">
         <v>-1.99253212300414</v>
       </c>
-      <c r="J76" s="27">
+      <c r="J76" s="26">
         <v>2.0830000000081101</v>
       </c>
-      <c r="O76" s="27">
+      <c r="O76" s="26">
         <v>11.872999999999999</v>
       </c>
       <c r="P76" s="20">
@@ -4957,19 +5019,19 @@
       <c r="B77" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C77" s="20">
+      <c r="C77" s="31">
         <v>0.379</v>
       </c>
-      <c r="D77" s="27">
+      <c r="D77" s="26">
         <v>-6.9569999999999999</v>
       </c>
-      <c r="E77" s="27">
+      <c r="E77" s="26">
         <v>-2.0155334705947299</v>
       </c>
-      <c r="J77" s="27">
+      <c r="J77" s="26">
         <v>5.5389999999999997</v>
       </c>
-      <c r="O77" s="27">
+      <c r="O77" s="26">
         <v>14.304133448972699</v>
       </c>
       <c r="P77" s="20">
@@ -4983,6 +5045,116 @@
       </c>
       <c r="X77" s="20">
         <v>0.39100000000000001</v>
+      </c>
+    </row>
+    <row r="78" spans="1:24">
+      <c r="A78" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C78" s="18">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:24">
+      <c r="A79" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C79" s="18">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:24">
+      <c r="A80" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C80" s="18">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C81" s="18">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3">
+      <c r="A82" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C82" s="18">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3">
+      <c r="A83" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C83" s="18">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3">
+      <c r="A84" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C84" s="18">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3">
+      <c r="A85" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C85" s="18">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3">
+      <c r="A86" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C86" s="18">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3">
+      <c r="A87" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C87" s="18">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -5240,171 +5412,171 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:22" s="25" customFormat="1">
-      <c r="A5" s="25">
+    <row r="5" spans="1:22" s="24" customFormat="1">
+      <c r="A5" s="24">
         <v>4</v>
       </c>
-      <c r="B5" s="26">
+      <c r="B5" s="25">
         <v>0.1</v>
       </c>
-      <c r="C5" s="25">
+      <c r="C5" s="24">
         <v>1.18</v>
       </c>
-      <c r="D5" s="25">
+      <c r="D5" s="24">
         <v>2.2029999999999998</v>
       </c>
-      <c r="H5" s="25">
+      <c r="H5" s="24">
         <v>2.2029999999999998</v>
       </c>
-      <c r="I5" s="25">
-        <v>0</v>
-      </c>
-      <c r="J5" s="25">
-        <v>0</v>
-      </c>
-      <c r="K5" s="25">
+      <c r="I5" s="24">
+        <v>0</v>
+      </c>
+      <c r="J5" s="24">
+        <v>0</v>
+      </c>
+      <c r="K5" s="24">
         <v>1.2795499999999999E-4</v>
       </c>
-      <c r="L5" s="25">
-        <v>0</v>
-      </c>
-      <c r="M5" s="25">
-        <v>0</v>
-      </c>
-      <c r="N5" s="25">
+      <c r="L5" s="24">
+        <v>0</v>
+      </c>
+      <c r="M5" s="24">
+        <v>0</v>
+      </c>
+      <c r="N5" s="24">
         <v>1.93</v>
       </c>
-      <c r="O5" s="25">
+      <c r="O5" s="24">
         <v>2.44</v>
       </c>
-      <c r="Q5" s="26">
+      <c r="Q5" s="25">
         <v>0.35967375000000001</v>
       </c>
-      <c r="R5" s="26" t="s">
+      <c r="R5" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="S5" s="26">
+      <c r="S5" s="25">
         <v>5</v>
       </c>
-      <c r="T5" s="26" t="s">
+      <c r="T5" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="U5" s="26">
+      <c r="U5" s="25">
         <v>3</v>
       </c>
-      <c r="V5" s="26" t="s">
+      <c r="V5" s="25" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:22" s="25" customFormat="1">
-      <c r="A6" s="25">
+    <row r="6" spans="1:22" s="24" customFormat="1">
+      <c r="A6" s="24">
         <v>5</v>
       </c>
-      <c r="B6" s="26">
+      <c r="B6" s="25">
         <v>0.1</v>
       </c>
-      <c r="C6" s="25">
+      <c r="C6" s="24">
         <v>1.127</v>
       </c>
-      <c r="D6" s="25">
+      <c r="D6" s="24">
         <v>2.0979999999999999</v>
       </c>
-      <c r="H6" s="25">
+      <c r="H6" s="24">
         <v>2.0979999999999999</v>
       </c>
-      <c r="I6" s="25">
+      <c r="I6" s="24">
         <v>1.6766474999999999E-2</v>
       </c>
-      <c r="J6" s="25">
-        <v>0</v>
-      </c>
-      <c r="K6" s="25">
+      <c r="J6" s="24">
+        <v>0</v>
+      </c>
+      <c r="K6" s="24">
         <v>1.5726999999999999E-4</v>
       </c>
-      <c r="L6" s="25">
-        <v>0</v>
-      </c>
-      <c r="M6" s="25">
-        <v>0</v>
-      </c>
-      <c r="N6" s="25">
+      <c r="L6" s="24">
+        <v>0</v>
+      </c>
+      <c r="M6" s="24">
+        <v>0</v>
+      </c>
+      <c r="N6" s="24">
         <v>2.0699999999999998</v>
       </c>
-      <c r="O6" s="25">
+      <c r="O6" s="24">
         <v>2.39</v>
       </c>
-      <c r="Q6" s="26">
+      <c r="Q6" s="25">
         <v>0.377942893</v>
       </c>
-      <c r="R6" s="26" t="s">
+      <c r="R6" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="S6" s="26">
+      <c r="S6" s="25">
         <v>5</v>
       </c>
-      <c r="T6" s="26" t="s">
+      <c r="T6" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="U6" s="26">
+      <c r="U6" s="25">
         <v>3</v>
       </c>
-      <c r="V6" s="26" t="s">
+      <c r="V6" s="25" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:22" s="25" customFormat="1">
-      <c r="A7" s="25">
+    <row r="7" spans="1:22" s="24" customFormat="1">
+      <c r="A7" s="24">
         <v>6</v>
       </c>
-      <c r="B7" s="26">
+      <c r="B7" s="25">
         <v>0.1</v>
       </c>
-      <c r="C7" s="25">
+      <c r="C7" s="24">
         <v>1.0980000000000001</v>
       </c>
-      <c r="D7" s="25">
+      <c r="D7" s="24">
         <v>2.0550000000000002</v>
       </c>
-      <c r="H7" s="25">
+      <c r="H7" s="24">
         <v>2.0550000000000002</v>
       </c>
-      <c r="I7" s="25">
-        <v>0</v>
-      </c>
-      <c r="J7" s="25">
-        <v>0</v>
-      </c>
-      <c r="K7" s="25">
+      <c r="I7" s="24">
+        <v>0</v>
+      </c>
+      <c r="J7" s="24">
+        <v>0</v>
+      </c>
+      <c r="K7" s="24">
         <v>1.3422099999999999E-4</v>
       </c>
-      <c r="L7" s="25">
-        <v>0</v>
-      </c>
-      <c r="M7" s="25">
-        <v>0</v>
-      </c>
-      <c r="N7" s="25">
+      <c r="L7" s="24">
+        <v>0</v>
+      </c>
+      <c r="M7" s="24">
+        <v>0</v>
+      </c>
+      <c r="N7" s="24">
         <v>1.97</v>
       </c>
-      <c r="O7" s="25">
+      <c r="O7" s="24">
         <v>2.1800000000000002</v>
       </c>
-      <c r="Q7" s="26">
+      <c r="Q7" s="25">
         <v>0.33645671399999999</v>
       </c>
-      <c r="R7" s="26" t="s">
+      <c r="R7" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="S7" s="26">
+      <c r="S7" s="25">
         <v>5</v>
       </c>
-      <c r="T7" s="26" t="s">
+      <c r="T7" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="U7" s="26">
+      <c r="U7" s="25">
         <v>3</v>
       </c>
-      <c r="V7" s="26" t="s">
+      <c r="V7" s="25" t="s">
         <v>104</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: connect the proteomices with trait
</commit_message>
<xml_diff>
--- a/data/proteomics/physiology_collection.xlsx
+++ b/data/proteomics/physiology_collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Documents/GitHub/large_scale_yeast_proteomics_analysis/data/proteomics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C2207DB-0300-7D49-BAA7-86BDB2FF07A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6639D6A2-DB14-1A4A-A425-850FBF6C7C1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2360" yWindow="500" windowWidth="37660" windowHeight="22540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2856" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2895" uniqueCount="511">
   <si>
     <t>sample</t>
   </si>
@@ -1722,6 +1722,63 @@
   </si>
   <si>
     <t>sysbio_Kate</t>
+  </si>
+  <si>
+    <t>Trehalose</t>
+  </si>
+  <si>
+    <t>Glucose</t>
+  </si>
+  <si>
+    <t>Maltose</t>
+  </si>
+  <si>
+    <t>Galactose</t>
+  </si>
+  <si>
+    <t>cycloheximide_inhibition_miu=0.12</t>
+  </si>
+  <si>
+    <t>cycloheximide_inhibition_miu=0.39</t>
+  </si>
+  <si>
+    <t>cycloheximide_inhibition_miu=0.32</t>
+  </si>
+  <si>
+    <t>cycloheximide_inhibition_miu=0.2</t>
+  </si>
+  <si>
+    <t>maltose</t>
+  </si>
+  <si>
+    <t>oleate</t>
+  </si>
+  <si>
+    <t>fructose</t>
+  </si>
+  <si>
+    <t>sucrose</t>
+  </si>
+  <si>
+    <t>trehalose</t>
+  </si>
+  <si>
+    <t>lactate</t>
+  </si>
+  <si>
+    <t>acetate</t>
+  </si>
+  <si>
+    <t>pryuvate</t>
+  </si>
+  <si>
+    <t>glycerol</t>
+  </si>
+  <si>
+    <t>galactose</t>
+  </si>
+  <si>
+    <t>raffinose</t>
   </si>
 </sst>
 </file>
@@ -1982,7 +2039,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="42">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2210,6 +2267,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="14">
     <border>
@@ -2416,7 +2479,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2659,6 +2722,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="41" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="41" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="42" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -9137,7 +9209,9 @@
       <c r="F100" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G100" s="61"/>
+      <c r="G100" s="74" t="s">
+        <v>106</v>
+      </c>
       <c r="H100" s="12" t="s">
         <v>172</v>
       </c>
@@ -9164,7 +9238,9 @@
       <c r="F101" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G101" s="61"/>
+      <c r="G101" s="74" t="s">
+        <v>107</v>
+      </c>
       <c r="H101" s="12" t="s">
         <v>172</v>
       </c>
@@ -9191,7 +9267,9 @@
       <c r="F102" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G102" s="61"/>
+      <c r="G102" s="74" t="s">
+        <v>108</v>
+      </c>
       <c r="H102" s="12" t="s">
         <v>172</v>
       </c>
@@ -9218,7 +9296,9 @@
       <c r="F103" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G103" s="61"/>
+      <c r="G103" s="74" t="s">
+        <v>109</v>
+      </c>
       <c r="H103" s="12" t="s">
         <v>172</v>
       </c>
@@ -9245,7 +9325,9 @@
       <c r="F104" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G104" s="61"/>
+      <c r="G104" s="74" t="s">
+        <v>110</v>
+      </c>
       <c r="H104" s="12" t="s">
         <v>172</v>
       </c>
@@ -9272,7 +9354,9 @@
       <c r="F105" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G105" s="61"/>
+      <c r="G105" s="74" t="s">
+        <v>111</v>
+      </c>
       <c r="H105" s="12" t="s">
         <v>172</v>
       </c>
@@ -9299,7 +9383,9 @@
       <c r="F106" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G106" s="61"/>
+      <c r="G106" s="74" t="s">
+        <v>112</v>
+      </c>
       <c r="H106" s="12" t="s">
         <v>172</v>
       </c>
@@ -9326,7 +9412,9 @@
       <c r="F107" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G107" s="61"/>
+      <c r="G107" s="74" t="s">
+        <v>113</v>
+      </c>
       <c r="H107" s="12" t="s">
         <v>172</v>
       </c>
@@ -9353,7 +9441,9 @@
       <c r="F108" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G108" s="61"/>
+      <c r="G108" s="74" t="s">
+        <v>114</v>
+      </c>
       <c r="H108" s="12" t="s">
         <v>172</v>
       </c>
@@ -9380,7 +9470,9 @@
       <c r="F109" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G109" s="61"/>
+      <c r="G109" s="74" t="s">
+        <v>115</v>
+      </c>
       <c r="H109" s="12" t="s">
         <v>172</v>
       </c>
@@ -9407,7 +9499,9 @@
       <c r="F110" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="G110" s="60"/>
+      <c r="G110" s="10" t="s">
+        <v>500</v>
+      </c>
       <c r="H110" s="13" t="s">
         <v>209</v>
       </c>
@@ -9437,7 +9531,9 @@
       <c r="F111" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G111" s="61"/>
+      <c r="G111" s="6" t="s">
+        <v>501</v>
+      </c>
       <c r="H111" s="5" t="s">
         <v>209</v>
       </c>
@@ -9467,7 +9563,9 @@
       <c r="F112" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G112" s="61"/>
+      <c r="G112" s="6" t="s">
+        <v>502</v>
+      </c>
       <c r="H112" s="5" t="s">
         <v>209</v>
       </c>
@@ -9497,7 +9595,9 @@
       <c r="F113" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G113" s="61"/>
+      <c r="G113" s="6" t="s">
+        <v>503</v>
+      </c>
       <c r="H113" s="5" t="s">
         <v>209</v>
       </c>
@@ -9527,7 +9627,9 @@
       <c r="F114" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G114" s="61"/>
+      <c r="G114" s="6" t="s">
+        <v>504</v>
+      </c>
       <c r="H114" s="5" t="s">
         <v>209</v>
       </c>
@@ -9557,7 +9659,9 @@
       <c r="F115" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G115" s="61"/>
+      <c r="G115" s="6" t="s">
+        <v>505</v>
+      </c>
       <c r="H115" s="5" t="s">
         <v>209</v>
       </c>
@@ -9587,7 +9691,9 @@
       <c r="F116" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G116" s="61"/>
+      <c r="G116" s="6" t="s">
+        <v>506</v>
+      </c>
       <c r="H116" s="5" t="s">
         <v>209</v>
       </c>
@@ -9617,7 +9723,9 @@
       <c r="F117" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G117" s="61"/>
+      <c r="G117" s="6" t="s">
+        <v>507</v>
+      </c>
       <c r="H117" s="5" t="s">
         <v>209</v>
       </c>
@@ -9647,7 +9755,9 @@
       <c r="F118" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G118" s="61"/>
+      <c r="G118" s="6" t="s">
+        <v>508</v>
+      </c>
       <c r="H118" s="5" t="s">
         <v>209</v>
       </c>
@@ -9677,7 +9787,9 @@
       <c r="F119" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G119" s="61"/>
+      <c r="G119" s="6" t="s">
+        <v>509</v>
+      </c>
       <c r="H119" s="5" t="s">
         <v>209</v>
       </c>
@@ -9707,7 +9819,9 @@
       <c r="F120" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="G120" s="62"/>
+      <c r="G120" s="11" t="s">
+        <v>510</v>
+      </c>
       <c r="H120" s="14" t="s">
         <v>209</v>
       </c>
@@ -10785,7 +10899,7 @@
       <c r="B159" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="C159" s="37" t="s">
+      <c r="C159" s="88" t="s">
         <v>307</v>
       </c>
       <c r="D159" s="38" t="s">
@@ -10797,12 +10911,15 @@
       <c r="F159" s="13" t="s">
         <v>128</v>
       </c>
+      <c r="G159" s="86" t="s">
+        <v>492</v>
+      </c>
       <c r="I159" s="13">
         <v>5.1999999999999998E-2</v>
       </c>
       <c r="X159" s="31"/>
     </row>
-    <row r="160" spans="1:25">
+    <row r="160" spans="1:25" ht="14" customHeight="1">
       <c r="A160" s="6" t="s">
         <v>177</v>
       </c>
@@ -10820,6 +10937,9 @@
       </c>
       <c r="F160" s="5" t="s">
         <v>128</v>
+      </c>
+      <c r="G160" s="87" t="s">
+        <v>492</v>
       </c>
       <c r="I160" s="5">
         <v>5.0999999999999997E-2</v>
@@ -10844,6 +10964,9 @@
       <c r="F161" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G161" s="87" t="s">
+        <v>492</v>
+      </c>
       <c r="I161" s="5">
         <v>4.8000000000000001E-2</v>
       </c>
@@ -10867,6 +10990,9 @@
       <c r="F162" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G162" s="87" t="s">
+        <v>492</v>
+      </c>
       <c r="I162" s="5">
         <v>4.7E-2</v>
       </c>
@@ -10890,6 +11016,9 @@
       <c r="F163" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G163" s="6" t="s">
+        <v>495</v>
+      </c>
       <c r="I163" s="5">
         <v>0.16500000000000001</v>
       </c>
@@ -10913,6 +11042,9 @@
       <c r="F164" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G164" s="6" t="s">
+        <v>495</v>
+      </c>
       <c r="I164" s="5">
         <v>0.182</v>
       </c>
@@ -10936,6 +11068,9 @@
       <c r="F165" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G165" s="6" t="s">
+        <v>494</v>
+      </c>
       <c r="I165" s="5">
         <v>0.27500000000000002</v>
       </c>
@@ -10959,6 +11094,9 @@
       <c r="F166" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G166" s="6" t="s">
+        <v>494</v>
+      </c>
       <c r="I166" s="5">
         <v>0.29099999999999998</v>
       </c>
@@ -10982,6 +11120,9 @@
       <c r="F167" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G167" s="6" t="s">
+        <v>493</v>
+      </c>
       <c r="I167" s="5">
         <v>0.373</v>
       </c>
@@ -11005,6 +11146,9 @@
       <c r="F168" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G168" s="6" t="s">
+        <v>493</v>
+      </c>
       <c r="I168" s="5">
         <v>0.36899999999999999</v>
       </c>
@@ -11028,6 +11172,9 @@
       <c r="F169" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G169" s="5" t="s">
+        <v>496</v>
+      </c>
       <c r="I169" s="5">
         <v>0.121</v>
       </c>
@@ -11051,6 +11198,9 @@
       <c r="F170" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G170" s="5" t="s">
+        <v>496</v>
+      </c>
       <c r="I170" s="5">
         <v>0.106</v>
       </c>
@@ -11074,6 +11224,9 @@
       <c r="F171" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G171" s="5" t="s">
+        <v>499</v>
+      </c>
       <c r="I171" s="5">
         <v>0.2</v>
       </c>
@@ -11097,6 +11250,9 @@
       <c r="F172" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G172" s="5" t="s">
+        <v>499</v>
+      </c>
       <c r="I172" s="5">
         <v>0.20100000000000001</v>
       </c>
@@ -11120,6 +11276,9 @@
       <c r="F173" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G173" s="5" t="s">
+        <v>498</v>
+      </c>
       <c r="I173" s="5">
         <v>0.32700000000000001</v>
       </c>
@@ -11143,6 +11302,9 @@
       <c r="F174" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G174" s="5" t="s">
+        <v>498</v>
+      </c>
       <c r="I174" s="5">
         <v>0.318</v>
       </c>
@@ -11166,6 +11328,9 @@
       <c r="F175" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G175" s="5" t="s">
+        <v>497</v>
+      </c>
       <c r="I175" s="5">
         <v>0.42099999999999999</v>
       </c>
@@ -11188,6 +11353,9 @@
       </c>
       <c r="F176" s="5" t="s">
         <v>128</v>
+      </c>
+      <c r="G176" s="5" t="s">
+        <v>497</v>
       </c>
       <c r="I176" s="5">
         <v>0.39900000000000002</v>
@@ -13907,6 +14075,9 @@
     </row>
   </sheetData>
   <phoneticPr fontId="26" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C159" r:id="rId1" xr:uid="{BF63034B-E53E-AA4F-9F22-3EC9CCE474BD}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: add code for figure
</commit_message>
<xml_diff>
--- a/data/proteomics/physiology_collection.xlsx
+++ b/data/proteomics/physiology_collection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Documents/GitHub/large_scale_yeast_proteomics_analysis/data/proteomics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2F2BCDA-BAE1-254D-A623-0104609C5D94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDA4A4FF-7155-8F45-844E-1CF31281AA18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2360" yWindow="500" windowWidth="37660" windowHeight="22540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="26000" windowHeight="16300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="cell cycle_kate" sheetId="5" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AE$158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$G$1:$G$301</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Supplementary File 1e vip'!$B$1:$B$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2870" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2958" uniqueCount="518">
   <si>
     <t>sample</t>
   </si>
@@ -1244,9 +1244,6 @@
   </si>
   <si>
     <t>Ethanol_phase</t>
-  </si>
-  <si>
-    <t>condition_detail</t>
   </si>
   <si>
     <t>https://doi.org/10.1038/s41467-022-30513-5</t>
@@ -1777,6 +1774,30 @@
   </si>
   <si>
     <t>raffinose</t>
+  </si>
+  <si>
+    <t>Chemostats_C_limit_miu=0.34</t>
+  </si>
+  <si>
+    <t>Chemostats_C_limit_miu=0.32</t>
+  </si>
+  <si>
+    <t>Chemostats_C_limit_miu=0.3</t>
+  </si>
+  <si>
+    <t>Chemostats_C_limit_miu=0.27</t>
+  </si>
+  <si>
+    <t>Chemostats_C_limit_miu=0.20</t>
+  </si>
+  <si>
+    <t>Chemostats_C_limit_miu=0.23</t>
+  </si>
+  <si>
+    <t>FG_CN4_D= 0.26 or 0.32</t>
+  </si>
+  <si>
+    <t>condition_unique</t>
   </si>
 </sst>
 </file>
@@ -2477,7 +2498,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2647,9 +2668,6 @@
     <xf numFmtId="0" fontId="36" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -2705,9 +2723,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3120,7 +3135,7 @@
   <sheetData>
     <row r="1" spans="1:31" s="28" customFormat="1" ht="19">
       <c r="A1" s="28" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B1" s="28" t="s">
         <v>105</v>
@@ -3137,8 +3152,8 @@
       <c r="F1" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="G1" s="79" t="s">
-        <v>398</v>
+      <c r="G1" s="78" t="s">
+        <v>517</v>
       </c>
       <c r="H1" s="28" t="s">
         <v>171</v>
@@ -3218,7 +3233,7 @@
         <v>386</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>325</v>
@@ -3250,7 +3265,7 @@
         <v>387</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>325</v>
@@ -3282,7 +3297,7 @@
         <v>388</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>325</v>
@@ -3314,7 +3329,7 @@
         <v>389</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>325</v>
@@ -3338,7 +3353,7 @@
         <v>390</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>325</v>
@@ -3362,7 +3377,7 @@
         <v>391</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>325</v>
@@ -3386,7 +3401,7 @@
         <v>392</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>325</v>
@@ -3410,7 +3425,7 @@
         <v>393</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>325</v>
@@ -3434,7 +3449,7 @@
         <v>394</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>325</v>
@@ -3454,11 +3469,11 @@
       <c r="X10" s="31"/>
     </row>
     <row r="11" spans="1:31" s="32" customFormat="1">
-      <c r="A11" s="65" t="s">
+      <c r="A11" s="64" t="s">
         <v>14</v>
       </c>
       <c r="B11" s="25" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C11" s="25" t="s">
         <v>310</v>
@@ -3472,7 +3487,9 @@
       <c r="F11" s="25" t="s">
         <v>128</v>
       </c>
-      <c r="G11" s="61"/>
+      <c r="G11" s="64" t="s">
+        <v>14</v>
+      </c>
       <c r="H11" s="26" t="s">
         <v>172</v>
       </c>
@@ -3511,11 +3528,11 @@
       </c>
     </row>
     <row r="12" spans="1:31">
-      <c r="A12" s="66" t="s">
+      <c r="A12" s="65" t="s">
         <v>15</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>324</v>
@@ -3597,11 +3614,11 @@
       </c>
     </row>
     <row r="13" spans="1:31">
-      <c r="A13" s="66" t="s">
+      <c r="A13" s="65" t="s">
         <v>16</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>324</v>
@@ -3683,11 +3700,11 @@
       </c>
     </row>
     <row r="14" spans="1:31">
-      <c r="A14" s="66" t="s">
+      <c r="A14" s="65" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>324</v>
@@ -3769,11 +3786,11 @@
       </c>
     </row>
     <row r="15" spans="1:31">
-      <c r="A15" s="66" t="s">
+      <c r="A15" s="65" t="s">
         <v>18</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>324</v>
@@ -3855,11 +3872,11 @@
       </c>
     </row>
     <row r="16" spans="1:31">
-      <c r="A16" s="66" t="s">
+      <c r="A16" s="65" t="s">
         <v>19</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>324</v>
@@ -3941,11 +3958,11 @@
       </c>
     </row>
     <row r="17" spans="1:30">
-      <c r="A17" s="66" t="s">
+      <c r="A17" s="65" t="s">
         <v>20</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>324</v>
@@ -4027,11 +4044,11 @@
       </c>
     </row>
     <row r="18" spans="1:30">
-      <c r="A18" s="66" t="s">
+      <c r="A18" s="65" t="s">
         <v>21</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>324</v>
@@ -4113,11 +4130,11 @@
       </c>
     </row>
     <row r="19" spans="1:30">
-      <c r="A19" s="66" t="s">
+      <c r="A19" s="65" t="s">
         <v>22</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>324</v>
@@ -4199,11 +4216,11 @@
       </c>
     </row>
     <row r="20" spans="1:30">
-      <c r="A20" s="66" t="s">
+      <c r="A20" s="65" t="s">
         <v>23</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>324</v>
@@ -4285,11 +4302,11 @@
       </c>
     </row>
     <row r="21" spans="1:30">
-      <c r="A21" s="66" t="s">
+      <c r="A21" s="65" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>324</v>
@@ -4371,11 +4388,11 @@
       </c>
     </row>
     <row r="22" spans="1:30">
-      <c r="A22" s="66" t="s">
+      <c r="A22" s="65" t="s">
         <v>25</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>324</v>
@@ -4457,11 +4474,11 @@
       </c>
     </row>
     <row r="23" spans="1:30">
-      <c r="A23" s="66" t="s">
+      <c r="A23" s="65" t="s">
         <v>26</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>324</v>
@@ -4543,11 +4560,11 @@
       </c>
     </row>
     <row r="24" spans="1:30">
-      <c r="A24" s="66" t="s">
+      <c r="A24" s="65" t="s">
         <v>27</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>324</v>
@@ -4629,11 +4646,11 @@
       </c>
     </row>
     <row r="25" spans="1:30">
-      <c r="A25" s="66" t="s">
+      <c r="A25" s="65" t="s">
         <v>28</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>324</v>
@@ -4715,11 +4732,11 @@
       </c>
     </row>
     <row r="26" spans="1:30">
-      <c r="A26" s="66" t="s">
+      <c r="A26" s="65" t="s">
         <v>29</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>324</v>
@@ -4801,11 +4818,11 @@
       </c>
     </row>
     <row r="27" spans="1:30">
-      <c r="A27" s="66" t="s">
+      <c r="A27" s="65" t="s">
         <v>30</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>324</v>
@@ -4887,11 +4904,11 @@
       </c>
     </row>
     <row r="28" spans="1:30">
-      <c r="A28" s="66" t="s">
+      <c r="A28" s="65" t="s">
         <v>31</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>324</v>
@@ -4973,11 +4990,11 @@
       </c>
     </row>
     <row r="29" spans="1:30">
-      <c r="A29" s="66" t="s">
+      <c r="A29" s="65" t="s">
         <v>32</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>324</v>
@@ -5059,11 +5076,11 @@
       </c>
     </row>
     <row r="30" spans="1:30">
-      <c r="A30" s="66" t="s">
+      <c r="A30" s="65" t="s">
         <v>33</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>324</v>
@@ -5145,11 +5162,11 @@
       </c>
     </row>
     <row r="31" spans="1:30">
-      <c r="A31" s="66" t="s">
+      <c r="A31" s="65" t="s">
         <v>34</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>324</v>
@@ -5231,11 +5248,11 @@
       </c>
     </row>
     <row r="32" spans="1:30">
-      <c r="A32" s="66" t="s">
+      <c r="A32" s="65" t="s">
         <v>35</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>324</v>
@@ -5317,11 +5334,11 @@
       </c>
     </row>
     <row r="33" spans="1:31">
-      <c r="A33" s="66" t="s">
+      <c r="A33" s="65" t="s">
         <v>36</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>324</v>
@@ -5406,11 +5423,11 @@
       </c>
     </row>
     <row r="34" spans="1:31">
-      <c r="A34" s="66" t="s">
+      <c r="A34" s="65" t="s">
         <v>37</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>324</v>
@@ -5495,11 +5512,11 @@
       </c>
     </row>
     <row r="35" spans="1:31">
-      <c r="A35" s="66" t="s">
+      <c r="A35" s="65" t="s">
         <v>38</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>324</v>
@@ -5584,11 +5601,11 @@
       </c>
     </row>
     <row r="36" spans="1:31">
-      <c r="A36" s="66" t="s">
+      <c r="A36" s="65" t="s">
         <v>39</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>324</v>
@@ -5673,11 +5690,11 @@
       </c>
     </row>
     <row r="37" spans="1:31">
-      <c r="A37" s="66" t="s">
+      <c r="A37" s="65" t="s">
         <v>40</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>324</v>
@@ -5762,11 +5779,11 @@
       </c>
     </row>
     <row r="38" spans="1:31">
-      <c r="A38" s="66" t="s">
+      <c r="A38" s="65" t="s">
         <v>41</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>324</v>
@@ -5851,11 +5868,11 @@
       </c>
     </row>
     <row r="39" spans="1:31">
-      <c r="A39" s="66" t="s">
+      <c r="A39" s="65" t="s">
         <v>42</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>324</v>
@@ -5937,11 +5954,11 @@
       </c>
     </row>
     <row r="40" spans="1:31">
-      <c r="A40" s="66" t="s">
+      <c r="A40" s="65" t="s">
         <v>43</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>324</v>
@@ -6023,11 +6040,11 @@
       </c>
     </row>
     <row r="41" spans="1:31">
-      <c r="A41" s="66" t="s">
+      <c r="A41" s="65" t="s">
         <v>44</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>324</v>
@@ -6109,11 +6126,11 @@
       </c>
     </row>
     <row r="42" spans="1:31">
-      <c r="A42" s="66" t="s">
+      <c r="A42" s="65" t="s">
         <v>45</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>324</v>
@@ -6195,11 +6212,11 @@
       </c>
     </row>
     <row r="43" spans="1:31">
-      <c r="A43" s="66" t="s">
+      <c r="A43" s="65" t="s">
         <v>46</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>324</v>
@@ -6281,11 +6298,11 @@
       </c>
     </row>
     <row r="44" spans="1:31">
-      <c r="A44" s="66" t="s">
+      <c r="A44" s="65" t="s">
         <v>47</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C44" s="6" t="s">
         <v>324</v>
@@ -6367,11 +6384,11 @@
       </c>
     </row>
     <row r="45" spans="1:31">
-      <c r="A45" s="66" t="s">
+      <c r="A45" s="65" t="s">
         <v>48</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>324</v>
@@ -6453,11 +6470,11 @@
       </c>
     </row>
     <row r="46" spans="1:31">
-      <c r="A46" s="66" t="s">
+      <c r="A46" s="65" t="s">
         <v>49</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C46" s="6" t="s">
         <v>324</v>
@@ -6539,11 +6556,11 @@
       </c>
     </row>
     <row r="47" spans="1:31">
-      <c r="A47" s="66" t="s">
+      <c r="A47" s="65" t="s">
         <v>50</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>324</v>
@@ -6625,11 +6642,11 @@
       </c>
     </row>
     <row r="48" spans="1:31">
-      <c r="A48" s="66" t="s">
+      <c r="A48" s="65" t="s">
         <v>51</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C48" s="6" t="s">
         <v>324</v>
@@ -6711,11 +6728,11 @@
       </c>
     </row>
     <row r="49" spans="1:30">
-      <c r="A49" s="66" t="s">
+      <c r="A49" s="65" t="s">
         <v>52</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>324</v>
@@ -6797,11 +6814,11 @@
       </c>
     </row>
     <row r="50" spans="1:30">
-      <c r="A50" s="66" t="s">
+      <c r="A50" s="65" t="s">
         <v>53</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>324</v>
@@ -6883,11 +6900,11 @@
       </c>
     </row>
     <row r="51" spans="1:30">
-      <c r="A51" s="66" t="s">
+      <c r="A51" s="65" t="s">
         <v>54</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>324</v>
@@ -6969,11 +6986,11 @@
       </c>
     </row>
     <row r="52" spans="1:30">
-      <c r="A52" s="66" t="s">
+      <c r="A52" s="65" t="s">
         <v>55</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>324</v>
@@ -7055,11 +7072,11 @@
       </c>
     </row>
     <row r="53" spans="1:30">
-      <c r="A53" s="66" t="s">
+      <c r="A53" s="65" t="s">
         <v>56</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>324</v>
@@ -7140,37 +7157,39 @@
         <v>0.42361575000000001</v>
       </c>
     </row>
-    <row r="54" spans="1:30" s="83" customFormat="1">
-      <c r="A54" s="80" t="s">
+    <row r="54" spans="1:30" s="81" customFormat="1">
+      <c r="A54" s="79" t="s">
         <v>57</v>
       </c>
-      <c r="B54" s="80" t="s">
-        <v>488</v>
-      </c>
-      <c r="C54" s="80" t="s">
+      <c r="B54" s="79" t="s">
+        <v>487</v>
+      </c>
+      <c r="C54" s="79" t="s">
         <v>339</v>
       </c>
-      <c r="D54" s="80" t="s">
-        <v>169</v>
-      </c>
-      <c r="E54" s="80" t="s">
+      <c r="D54" s="79" t="s">
+        <v>169</v>
+      </c>
+      <c r="E54" s="79" t="s">
         <v>301</v>
       </c>
-      <c r="F54" s="80" t="s">
+      <c r="F54" s="79" t="s">
         <v>167</v>
       </c>
-      <c r="G54" s="81"/>
-      <c r="H54" s="80"/>
-      <c r="I54" s="82">
+      <c r="G54" s="79" t="s">
+        <v>57</v>
+      </c>
+      <c r="H54" s="79"/>
+      <c r="I54" s="80">
         <v>0.1</v>
       </c>
     </row>
     <row r="55" spans="1:30" s="13" customFormat="1">
       <c r="A55" s="10" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C55" s="10" t="s">
         <v>326</v>
@@ -7205,10 +7224,10 @@
     </row>
     <row r="56" spans="1:30">
       <c r="A56" s="6" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>326</v>
@@ -7243,10 +7262,10 @@
     </row>
     <row r="57" spans="1:30">
       <c r="A57" s="6" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>326</v>
@@ -7281,10 +7300,10 @@
     </row>
     <row r="58" spans="1:30">
       <c r="A58" s="6" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>326</v>
@@ -7319,10 +7338,10 @@
     </row>
     <row r="59" spans="1:30">
       <c r="A59" s="6" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>326</v>
@@ -7360,10 +7379,10 @@
     </row>
     <row r="60" spans="1:30">
       <c r="A60" s="6" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>326</v>
@@ -7401,10 +7420,10 @@
     </row>
     <row r="61" spans="1:30">
       <c r="A61" s="6" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>326</v>
@@ -7442,10 +7461,10 @@
     </row>
     <row r="62" spans="1:30">
       <c r="A62" s="6" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>326</v>
@@ -7483,10 +7502,10 @@
     </row>
     <row r="63" spans="1:30">
       <c r="A63" s="6" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>326</v>
@@ -7524,10 +7543,10 @@
     </row>
     <row r="64" spans="1:30" s="14" customFormat="1">
       <c r="A64" s="11" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C64" s="11" t="s">
         <v>326</v>
@@ -7564,7 +7583,7 @@
       </c>
     </row>
     <row r="65" spans="1:30" s="13" customFormat="1">
-      <c r="A65" s="67" t="s">
+      <c r="A65" s="66" t="s">
         <v>62</v>
       </c>
       <c r="B65" s="10" t="s">
@@ -7582,14 +7601,16 @@
       <c r="F65" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="G65" s="58"/>
+      <c r="G65" s="66" t="s">
+        <v>62</v>
+      </c>
       <c r="H65" s="10"/>
       <c r="I65" s="13">
         <v>0.1</v>
       </c>
     </row>
     <row r="66" spans="1:30">
-      <c r="A66" s="68" t="s">
+      <c r="A66" s="67" t="s">
         <v>63</v>
       </c>
       <c r="B66" s="6" t="s">
@@ -7607,14 +7628,16 @@
       <c r="F66" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G66" s="59"/>
+      <c r="G66" s="67" t="s">
+        <v>63</v>
+      </c>
       <c r="H66" s="6"/>
       <c r="I66" s="5">
         <v>0.1</v>
       </c>
     </row>
     <row r="67" spans="1:30">
-      <c r="A67" s="68" t="s">
+      <c r="A67" s="67" t="s">
         <v>64</v>
       </c>
       <c r="B67" s="6" t="s">
@@ -7632,14 +7655,16 @@
       <c r="F67" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G67" s="59"/>
+      <c r="G67" s="67" t="s">
+        <v>64</v>
+      </c>
       <c r="H67" s="6"/>
       <c r="I67" s="5">
         <v>0.1</v>
       </c>
     </row>
     <row r="68" spans="1:30">
-      <c r="A68" s="68" t="s">
+      <c r="A68" s="67" t="s">
         <v>65</v>
       </c>
       <c r="B68" s="6" t="s">
@@ -7657,14 +7682,16 @@
       <c r="F68" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G68" s="59"/>
+      <c r="G68" s="67" t="s">
+        <v>65</v>
+      </c>
       <c r="H68" s="6"/>
       <c r="I68" s="5">
         <v>0.1</v>
       </c>
     </row>
     <row r="69" spans="1:30">
-      <c r="A69" s="68" t="s">
+      <c r="A69" s="67" t="s">
         <v>66</v>
       </c>
       <c r="B69" s="6" t="s">
@@ -7682,11 +7709,13 @@
       <c r="F69" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G69" s="59"/>
+      <c r="G69" s="67" t="s">
+        <v>516</v>
+      </c>
       <c r="H69" s="6"/>
     </row>
     <row r="70" spans="1:30">
-      <c r="A70" s="68" t="s">
+      <c r="A70" s="67" t="s">
         <v>67</v>
       </c>
       <c r="B70" s="6" t="s">
@@ -7704,11 +7733,13 @@
       <c r="F70" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G70" s="59"/>
+      <c r="G70" s="67" t="s">
+        <v>516</v>
+      </c>
       <c r="H70" s="6"/>
     </row>
     <row r="71" spans="1:30">
-      <c r="A71" s="68" t="s">
+      <c r="A71" s="67" t="s">
         <v>68</v>
       </c>
       <c r="B71" s="6" t="s">
@@ -7726,11 +7757,13 @@
       <c r="F71" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G71" s="59"/>
+      <c r="G71" s="67" t="s">
+        <v>516</v>
+      </c>
       <c r="H71" s="6"/>
     </row>
     <row r="72" spans="1:30">
-      <c r="A72" s="68" t="s">
+      <c r="A72" s="67" t="s">
         <v>69</v>
       </c>
       <c r="B72" s="6" t="s">
@@ -7748,15 +7781,17 @@
       <c r="F72" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G72" s="59"/>
+      <c r="G72" s="67" t="s">
+        <v>516</v>
+      </c>
       <c r="H72" s="6"/>
     </row>
     <row r="73" spans="1:30" s="29" customFormat="1">
-      <c r="A73" s="69" t="s">
-        <v>418</v>
+      <c r="A73" s="68" t="s">
+        <v>417</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C73" s="10" t="s">
         <v>327</v>
@@ -7770,7 +7805,7 @@
       <c r="F73" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="G73" s="62" t="s">
+      <c r="G73" s="61" t="s">
         <v>104</v>
       </c>
       <c r="H73" s="22" t="s">
@@ -7805,11 +7840,11 @@
       </c>
     </row>
     <row r="74" spans="1:30" s="30" customFormat="1">
-      <c r="A74" s="70" t="s">
-        <v>419</v>
+      <c r="A74" s="69" t="s">
+        <v>418</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C74" s="6" t="s">
         <v>327</v>
@@ -7823,7 +7858,7 @@
       <c r="F74" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G74" s="63" t="s">
+      <c r="G74" s="62" t="s">
         <v>104</v>
       </c>
       <c r="H74" s="12" t="s">
@@ -7858,11 +7893,11 @@
       </c>
     </row>
     <row r="75" spans="1:30" s="30" customFormat="1">
-      <c r="A75" s="70" t="s">
-        <v>420</v>
+      <c r="A75" s="69" t="s">
+        <v>419</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C75" s="6" t="s">
         <v>327</v>
@@ -7876,7 +7911,7 @@
       <c r="F75" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G75" s="63" t="s">
+      <c r="G75" s="62" t="s">
         <v>104</v>
       </c>
       <c r="H75" s="12" t="s">
@@ -7911,14 +7946,14 @@
       </c>
     </row>
     <row r="76" spans="1:30">
-      <c r="A76" s="70" t="s">
-        <v>421</v>
+      <c r="A76" s="69" t="s">
+        <v>420</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D76" s="6" t="s">
         <v>170</v>
@@ -7964,14 +7999,14 @@
       </c>
     </row>
     <row r="77" spans="1:30">
-      <c r="A77" s="70" t="s">
-        <v>422</v>
+      <c r="A77" s="69" t="s">
+        <v>421</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>170</v>
@@ -8017,14 +8052,14 @@
       </c>
     </row>
     <row r="78" spans="1:30">
-      <c r="A78" s="70" t="s">
-        <v>423</v>
+      <c r="A78" s="69" t="s">
+        <v>422</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D78" s="6" t="s">
         <v>170</v>
@@ -8070,14 +8105,14 @@
       </c>
     </row>
     <row r="79" spans="1:30">
-      <c r="A79" s="70" t="s">
-        <v>424</v>
+      <c r="A79" s="69" t="s">
+        <v>423</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D79" s="6" t="s">
         <v>170</v>
@@ -8123,14 +8158,14 @@
       </c>
     </row>
     <row r="80" spans="1:30">
-      <c r="A80" s="70" t="s">
-        <v>425</v>
+      <c r="A80" s="69" t="s">
+        <v>424</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D80" s="6" t="s">
         <v>170</v>
@@ -8176,14 +8211,14 @@
       </c>
     </row>
     <row r="81" spans="1:30">
-      <c r="A81" s="70" t="s">
-        <v>426</v>
+      <c r="A81" s="69" t="s">
+        <v>425</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D81" s="6" t="s">
         <v>170</v>
@@ -8229,14 +8264,14 @@
       </c>
     </row>
     <row r="82" spans="1:30">
-      <c r="A82" s="70" t="s">
-        <v>427</v>
+      <c r="A82" s="69" t="s">
+        <v>426</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D82" s="6" t="s">
         <v>170</v>
@@ -8282,14 +8317,14 @@
       </c>
     </row>
     <row r="83" spans="1:30">
-      <c r="A83" s="70" t="s">
-        <v>428</v>
+      <c r="A83" s="69" t="s">
+        <v>427</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D83" s="6" t="s">
         <v>170</v>
@@ -8335,14 +8370,14 @@
       </c>
     </row>
     <row r="84" spans="1:30">
-      <c r="A84" s="70" t="s">
-        <v>429</v>
+      <c r="A84" s="69" t="s">
+        <v>428</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D84" s="6" t="s">
         <v>170</v>
@@ -8388,14 +8423,14 @@
       </c>
     </row>
     <row r="85" spans="1:30">
-      <c r="A85" s="70" t="s">
-        <v>430</v>
+      <c r="A85" s="69" t="s">
+        <v>429</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="D85" s="6" t="s">
         <v>170</v>
@@ -8441,14 +8476,14 @@
       </c>
     </row>
     <row r="86" spans="1:30">
-      <c r="A86" s="70" t="s">
-        <v>431</v>
+      <c r="A86" s="69" t="s">
+        <v>430</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="D86" s="6" t="s">
         <v>170</v>
@@ -8494,14 +8529,14 @@
       </c>
     </row>
     <row r="87" spans="1:30">
-      <c r="A87" s="70" t="s">
-        <v>432</v>
+      <c r="A87" s="69" t="s">
+        <v>431</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="D87" s="6" t="s">
         <v>170</v>
@@ -8547,14 +8582,14 @@
       </c>
     </row>
     <row r="88" spans="1:30">
-      <c r="A88" s="70" t="s">
-        <v>433</v>
+      <c r="A88" s="69" t="s">
+        <v>432</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D88" s="6" t="s">
         <v>170</v>
@@ -8600,14 +8635,14 @@
       </c>
     </row>
     <row r="89" spans="1:30">
-      <c r="A89" s="70" t="s">
-        <v>434</v>
+      <c r="A89" s="69" t="s">
+        <v>433</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D89" s="6" t="s">
         <v>170</v>
@@ -8653,14 +8688,14 @@
       </c>
     </row>
     <row r="90" spans="1:30">
-      <c r="A90" s="70" t="s">
-        <v>435</v>
+      <c r="A90" s="69" t="s">
+        <v>434</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D90" s="6" t="s">
         <v>170</v>
@@ -8706,14 +8741,14 @@
       </c>
     </row>
     <row r="91" spans="1:30">
-      <c r="A91" s="70" t="s">
-        <v>436</v>
+      <c r="A91" s="69" t="s">
+        <v>435</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="D91" s="6" t="s">
         <v>170</v>
@@ -8759,14 +8794,14 @@
       </c>
     </row>
     <row r="92" spans="1:30">
-      <c r="A92" s="70" t="s">
-        <v>437</v>
+      <c r="A92" s="69" t="s">
+        <v>436</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="D92" s="6" t="s">
         <v>170</v>
@@ -8812,14 +8847,14 @@
       </c>
     </row>
     <row r="93" spans="1:30">
-      <c r="A93" s="70" t="s">
-        <v>438</v>
+      <c r="A93" s="69" t="s">
+        <v>437</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="D93" s="6" t="s">
         <v>170</v>
@@ -8865,14 +8900,14 @@
       </c>
     </row>
     <row r="94" spans="1:30">
-      <c r="A94" s="70" t="s">
-        <v>439</v>
+      <c r="A94" s="69" t="s">
+        <v>438</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="D94" s="6" t="s">
         <v>170</v>
@@ -8918,14 +8953,14 @@
       </c>
     </row>
     <row r="95" spans="1:30">
-      <c r="A95" s="70" t="s">
-        <v>440</v>
+      <c r="A95" s="69" t="s">
+        <v>439</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="D95" s="6" t="s">
         <v>170</v>
@@ -8971,14 +9006,14 @@
       </c>
     </row>
     <row r="96" spans="1:30">
-      <c r="A96" s="70" t="s">
-        <v>441</v>
+      <c r="A96" s="69" t="s">
+        <v>440</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="D96" s="6" t="s">
         <v>170</v>
@@ -9024,14 +9059,14 @@
       </c>
     </row>
     <row r="97" spans="1:30">
-      <c r="A97" s="70" t="s">
-        <v>442</v>
+      <c r="A97" s="69" t="s">
+        <v>441</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D97" s="6" t="s">
         <v>170</v>
@@ -9077,14 +9112,14 @@
       </c>
     </row>
     <row r="98" spans="1:30">
-      <c r="A98" s="70" t="s">
-        <v>443</v>
+      <c r="A98" s="69" t="s">
+        <v>442</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C98" s="6" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D98" s="6" t="s">
         <v>170</v>
@@ -9130,14 +9165,14 @@
       </c>
     </row>
     <row r="99" spans="1:30" s="14" customFormat="1">
-      <c r="A99" s="71" t="s">
-        <v>444</v>
+      <c r="A99" s="70" t="s">
+        <v>443</v>
       </c>
       <c r="B99" s="11" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C99" s="11" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D99" s="11" t="s">
         <v>170</v>
@@ -9183,11 +9218,11 @@
       </c>
     </row>
     <row r="100" spans="1:30">
-      <c r="A100" s="72" t="s">
+      <c r="A100" s="71" t="s">
         <v>106</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C100" s="6" t="s">
         <v>328</v>
@@ -9201,7 +9236,7 @@
       <c r="F100" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G100" s="72" t="s">
+      <c r="G100" s="71" t="s">
         <v>106</v>
       </c>
       <c r="H100" s="12" t="s">
@@ -9212,11 +9247,11 @@
       </c>
     </row>
     <row r="101" spans="1:30">
-      <c r="A101" s="72" t="s">
+      <c r="A101" s="71" t="s">
         <v>107</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C101" s="6" t="s">
         <v>328</v>
@@ -9230,7 +9265,7 @@
       <c r="F101" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G101" s="72" t="s">
+      <c r="G101" s="71" t="s">
         <v>107</v>
       </c>
       <c r="H101" s="12" t="s">
@@ -9241,11 +9276,11 @@
       </c>
     </row>
     <row r="102" spans="1:30">
-      <c r="A102" s="72" t="s">
+      <c r="A102" s="71" t="s">
         <v>108</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C102" s="6" t="s">
         <v>328</v>
@@ -9259,7 +9294,7 @@
       <c r="F102" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G102" s="72" t="s">
+      <c r="G102" s="71" t="s">
         <v>108</v>
       </c>
       <c r="H102" s="12" t="s">
@@ -9270,11 +9305,11 @@
       </c>
     </row>
     <row r="103" spans="1:30">
-      <c r="A103" s="72" t="s">
+      <c r="A103" s="71" t="s">
         <v>109</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C103" s="6" t="s">
         <v>328</v>
@@ -9288,7 +9323,7 @@
       <c r="F103" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G103" s="72" t="s">
+      <c r="G103" s="71" t="s">
         <v>109</v>
       </c>
       <c r="H103" s="12" t="s">
@@ -9299,11 +9334,11 @@
       </c>
     </row>
     <row r="104" spans="1:30">
-      <c r="A104" s="72" t="s">
+      <c r="A104" s="71" t="s">
         <v>110</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C104" s="6" t="s">
         <v>328</v>
@@ -9317,7 +9352,7 @@
       <c r="F104" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G104" s="72" t="s">
+      <c r="G104" s="71" t="s">
         <v>110</v>
       </c>
       <c r="H104" s="12" t="s">
@@ -9328,11 +9363,11 @@
       </c>
     </row>
     <row r="105" spans="1:30">
-      <c r="A105" s="72" t="s">
+      <c r="A105" s="71" t="s">
         <v>111</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C105" s="6" t="s">
         <v>328</v>
@@ -9346,7 +9381,7 @@
       <c r="F105" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G105" s="72" t="s">
+      <c r="G105" s="71" t="s">
         <v>111</v>
       </c>
       <c r="H105" s="12" t="s">
@@ -9357,11 +9392,11 @@
       </c>
     </row>
     <row r="106" spans="1:30">
-      <c r="A106" s="72" t="s">
+      <c r="A106" s="71" t="s">
         <v>112</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C106" s="6" t="s">
         <v>328</v>
@@ -9375,7 +9410,7 @@
       <c r="F106" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G106" s="72" t="s">
+      <c r="G106" s="71" t="s">
         <v>112</v>
       </c>
       <c r="H106" s="12" t="s">
@@ -9386,11 +9421,11 @@
       </c>
     </row>
     <row r="107" spans="1:30">
-      <c r="A107" s="72" t="s">
+      <c r="A107" s="71" t="s">
         <v>113</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C107" s="6" t="s">
         <v>328</v>
@@ -9404,7 +9439,7 @@
       <c r="F107" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G107" s="72" t="s">
+      <c r="G107" s="71" t="s">
         <v>113</v>
       </c>
       <c r="H107" s="12" t="s">
@@ -9415,11 +9450,11 @@
       </c>
     </row>
     <row r="108" spans="1:30">
-      <c r="A108" s="72" t="s">
+      <c r="A108" s="71" t="s">
         <v>114</v>
       </c>
       <c r="B108" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C108" s="6" t="s">
         <v>328</v>
@@ -9433,7 +9468,7 @@
       <c r="F108" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G108" s="72" t="s">
+      <c r="G108" s="71" t="s">
         <v>114</v>
       </c>
       <c r="H108" s="12" t="s">
@@ -9444,11 +9479,11 @@
       </c>
     </row>
     <row r="109" spans="1:30" ht="14" customHeight="1">
-      <c r="A109" s="72" t="s">
+      <c r="A109" s="71" t="s">
         <v>115</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C109" s="6" t="s">
         <v>328</v>
@@ -9462,7 +9497,7 @@
       <c r="F109" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G109" s="72" t="s">
+      <c r="G109" s="71" t="s">
         <v>115</v>
       </c>
       <c r="H109" s="12" t="s">
@@ -9492,7 +9527,7 @@
         <v>128</v>
       </c>
       <c r="G110" s="10" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="H110" s="13" t="s">
         <v>209</v>
@@ -9524,7 +9559,7 @@
         <v>128</v>
       </c>
       <c r="G111" s="6" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="H111" s="5" t="s">
         <v>209</v>
@@ -9556,7 +9591,7 @@
         <v>128</v>
       </c>
       <c r="G112" s="6" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="H112" s="5" t="s">
         <v>209</v>
@@ -9588,7 +9623,7 @@
         <v>128</v>
       </c>
       <c r="G113" s="6" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="H113" s="5" t="s">
         <v>209</v>
@@ -9620,7 +9655,7 @@
         <v>128</v>
       </c>
       <c r="G114" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="H114" s="5" t="s">
         <v>209</v>
@@ -9652,7 +9687,7 @@
         <v>128</v>
       </c>
       <c r="G115" s="6" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="H115" s="5" t="s">
         <v>209</v>
@@ -9684,7 +9719,7 @@
         <v>128</v>
       </c>
       <c r="G116" s="6" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="H116" s="5" t="s">
         <v>209</v>
@@ -9716,7 +9751,7 @@
         <v>128</v>
       </c>
       <c r="G117" s="6" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="H117" s="5" t="s">
         <v>209</v>
@@ -9748,7 +9783,7 @@
         <v>128</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H118" s="5" t="s">
         <v>209</v>
@@ -9780,7 +9815,7 @@
         <v>128</v>
       </c>
       <c r="G119" s="6" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H119" s="5" t="s">
         <v>209</v>
@@ -9812,7 +9847,7 @@
         <v>128</v>
       </c>
       <c r="G120" s="11" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="H120" s="14" t="s">
         <v>209</v>
@@ -9825,11 +9860,11 @@
       </c>
     </row>
     <row r="121" spans="1:24" s="13" customFormat="1">
-      <c r="A121" s="73" t="s">
+      <c r="A121" s="72" t="s">
         <v>129</v>
       </c>
       <c r="B121" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C121" s="10" t="s">
         <v>322</v>
@@ -9851,11 +9886,11 @@
       </c>
     </row>
     <row r="122" spans="1:24">
-      <c r="A122" s="74" t="s">
+      <c r="A122" s="73" t="s">
         <v>130</v>
       </c>
       <c r="B122" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C122" s="6" t="s">
         <v>322</v>
@@ -9877,11 +9912,11 @@
       </c>
     </row>
     <row r="123" spans="1:24">
-      <c r="A123" s="74" t="s">
+      <c r="A123" s="73" t="s">
         <v>131</v>
       </c>
       <c r="B123" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C123" s="6" t="s">
         <v>322</v>
@@ -9903,11 +9938,11 @@
       </c>
     </row>
     <row r="124" spans="1:24">
-      <c r="A124" s="74" t="s">
+      <c r="A124" s="73" t="s">
         <v>132</v>
       </c>
       <c r="B124" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C124" s="6" t="s">
         <v>322</v>
@@ -9929,11 +9964,11 @@
       </c>
     </row>
     <row r="125" spans="1:24">
-      <c r="A125" s="74" t="s">
+      <c r="A125" s="73" t="s">
         <v>133</v>
       </c>
       <c r="B125" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C125" s="6" t="s">
         <v>322</v>
@@ -9955,11 +9990,11 @@
       </c>
     </row>
     <row r="126" spans="1:24">
-      <c r="A126" s="74" t="s">
+      <c r="A126" s="73" t="s">
         <v>134</v>
       </c>
       <c r="B126" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C126" s="6" t="s">
         <v>322</v>
@@ -9981,11 +10016,11 @@
       </c>
     </row>
     <row r="127" spans="1:24">
-      <c r="A127" s="74" t="s">
+      <c r="A127" s="73" t="s">
         <v>135</v>
       </c>
       <c r="B127" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C127" s="6" t="s">
         <v>322</v>
@@ -10007,11 +10042,11 @@
       </c>
     </row>
     <row r="128" spans="1:24">
-      <c r="A128" s="74" t="s">
+      <c r="A128" s="73" t="s">
         <v>136</v>
       </c>
       <c r="B128" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C128" s="6" t="s">
         <v>322</v>
@@ -10033,11 +10068,11 @@
       </c>
     </row>
     <row r="129" spans="1:9">
-      <c r="A129" s="74" t="s">
+      <c r="A129" s="73" t="s">
         <v>137</v>
       </c>
       <c r="B129" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C129" s="6" t="s">
         <v>322</v>
@@ -10059,11 +10094,11 @@
       </c>
     </row>
     <row r="130" spans="1:9">
-      <c r="A130" s="74" t="s">
+      <c r="A130" s="73" t="s">
         <v>138</v>
       </c>
       <c r="B130" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C130" s="6" t="s">
         <v>322</v>
@@ -10085,11 +10120,11 @@
       </c>
     </row>
     <row r="131" spans="1:9">
-      <c r="A131" s="74" t="s">
+      <c r="A131" s="73" t="s">
         <v>139</v>
       </c>
       <c r="B131" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C131" s="6" t="s">
         <v>322</v>
@@ -10111,11 +10146,11 @@
       </c>
     </row>
     <row r="132" spans="1:9">
-      <c r="A132" s="74" t="s">
+      <c r="A132" s="73" t="s">
         <v>140</v>
       </c>
       <c r="B132" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C132" s="6" t="s">
         <v>322</v>
@@ -10137,11 +10172,11 @@
       </c>
     </row>
     <row r="133" spans="1:9">
-      <c r="A133" s="74" t="s">
+      <c r="A133" s="73" t="s">
         <v>141</v>
       </c>
       <c r="B133" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C133" s="6" t="s">
         <v>322</v>
@@ -10163,11 +10198,11 @@
       </c>
     </row>
     <row r="134" spans="1:9">
-      <c r="A134" s="74" t="s">
+      <c r="A134" s="73" t="s">
         <v>142</v>
       </c>
       <c r="B134" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C134" s="6" t="s">
         <v>322</v>
@@ -10189,11 +10224,11 @@
       </c>
     </row>
     <row r="135" spans="1:9">
-      <c r="A135" s="74" t="s">
+      <c r="A135" s="73" t="s">
         <v>143</v>
       </c>
       <c r="B135" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C135" s="6" t="s">
         <v>322</v>
@@ -10215,11 +10250,11 @@
       </c>
     </row>
     <row r="136" spans="1:9">
-      <c r="A136" s="74" t="s">
+      <c r="A136" s="73" t="s">
         <v>144</v>
       </c>
       <c r="B136" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C136" s="6" t="s">
         <v>322</v>
@@ -10241,11 +10276,11 @@
       </c>
     </row>
     <row r="137" spans="1:9">
-      <c r="A137" s="74" t="s">
+      <c r="A137" s="73" t="s">
         <v>145</v>
       </c>
       <c r="B137" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C137" s="6" t="s">
         <v>322</v>
@@ -10267,11 +10302,11 @@
       </c>
     </row>
     <row r="138" spans="1:9">
-      <c r="A138" s="74" t="s">
+      <c r="A138" s="73" t="s">
         <v>146</v>
       </c>
       <c r="B138" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C138" s="6" t="s">
         <v>322</v>
@@ -10293,11 +10328,11 @@
       </c>
     </row>
     <row r="139" spans="1:9">
-      <c r="A139" s="74" t="s">
+      <c r="A139" s="73" t="s">
         <v>147</v>
       </c>
       <c r="B139" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C139" s="6" t="s">
         <v>322</v>
@@ -10319,11 +10354,11 @@
       </c>
     </row>
     <row r="140" spans="1:9">
-      <c r="A140" s="74" t="s">
+      <c r="A140" s="73" t="s">
         <v>148</v>
       </c>
       <c r="B140" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C140" s="6" t="s">
         <v>322</v>
@@ -10345,11 +10380,11 @@
       </c>
     </row>
     <row r="141" spans="1:9">
-      <c r="A141" s="74" t="s">
+      <c r="A141" s="73" t="s">
         <v>149</v>
       </c>
       <c r="B141" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C141" s="6" t="s">
         <v>322</v>
@@ -10371,11 +10406,11 @@
       </c>
     </row>
     <row r="142" spans="1:9">
-      <c r="A142" s="74" t="s">
+      <c r="A142" s="73" t="s">
         <v>150</v>
       </c>
       <c r="B142" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C142" s="6" t="s">
         <v>322</v>
@@ -10397,11 +10432,11 @@
       </c>
     </row>
     <row r="143" spans="1:9">
-      <c r="A143" s="74" t="s">
+      <c r="A143" s="73" t="s">
         <v>151</v>
       </c>
       <c r="B143" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C143" s="6" t="s">
         <v>322</v>
@@ -10423,11 +10458,11 @@
       </c>
     </row>
     <row r="144" spans="1:9">
-      <c r="A144" s="74" t="s">
+      <c r="A144" s="73" t="s">
         <v>152</v>
       </c>
       <c r="B144" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C144" s="6" t="s">
         <v>322</v>
@@ -10449,11 +10484,11 @@
       </c>
     </row>
     <row r="145" spans="1:25">
-      <c r="A145" s="74" t="s">
+      <c r="A145" s="73" t="s">
         <v>153</v>
       </c>
       <c r="B145" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C145" s="6" t="s">
         <v>322</v>
@@ -10475,11 +10510,11 @@
       </c>
     </row>
     <row r="146" spans="1:25">
-      <c r="A146" s="74" t="s">
+      <c r="A146" s="73" t="s">
         <v>154</v>
       </c>
       <c r="B146" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C146" s="6" t="s">
         <v>322</v>
@@ -10501,11 +10536,11 @@
       </c>
     </row>
     <row r="147" spans="1:25">
-      <c r="A147" s="74" t="s">
+      <c r="A147" s="73" t="s">
         <v>155</v>
       </c>
       <c r="B147" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C147" s="6" t="s">
         <v>322</v>
@@ -10527,11 +10562,11 @@
       </c>
     </row>
     <row r="148" spans="1:25">
-      <c r="A148" s="74" t="s">
+      <c r="A148" s="73" t="s">
         <v>156</v>
       </c>
       <c r="B148" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C148" s="6" t="s">
         <v>322</v>
@@ -10553,11 +10588,11 @@
       </c>
     </row>
     <row r="149" spans="1:25">
-      <c r="A149" s="74" t="s">
+      <c r="A149" s="73" t="s">
         <v>157</v>
       </c>
       <c r="B149" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C149" s="6" t="s">
         <v>322</v>
@@ -10579,11 +10614,11 @@
       </c>
     </row>
     <row r="150" spans="1:25" s="14" customFormat="1">
-      <c r="A150" s="75" t="s">
+      <c r="A150" s="74" t="s">
         <v>158</v>
       </c>
       <c r="B150" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C150" s="11" t="s">
         <v>322</v>
@@ -10609,7 +10644,7 @@
         <v>159</v>
       </c>
       <c r="B151" s="10" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C151" s="10" t="s">
         <v>323</v>
@@ -10644,7 +10679,7 @@
         <v>160</v>
       </c>
       <c r="B152" s="10" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C152" s="6" t="s">
         <v>323</v>
@@ -10679,7 +10714,7 @@
         <v>161</v>
       </c>
       <c r="B153" s="10" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C153" s="6" t="s">
         <v>323</v>
@@ -10714,7 +10749,7 @@
         <v>162</v>
       </c>
       <c r="B154" s="10" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C154" s="6" t="s">
         <v>323</v>
@@ -10749,7 +10784,7 @@
         <v>163</v>
       </c>
       <c r="B155" s="10" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C155" s="6" t="s">
         <v>323</v>
@@ -10784,7 +10819,7 @@
         <v>164</v>
       </c>
       <c r="B156" s="10" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C156" s="6" t="s">
         <v>323</v>
@@ -10819,7 +10854,7 @@
         <v>165</v>
       </c>
       <c r="B157" s="10" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C157" s="6" t="s">
         <v>323</v>
@@ -10854,7 +10889,7 @@
         <v>166</v>
       </c>
       <c r="B158" s="10" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C158" s="6" t="s">
         <v>323</v>
@@ -10891,7 +10926,7 @@
       <c r="B159" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="C159" s="86" t="s">
+      <c r="C159" s="84" t="s">
         <v>307</v>
       </c>
       <c r="D159" s="36" t="s">
@@ -10903,8 +10938,8 @@
       <c r="F159" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="G159" s="84" t="s">
-        <v>492</v>
+      <c r="G159" s="82" t="s">
+        <v>491</v>
       </c>
       <c r="I159" s="13">
         <v>5.1999999999999998E-2</v>
@@ -10930,8 +10965,8 @@
       <c r="F160" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G160" s="85" t="s">
-        <v>492</v>
+      <c r="G160" s="83" t="s">
+        <v>491</v>
       </c>
       <c r="I160" s="5">
         <v>5.0999999999999997E-2</v>
@@ -10956,8 +10991,8 @@
       <c r="F161" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G161" s="85" t="s">
-        <v>492</v>
+      <c r="G161" s="83" t="s">
+        <v>491</v>
       </c>
       <c r="I161" s="5">
         <v>4.8000000000000001E-2</v>
@@ -10982,8 +11017,8 @@
       <c r="F162" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G162" s="85" t="s">
-        <v>492</v>
+      <c r="G162" s="83" t="s">
+        <v>491</v>
       </c>
       <c r="I162" s="5">
         <v>4.7E-2</v>
@@ -11009,7 +11044,7 @@
         <v>128</v>
       </c>
       <c r="G163" s="6" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="I163" s="5">
         <v>0.16500000000000001</v>
@@ -11035,7 +11070,7 @@
         <v>128</v>
       </c>
       <c r="G164" s="6" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="I164" s="5">
         <v>0.182</v>
@@ -11061,7 +11096,7 @@
         <v>128</v>
       </c>
       <c r="G165" s="6" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="I165" s="5">
         <v>0.27500000000000002</v>
@@ -11087,7 +11122,7 @@
         <v>128</v>
       </c>
       <c r="G166" s="6" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="I166" s="5">
         <v>0.29099999999999998</v>
@@ -11113,7 +11148,7 @@
         <v>128</v>
       </c>
       <c r="G167" s="6" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="I167" s="5">
         <v>0.373</v>
@@ -11139,7 +11174,7 @@
         <v>128</v>
       </c>
       <c r="G168" s="6" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="I168" s="5">
         <v>0.36899999999999999</v>
@@ -11165,7 +11200,7 @@
         <v>128</v>
       </c>
       <c r="G169" s="5" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="I169" s="5">
         <v>0.121</v>
@@ -11191,7 +11226,7 @@
         <v>128</v>
       </c>
       <c r="G170" s="5" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="I170" s="5">
         <v>0.106</v>
@@ -11217,7 +11252,7 @@
         <v>128</v>
       </c>
       <c r="G171" s="5" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="I171" s="5">
         <v>0.2</v>
@@ -11243,7 +11278,7 @@
         <v>128</v>
       </c>
       <c r="G172" s="5" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="I172" s="5">
         <v>0.20100000000000001</v>
@@ -11269,7 +11304,7 @@
         <v>128</v>
       </c>
       <c r="G173" s="5" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="I173" s="5">
         <v>0.32700000000000001</v>
@@ -11295,7 +11330,7 @@
         <v>128</v>
       </c>
       <c r="G174" s="5" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="I174" s="5">
         <v>0.318</v>
@@ -11321,7 +11356,7 @@
         <v>128</v>
       </c>
       <c r="G175" s="5" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="I175" s="5">
         <v>0.42099999999999999</v>
@@ -11347,7 +11382,7 @@
         <v>128</v>
       </c>
       <c r="G176" s="5" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="I176" s="5">
         <v>0.39900000000000002</v>
@@ -11372,6 +11407,9 @@
       <c r="F177" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G177" s="6" t="s">
+        <v>514</v>
+      </c>
       <c r="I177" s="5">
         <v>0.19600000000000001</v>
       </c>
@@ -11395,6 +11433,9 @@
       <c r="F178" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G178" s="6" t="s">
+        <v>514</v>
+      </c>
       <c r="I178" s="5">
         <v>0.20200000000000001</v>
       </c>
@@ -11418,6 +11459,9 @@
       <c r="F179" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G179" s="6" t="s">
+        <v>515</v>
+      </c>
       <c r="I179" s="5">
         <v>0.22900000000000001</v>
       </c>
@@ -11441,6 +11485,9 @@
       <c r="F180" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G180" s="6" t="s">
+        <v>515</v>
+      </c>
       <c r="I180" s="5">
         <v>0.22500000000000001</v>
       </c>
@@ -11464,6 +11511,9 @@
       <c r="F181" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G181" s="6" t="s">
+        <v>513</v>
+      </c>
       <c r="I181" s="5">
         <v>0.26800000000000002</v>
       </c>
@@ -11487,6 +11537,9 @@
       <c r="F182" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G182" s="6" t="s">
+        <v>513</v>
+      </c>
       <c r="I182" s="5">
         <v>0.27300000000000002</v>
       </c>
@@ -11510,6 +11563,9 @@
       <c r="F183" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G183" s="6" t="s">
+        <v>512</v>
+      </c>
       <c r="I183" s="5">
         <v>0.30299999999999999</v>
       </c>
@@ -11533,6 +11589,9 @@
       <c r="F184" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G184" s="6" t="s">
+        <v>512</v>
+      </c>
       <c r="I184" s="5">
         <v>0.30199999999999999</v>
       </c>
@@ -11556,6 +11615,9 @@
       <c r="F185" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G185" s="6" t="s">
+        <v>512</v>
+      </c>
       <c r="I185" s="5">
         <v>0.3</v>
       </c>
@@ -11579,6 +11641,9 @@
       <c r="F186" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G186" s="6" t="s">
+        <v>512</v>
+      </c>
       <c r="I186" s="5">
         <v>0.30099999999999999</v>
       </c>
@@ -11602,6 +11667,9 @@
       <c r="F187" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G187" s="6" t="s">
+        <v>511</v>
+      </c>
       <c r="I187" s="5">
         <v>0.316</v>
       </c>
@@ -11625,6 +11693,9 @@
       <c r="F188" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G188" s="6" t="s">
+        <v>511</v>
+      </c>
       <c r="I188" s="5">
         <v>0.32</v>
       </c>
@@ -11648,6 +11719,9 @@
       <c r="F189" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G189" s="6" t="s">
+        <v>510</v>
+      </c>
       <c r="I189" s="5">
         <v>0.33700000000000002</v>
       </c>
@@ -11671,12 +11745,15 @@
       <c r="F190" s="14" t="s">
         <v>167</v>
       </c>
+      <c r="G190" s="11" t="s">
+        <v>510</v>
+      </c>
       <c r="I190" s="14">
         <v>0.34</v>
       </c>
     </row>
     <row r="191" spans="1:9" s="13" customFormat="1">
-      <c r="A191" s="76" t="s">
+      <c r="A191" s="75" t="s">
         <v>210</v>
       </c>
       <c r="B191" s="13" t="s">
@@ -11693,6 +11770,9 @@
       </c>
       <c r="F191" s="13" t="s">
         <v>128</v>
+      </c>
+      <c r="G191" s="75" t="s">
+        <v>210</v>
       </c>
       <c r="I191" s="37">
         <v>0.255</v>
@@ -11717,6 +11797,9 @@
       <c r="F192" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G192" s="20" t="s">
+        <v>211</v>
+      </c>
       <c r="I192" s="17">
         <v>0.08</v>
       </c>
@@ -11740,6 +11823,9 @@
       <c r="F193" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G193" s="20" t="s">
+        <v>212</v>
+      </c>
       <c r="I193" s="17">
         <v>0.16</v>
       </c>
@@ -11763,6 +11849,9 @@
       <c r="F194" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G194" s="20" t="s">
+        <v>213</v>
+      </c>
       <c r="I194" s="17">
         <v>0.22</v>
       </c>
@@ -11786,6 +11875,9 @@
       <c r="F195" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G195" s="20" t="s">
+        <v>214</v>
+      </c>
       <c r="I195" s="17">
         <v>0.28000000000000003</v>
       </c>
@@ -11809,6 +11901,9 @@
       <c r="F196" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G196" s="20" t="s">
+        <v>215</v>
+      </c>
       <c r="I196" s="17">
         <v>0.08</v>
       </c>
@@ -11832,6 +11927,9 @@
       <c r="F197" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G197" s="20" t="s">
+        <v>216</v>
+      </c>
       <c r="I197" s="17">
         <v>0.16</v>
       </c>
@@ -11855,6 +11953,9 @@
       <c r="F198" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G198" s="20" t="s">
+        <v>217</v>
+      </c>
       <c r="I198" s="17">
         <v>0.22</v>
       </c>
@@ -11878,6 +11979,9 @@
       <c r="F199" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G199" s="20" t="s">
+        <v>218</v>
+      </c>
       <c r="I199" s="17">
         <v>0.28000000000000003</v>
       </c>
@@ -11901,6 +12005,9 @@
       <c r="F200" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G200" s="20" t="s">
+        <v>219</v>
+      </c>
       <c r="I200" s="17">
         <v>0.08</v>
       </c>
@@ -11924,6 +12031,9 @@
       <c r="F201" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G201" s="20" t="s">
+        <v>220</v>
+      </c>
       <c r="I201" s="17">
         <v>0.16</v>
       </c>
@@ -11947,6 +12057,9 @@
       <c r="F202" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G202" s="20" t="s">
+        <v>221</v>
+      </c>
       <c r="I202" s="17">
         <v>0.22</v>
       </c>
@@ -11970,6 +12083,9 @@
       <c r="F203" s="5" t="s">
         <v>167</v>
       </c>
+      <c r="G203" s="20" t="s">
+        <v>222</v>
+      </c>
       <c r="I203" s="17">
         <v>0.28000000000000003</v>
       </c>
@@ -12162,7 +12278,7 @@
       </c>
     </row>
     <row r="212" spans="1:7" s="14" customFormat="1">
-      <c r="A212" s="77" t="s">
+      <c r="A212" s="76" t="s">
         <v>231</v>
       </c>
       <c r="B212" s="14" t="s">
@@ -12185,7 +12301,7 @@
       </c>
     </row>
     <row r="213" spans="1:7">
-      <c r="A213" s="72" t="s">
+      <c r="A213" s="71" t="s">
         <v>232</v>
       </c>
       <c r="B213" s="5" t="s">
@@ -12200,9 +12316,12 @@
       <c r="E213" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G213" s="71" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="214" spans="1:7">
-      <c r="A214" s="72" t="s">
+      <c r="A214" s="71" t="s">
         <v>233</v>
       </c>
       <c r="B214" s="5" t="s">
@@ -12217,9 +12336,12 @@
       <c r="E214" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G214" s="71" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="215" spans="1:7">
-      <c r="A215" s="72" t="s">
+      <c r="A215" s="71" t="s">
         <v>234</v>
       </c>
       <c r="B215" s="5" t="s">
@@ -12234,9 +12356,12 @@
       <c r="E215" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G215" s="71" t="s">
+        <v>234</v>
+      </c>
     </row>
     <row r="216" spans="1:7">
-      <c r="A216" s="72" t="s">
+      <c r="A216" s="71" t="s">
         <v>235</v>
       </c>
       <c r="B216" s="5" t="s">
@@ -12251,9 +12376,12 @@
       <c r="E216" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G216" s="71" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="217" spans="1:7">
-      <c r="A217" s="72" t="s">
+      <c r="A217" s="71" t="s">
         <v>236</v>
       </c>
       <c r="B217" s="5" t="s">
@@ -12268,9 +12396,12 @@
       <c r="E217" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G217" s="71" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="218" spans="1:7">
-      <c r="A218" s="72" t="s">
+      <c r="A218" s="71" t="s">
         <v>237</v>
       </c>
       <c r="B218" s="5" t="s">
@@ -12285,9 +12416,12 @@
       <c r="E218" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G218" s="71" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="219" spans="1:7">
-      <c r="A219" s="72" t="s">
+      <c r="A219" s="71" t="s">
         <v>238</v>
       </c>
       <c r="B219" s="5" t="s">
@@ -12302,9 +12436,12 @@
       <c r="E219" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G219" s="71" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="220" spans="1:7">
-      <c r="A220" s="72" t="s">
+      <c r="A220" s="71" t="s">
         <v>239</v>
       </c>
       <c r="B220" s="5" t="s">
@@ -12319,9 +12456,12 @@
       <c r="E220" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G220" s="71" t="s">
+        <v>239</v>
+      </c>
     </row>
     <row r="221" spans="1:7">
-      <c r="A221" s="72" t="s">
+      <c r="A221" s="71" t="s">
         <v>240</v>
       </c>
       <c r="B221" s="5" t="s">
@@ -12336,9 +12476,12 @@
       <c r="E221" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G221" s="71" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="222" spans="1:7">
-      <c r="A222" s="72" t="s">
+      <c r="A222" s="71" t="s">
         <v>241</v>
       </c>
       <c r="B222" s="5" t="s">
@@ -12353,9 +12496,12 @@
       <c r="E222" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G222" s="71" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="223" spans="1:7">
-      <c r="A223" s="72" t="s">
+      <c r="A223" s="71" t="s">
         <v>242</v>
       </c>
       <c r="B223" s="5" t="s">
@@ -12370,9 +12516,12 @@
       <c r="E223" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G223" s="71" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="224" spans="1:7">
-      <c r="A224" s="72" t="s">
+      <c r="A224" s="71" t="s">
         <v>243</v>
       </c>
       <c r="B224" s="5" t="s">
@@ -12387,9 +12536,12 @@
       <c r="E224" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G224" s="71" t="s">
+        <v>243</v>
+      </c>
     </row>
     <row r="225" spans="1:14">
-      <c r="A225" s="72" t="s">
+      <c r="A225" s="71" t="s">
         <v>244</v>
       </c>
       <c r="B225" s="5" t="s">
@@ -12404,9 +12556,12 @@
       <c r="E225" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G225" s="71" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="226" spans="1:14">
-      <c r="A226" s="72" t="s">
+      <c r="A226" s="71" t="s">
         <v>245</v>
       </c>
       <c r="B226" s="5" t="s">
@@ -12421,9 +12576,12 @@
       <c r="E226" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G226" s="71" t="s">
+        <v>245</v>
+      </c>
     </row>
     <row r="227" spans="1:14">
-      <c r="A227" s="72" t="s">
+      <c r="A227" s="71" t="s">
         <v>246</v>
       </c>
       <c r="B227" s="5" t="s">
@@ -12438,9 +12596,12 @@
       <c r="E227" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G227" s="71" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="228" spans="1:14">
-      <c r="A228" s="72" t="s">
+      <c r="A228" s="71" t="s">
         <v>247</v>
       </c>
       <c r="B228" s="5" t="s">
@@ -12455,9 +12616,12 @@
       <c r="E228" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G228" s="71" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="229" spans="1:14">
-      <c r="A229" s="72" t="s">
+      <c r="A229" s="71" t="s">
         <v>248</v>
       </c>
       <c r="B229" s="5" t="s">
@@ -12472,9 +12636,12 @@
       <c r="E229" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G229" s="71" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="230" spans="1:14">
-      <c r="A230" s="72" t="s">
+      <c r="A230" s="71" t="s">
         <v>249</v>
       </c>
       <c r="B230" s="5" t="s">
@@ -12489,9 +12656,12 @@
       <c r="E230" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G230" s="71" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="231" spans="1:14">
-      <c r="A231" s="72" t="s">
+      <c r="A231" s="71" t="s">
         <v>250</v>
       </c>
       <c r="B231" s="5" t="s">
@@ -12506,9 +12676,12 @@
       <c r="E231" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G231" s="71" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="232" spans="1:14">
-      <c r="A232" s="72" t="s">
+      <c r="A232" s="71" t="s">
         <v>251</v>
       </c>
       <c r="B232" s="5" t="s">
@@ -12523,9 +12696,12 @@
       <c r="E232" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G232" s="71" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="233" spans="1:14">
-      <c r="A233" s="72" t="s">
+      <c r="A233" s="71" t="s">
         <v>252</v>
       </c>
       <c r="B233" s="5" t="s">
@@ -12540,9 +12716,12 @@
       <c r="E233" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G233" s="71" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="234" spans="1:14">
-      <c r="A234" s="72" t="s">
+      <c r="A234" s="71" t="s">
         <v>253</v>
       </c>
       <c r="B234" s="5" t="s">
@@ -12557,9 +12736,12 @@
       <c r="E234" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G234" s="71" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="235" spans="1:14">
-      <c r="A235" s="72" t="s">
+      <c r="A235" s="71" t="s">
         <v>254</v>
       </c>
       <c r="B235" s="5" t="s">
@@ -12574,9 +12756,12 @@
       <c r="E235" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G235" s="71" t="s">
+        <v>254</v>
+      </c>
     </row>
     <row r="236" spans="1:14">
-      <c r="A236" s="72" t="s">
+      <c r="A236" s="71" t="s">
         <v>255</v>
       </c>
       <c r="B236" s="5" t="s">
@@ -12591,9 +12776,12 @@
       <c r="E236" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G236" s="71" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="237" spans="1:14" ht="18">
-      <c r="A237" s="72" t="s">
+      <c r="A237" s="71" t="s">
         <v>256</v>
       </c>
       <c r="B237" s="5" t="s">
@@ -12609,7 +12797,7 @@
         <v>301</v>
       </c>
       <c r="G237" s="55" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="H237" s="55"/>
       <c r="I237" s="55"/>
@@ -12620,7 +12808,7 @@
       <c r="N237" s="55"/>
     </row>
     <row r="238" spans="1:14" ht="19">
-      <c r="A238" s="72" t="s">
+      <c r="A238" s="71" t="s">
         <v>257</v>
       </c>
       <c r="B238" s="5" t="s">
@@ -12636,7 +12824,7 @@
         <v>301</v>
       </c>
       <c r="G238" s="55" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="H238" s="55"/>
       <c r="I238" s="55"/>
@@ -12647,7 +12835,7 @@
       <c r="N238" s="55"/>
     </row>
     <row r="239" spans="1:14" ht="18">
-      <c r="A239" s="72" t="s">
+      <c r="A239" s="71" t="s">
         <v>258</v>
       </c>
       <c r="B239" s="5" t="s">
@@ -12663,7 +12851,7 @@
         <v>301</v>
       </c>
       <c r="G239" s="55" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="H239" s="55"/>
       <c r="I239" s="55"/>
@@ -12674,7 +12862,7 @@
       <c r="N239" s="55"/>
     </row>
     <row r="240" spans="1:14">
-      <c r="A240" s="72" t="s">
+      <c r="A240" s="71" t="s">
         <v>259</v>
       </c>
       <c r="B240" s="5" t="s">
@@ -12689,9 +12877,12 @@
       <c r="E240" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G240" s="71" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="241" spans="1:14" ht="18">
-      <c r="A241" s="72" t="s">
+      <c r="A241" s="71" t="s">
         <v>260</v>
       </c>
       <c r="B241" s="5" t="s">
@@ -12707,7 +12898,7 @@
         <v>301</v>
       </c>
       <c r="G241" s="55" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="H241" s="55"/>
       <c r="I241" s="55"/>
@@ -12718,7 +12909,7 @@
       <c r="N241" s="55"/>
     </row>
     <row r="242" spans="1:14" ht="18">
-      <c r="A242" s="72" t="s">
+      <c r="A242" s="71" t="s">
         <v>261</v>
       </c>
       <c r="B242" s="5" t="s">
@@ -12734,7 +12925,7 @@
         <v>301</v>
       </c>
       <c r="G242" s="55" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H242" s="55"/>
       <c r="I242" s="55"/>
@@ -12745,7 +12936,7 @@
       <c r="N242" s="55"/>
     </row>
     <row r="243" spans="1:14">
-      <c r="A243" s="72" t="s">
+      <c r="A243" s="71" t="s">
         <v>262</v>
       </c>
       <c r="B243" s="5" t="s">
@@ -12760,9 +12951,12 @@
       <c r="E243" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G243" s="71" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="244" spans="1:14" ht="18">
-      <c r="A244" s="72" t="s">
+      <c r="A244" s="71" t="s">
         <v>263</v>
       </c>
       <c r="B244" s="5" t="s">
@@ -12778,7 +12972,7 @@
         <v>301</v>
       </c>
       <c r="G244" s="56" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="H244" s="56"/>
       <c r="I244" s="56"/>
@@ -12789,7 +12983,7 @@
       <c r="N244" s="56"/>
     </row>
     <row r="245" spans="1:14">
-      <c r="A245" s="72" t="s">
+      <c r="A245" s="71" t="s">
         <v>264</v>
       </c>
       <c r="B245" s="5" t="s">
@@ -12804,9 +12998,12 @@
       <c r="E245" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G245" s="71" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="246" spans="1:14" ht="18">
-      <c r="A246" s="72" t="s">
+      <c r="A246" s="71" t="s">
         <v>265</v>
       </c>
       <c r="B246" s="5" t="s">
@@ -12822,7 +13019,7 @@
         <v>301</v>
       </c>
       <c r="G246" s="57" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="H246" s="57"/>
       <c r="I246" s="57"/>
@@ -12833,7 +13030,7 @@
       <c r="N246" s="57"/>
     </row>
     <row r="247" spans="1:14">
-      <c r="A247" s="72" t="s">
+      <c r="A247" s="71" t="s">
         <v>266</v>
       </c>
       <c r="B247" s="5" t="s">
@@ -12848,9 +13045,12 @@
       <c r="E247" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G247" s="71" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="248" spans="1:14" ht="18">
-      <c r="A248" s="72" t="s">
+      <c r="A248" s="71" t="s">
         <v>267</v>
       </c>
       <c r="B248" s="5" t="s">
@@ -12866,7 +13066,7 @@
         <v>301</v>
       </c>
       <c r="G248" s="57" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="H248" s="57"/>
       <c r="I248" s="57"/>
@@ -12877,7 +13077,7 @@
       <c r="N248" s="57"/>
     </row>
     <row r="249" spans="1:14">
-      <c r="A249" s="72" t="s">
+      <c r="A249" s="71" t="s">
         <v>268</v>
       </c>
       <c r="B249" s="5" t="s">
@@ -12892,9 +13092,12 @@
       <c r="E249" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G249" s="71" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="250" spans="1:14" ht="18">
-      <c r="A250" s="72" t="s">
+      <c r="A250" s="71" t="s">
         <v>269</v>
       </c>
       <c r="B250" s="5" t="s">
@@ -12910,7 +13113,7 @@
         <v>301</v>
       </c>
       <c r="G250" s="57" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="H250" s="57"/>
       <c r="I250" s="57"/>
@@ -12921,7 +13124,7 @@
       <c r="N250" s="57"/>
     </row>
     <row r="251" spans="1:14">
-      <c r="A251" s="72" t="s">
+      <c r="A251" s="71" t="s">
         <v>270</v>
       </c>
       <c r="B251" s="5" t="s">
@@ -12936,9 +13139,12 @@
       <c r="E251" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G251" s="71" t="s">
+        <v>245</v>
+      </c>
     </row>
     <row r="252" spans="1:14" ht="18">
-      <c r="A252" s="72" t="s">
+      <c r="A252" s="71" t="s">
         <v>271</v>
       </c>
       <c r="B252" s="5" t="s">
@@ -12954,7 +13160,7 @@
         <v>301</v>
       </c>
       <c r="G252" s="57" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="H252" s="57"/>
       <c r="I252" s="57"/>
@@ -12965,7 +13171,7 @@
       <c r="N252" s="57"/>
     </row>
     <row r="253" spans="1:14" ht="18">
-      <c r="A253" s="72" t="s">
+      <c r="A253" s="71" t="s">
         <v>272</v>
       </c>
       <c r="B253" s="5" t="s">
@@ -12981,7 +13187,7 @@
         <v>301</v>
       </c>
       <c r="G253" s="57" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="H253" s="57"/>
       <c r="I253" s="57"/>
@@ -12992,7 +13198,7 @@
       <c r="N253" s="57"/>
     </row>
     <row r="254" spans="1:14">
-      <c r="A254" s="72" t="s">
+      <c r="A254" s="71" t="s">
         <v>70</v>
       </c>
       <c r="B254" s="5" t="s">
@@ -13007,9 +13213,12 @@
       <c r="E254" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G254" s="71" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="255" spans="1:14">
-      <c r="A255" s="72" t="s">
+      <c r="A255" s="71" t="s">
         <v>71</v>
       </c>
       <c r="B255" s="5" t="s">
@@ -13024,9 +13233,12 @@
       <c r="E255" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G255" s="71" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="256" spans="1:14">
-      <c r="A256" s="72" t="s">
+      <c r="A256" s="71" t="s">
         <v>72</v>
       </c>
       <c r="B256" s="5" t="s">
@@ -13041,9 +13253,12 @@
       <c r="E256" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G256" s="71" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="257" spans="1:8">
-      <c r="A257" s="72" t="s">
+      <c r="A257" s="71" t="s">
         <v>73</v>
       </c>
       <c r="B257" s="5" t="s">
@@ -13058,9 +13273,12 @@
       <c r="E257" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G257" s="71" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="258" spans="1:8">
-      <c r="A258" s="72" t="s">
+      <c r="A258" s="71" t="s">
         <v>74</v>
       </c>
       <c r="B258" s="5" t="s">
@@ -13075,419 +13293,422 @@
       <c r="E258" s="6" t="s">
         <v>301</v>
       </c>
+      <c r="G258" s="71" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="259" spans="1:8" s="13" customFormat="1">
-      <c r="A259" s="78" t="s">
+      <c r="A259" s="77" t="s">
+        <v>455</v>
+      </c>
+      <c r="B259" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C259" s="35" t="s">
+        <v>474</v>
+      </c>
+      <c r="D259" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E259" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="G259" s="77" t="s">
+        <v>476</v>
+      </c>
+      <c r="H259" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="260" spans="1:8">
+      <c r="A260" s="77" t="s">
         <v>456</v>
       </c>
-      <c r="B259" s="13" t="s">
+      <c r="B260" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C260" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C259" s="35" t="s">
+      <c r="D260" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E260" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D259" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E259" s="6" t="s">
+      <c r="G260" s="77" t="s">
         <v>476</v>
       </c>
-      <c r="G259" s="78" t="s">
+      <c r="H260" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="261" spans="1:8">
+      <c r="A261" s="77" t="s">
+        <v>457</v>
+      </c>
+      <c r="B261" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C261" s="35" t="s">
+        <v>474</v>
+      </c>
+      <c r="D261" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E261" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="G261" s="77" t="s">
+        <v>476</v>
+      </c>
+      <c r="H261" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="262" spans="1:8">
+      <c r="A262" s="77" t="s">
+        <v>458</v>
+      </c>
+      <c r="B262" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C262" s="35" t="s">
+        <v>474</v>
+      </c>
+      <c r="D262" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E262" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="G262" s="77" t="s">
         <v>477</v>
       </c>
-      <c r="H259" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="260" spans="1:8">
-      <c r="A260" s="78" t="s">
-        <v>457</v>
-      </c>
-      <c r="B260" s="13" t="s">
+      <c r="H262" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="263" spans="1:8">
+      <c r="A263" s="77" t="s">
+        <v>459</v>
+      </c>
+      <c r="B263" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C263" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C260" s="35" t="s">
+      <c r="D263" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E263" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D260" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E260" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G260" s="78" t="s">
+      <c r="G263" s="77" t="s">
         <v>477</v>
       </c>
-      <c r="H260" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="261" spans="1:8">
-      <c r="A261" s="78" t="s">
-        <v>458</v>
-      </c>
-      <c r="B261" s="13" t="s">
+      <c r="H263" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="264" spans="1:8">
+      <c r="A264" s="77" t="s">
+        <v>460</v>
+      </c>
+      <c r="B264" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C264" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C261" s="35" t="s">
+      <c r="D264" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E264" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D261" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E261" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G261" s="78" t="s">
+      <c r="G264" s="77" t="s">
         <v>477</v>
       </c>
-      <c r="H261" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="262" spans="1:8">
-      <c r="A262" s="78" t="s">
-        <v>459</v>
-      </c>
-      <c r="B262" s="13" t="s">
+      <c r="H264" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="265" spans="1:8">
+      <c r="A265" s="77" t="s">
+        <v>461</v>
+      </c>
+      <c r="B265" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C265" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C262" s="35" t="s">
+      <c r="D265" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E265" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D262" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E262" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G262" s="78" t="s">
+      <c r="G265" s="77" t="s">
+        <v>477</v>
+      </c>
+      <c r="H265" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="266" spans="1:8">
+      <c r="A266" s="77" t="s">
+        <v>462</v>
+      </c>
+      <c r="B266" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C266" s="35" t="s">
+        <v>474</v>
+      </c>
+      <c r="D266" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E266" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="G266" s="77" t="s">
         <v>478</v>
       </c>
-      <c r="H262" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="263" spans="1:8">
-      <c r="A263" s="78" t="s">
-        <v>460</v>
-      </c>
-      <c r="B263" s="13" t="s">
+      <c r="H266" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="267" spans="1:8">
+      <c r="A267" s="77" t="s">
+        <v>463</v>
+      </c>
+      <c r="B267" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C267" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C263" s="35" t="s">
+      <c r="D267" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E267" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D263" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E263" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G263" s="78" t="s">
+      <c r="G267" s="77" t="s">
         <v>478</v>
       </c>
-      <c r="H263" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="264" spans="1:8">
-      <c r="A264" s="78" t="s">
-        <v>461</v>
-      </c>
-      <c r="B264" s="13" t="s">
+      <c r="H267" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="268" spans="1:8">
+      <c r="A268" s="77" t="s">
+        <v>464</v>
+      </c>
+      <c r="B268" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C268" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C264" s="35" t="s">
+      <c r="D268" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E268" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D264" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E264" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G264" s="78" t="s">
+      <c r="G268" s="77" t="s">
         <v>478</v>
       </c>
-      <c r="H264" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="265" spans="1:8">
-      <c r="A265" s="78" t="s">
-        <v>462</v>
-      </c>
-      <c r="B265" s="13" t="s">
+      <c r="H268" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="269" spans="1:8">
+      <c r="A269" s="77" t="s">
+        <v>465</v>
+      </c>
+      <c r="B269" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C269" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C265" s="35" t="s">
+      <c r="D269" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E269" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D265" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E265" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G265" s="78" t="s">
+      <c r="G269" s="77" t="s">
         <v>478</v>
       </c>
-      <c r="H265" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="266" spans="1:8">
-      <c r="A266" s="78" t="s">
-        <v>463</v>
-      </c>
-      <c r="B266" s="13" t="s">
+      <c r="H269" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="270" spans="1:8">
+      <c r="A270" s="77" t="s">
+        <v>466</v>
+      </c>
+      <c r="B270" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C270" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C266" s="35" t="s">
+      <c r="D270" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E270" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D266" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E266" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G266" s="78" t="s">
+      <c r="G270" s="77" t="s">
         <v>479</v>
       </c>
-      <c r="H266" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="267" spans="1:8">
-      <c r="A267" s="78" t="s">
-        <v>464</v>
-      </c>
-      <c r="B267" s="13" t="s">
+      <c r="H270" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="271" spans="1:8">
+      <c r="A271" s="77" t="s">
+        <v>467</v>
+      </c>
+      <c r="B271" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C271" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C267" s="35" t="s">
+      <c r="D271" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E271" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D267" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E267" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G267" s="78" t="s">
+      <c r="G271" s="77" t="s">
         <v>479</v>
       </c>
-      <c r="H267" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="268" spans="1:8">
-      <c r="A268" s="78" t="s">
-        <v>465</v>
-      </c>
-      <c r="B268" s="13" t="s">
+      <c r="H271" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="272" spans="1:8">
+      <c r="A272" s="77" t="s">
+        <v>468</v>
+      </c>
+      <c r="B272" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C272" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C268" s="35" t="s">
+      <c r="D272" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E272" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D268" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E268" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G268" s="78" t="s">
+      <c r="G272" s="77" t="s">
         <v>479</v>
       </c>
-      <c r="H268" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="269" spans="1:8">
-      <c r="A269" s="78" t="s">
-        <v>466</v>
-      </c>
-      <c r="B269" s="13" t="s">
+      <c r="H272" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="273" spans="1:9">
+      <c r="A273" s="77" t="s">
+        <v>469</v>
+      </c>
+      <c r="B273" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C273" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C269" s="35" t="s">
+      <c r="D273" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E273" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D269" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E269" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G269" s="78" t="s">
+      <c r="G273" s="77" t="s">
         <v>479</v>
       </c>
-      <c r="H269" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="270" spans="1:8">
-      <c r="A270" s="78" t="s">
-        <v>467</v>
-      </c>
-      <c r="B270" s="13" t="s">
+      <c r="H273" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="274" spans="1:9">
+      <c r="A274" s="77" t="s">
+        <v>470</v>
+      </c>
+      <c r="B274" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C274" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C270" s="35" t="s">
+      <c r="D274" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E274" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D270" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E270" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G270" s="78" t="s">
+      <c r="G274" s="77" t="s">
         <v>480</v>
       </c>
-      <c r="H270" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="271" spans="1:8">
-      <c r="A271" s="78" t="s">
-        <v>468</v>
-      </c>
-      <c r="B271" s="13" t="s">
+      <c r="H274" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="275" spans="1:9">
+      <c r="A275" s="77" t="s">
+        <v>471</v>
+      </c>
+      <c r="B275" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C275" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C271" s="35" t="s">
+      <c r="D275" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E275" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D271" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E271" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G271" s="78" t="s">
+      <c r="G275" s="77" t="s">
         <v>480</v>
       </c>
-      <c r="H271" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="272" spans="1:8">
-      <c r="A272" s="78" t="s">
-        <v>469</v>
-      </c>
-      <c r="B272" s="13" t="s">
+      <c r="H275" s="13" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="276" spans="1:9">
+      <c r="A276" s="77" t="s">
+        <v>472</v>
+      </c>
+      <c r="B276" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="C276" s="35" t="s">
         <v>474</v>
       </c>
-      <c r="C272" s="35" t="s">
+      <c r="D276" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="E276" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="D272" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E272" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G272" s="78" t="s">
+      <c r="G276" s="77" t="s">
         <v>480</v>
       </c>
-      <c r="H272" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="273" spans="1:9">
-      <c r="A273" s="78" t="s">
-        <v>470</v>
-      </c>
-      <c r="B273" s="13" t="s">
-        <v>474</v>
-      </c>
-      <c r="C273" s="35" t="s">
-        <v>475</v>
-      </c>
-      <c r="D273" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E273" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G273" s="78" t="s">
-        <v>480</v>
-      </c>
-      <c r="H273" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="274" spans="1:9">
-      <c r="A274" s="78" t="s">
-        <v>471</v>
-      </c>
-      <c r="B274" s="13" t="s">
-        <v>474</v>
-      </c>
-      <c r="C274" s="35" t="s">
-        <v>475</v>
-      </c>
-      <c r="D274" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E274" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G274" s="78" t="s">
+      <c r="H276" s="13" t="s">
         <v>481</v>
-      </c>
-      <c r="H274" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="275" spans="1:9">
-      <c r="A275" s="78" t="s">
-        <v>472</v>
-      </c>
-      <c r="B275" s="13" t="s">
-        <v>474</v>
-      </c>
-      <c r="C275" s="35" t="s">
-        <v>475</v>
-      </c>
-      <c r="D275" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E275" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G275" s="78" t="s">
-        <v>481</v>
-      </c>
-      <c r="H275" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="276" spans="1:9">
-      <c r="A276" s="78" t="s">
-        <v>473</v>
-      </c>
-      <c r="B276" s="13" t="s">
-        <v>474</v>
-      </c>
-      <c r="C276" s="35" t="s">
-        <v>475</v>
-      </c>
-      <c r="D276" s="34" t="s">
-        <v>169</v>
-      </c>
-      <c r="E276" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G276" s="78" t="s">
-        <v>481</v>
-      </c>
-      <c r="H276" s="13" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="277" spans="1:9" s="15" customFormat="1">
@@ -13509,6 +13730,9 @@
       <c r="F277" s="15" t="s">
         <v>128</v>
       </c>
+      <c r="G277" s="7" t="s">
+        <v>276</v>
+      </c>
       <c r="I277" s="41">
         <v>0.52</v>
       </c>
@@ -13532,6 +13756,9 @@
       <c r="F278" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G278" s="7" t="s">
+        <v>277</v>
+      </c>
       <c r="I278" s="41">
         <v>0.12</v>
       </c>
@@ -13555,6 +13782,9 @@
       <c r="F279" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G279" s="7" t="s">
+        <v>278</v>
+      </c>
       <c r="I279" s="41">
         <v>0.18</v>
       </c>
@@ -13578,6 +13808,9 @@
       <c r="F280" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G280" s="7" t="s">
+        <v>279</v>
+      </c>
       <c r="I280" s="41">
         <v>0.23</v>
       </c>
@@ -13601,6 +13834,9 @@
       <c r="F281" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G281" s="7" t="s">
+        <v>280</v>
+      </c>
       <c r="I281" s="41">
         <v>0.34</v>
       </c>
@@ -13624,6 +13860,9 @@
       <c r="F282" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G282" s="7" t="s">
+        <v>281</v>
+      </c>
       <c r="I282" s="41">
         <v>0.45</v>
       </c>
@@ -13647,6 +13886,9 @@
       <c r="F283" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G283" s="7" t="s">
+        <v>282</v>
+      </c>
       <c r="I283" s="41">
         <v>0.12</v>
       </c>
@@ -13670,6 +13912,9 @@
       <c r="F284" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G284" s="7" t="s">
+        <v>283</v>
+      </c>
       <c r="I284" s="41">
         <v>0.18</v>
       </c>
@@ -13693,6 +13938,9 @@
       <c r="F285" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G285" s="7" t="s">
+        <v>284</v>
+      </c>
       <c r="I285" s="41">
         <v>0.23</v>
       </c>
@@ -13716,6 +13964,9 @@
       <c r="F286" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G286" s="7" t="s">
+        <v>285</v>
+      </c>
       <c r="I286" s="41">
         <v>0.34</v>
       </c>
@@ -13739,6 +13990,9 @@
       <c r="F287" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G287" s="7" t="s">
+        <v>286</v>
+      </c>
       <c r="I287" s="41">
         <v>0.45</v>
       </c>
@@ -13762,6 +14016,9 @@
       <c r="F288" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G288" s="7" t="s">
+        <v>287</v>
+      </c>
       <c r="I288" s="41">
         <v>0.12</v>
       </c>
@@ -13785,6 +14042,9 @@
       <c r="F289" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G289" s="7" t="s">
+        <v>288</v>
+      </c>
       <c r="I289" s="41">
         <v>0.18</v>
       </c>
@@ -13808,6 +14068,9 @@
       <c r="F290" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G290" s="7" t="s">
+        <v>289</v>
+      </c>
       <c r="I290" s="41">
         <v>0.23</v>
       </c>
@@ -13831,6 +14094,9 @@
       <c r="F291" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G291" s="7" t="s">
+        <v>290</v>
+      </c>
       <c r="I291" s="41">
         <v>0.34</v>
       </c>
@@ -13854,6 +14120,9 @@
       <c r="F292" s="15" t="s">
         <v>167</v>
       </c>
+      <c r="G292" s="7" t="s">
+        <v>291</v>
+      </c>
       <c r="I292" s="41">
         <v>0.45</v>
       </c>
@@ -13877,7 +14146,7 @@
       <c r="F293" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="G293" s="64" t="s">
+      <c r="G293" s="63" t="s">
         <v>376</v>
       </c>
     </row>
@@ -13900,7 +14169,7 @@
       <c r="F294" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="G294" s="64" t="s">
+      <c r="G294" s="63" t="s">
         <v>376</v>
       </c>
     </row>
@@ -13923,7 +14192,7 @@
       <c r="F295" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="G295" s="64" t="s">
+      <c r="G295" s="63" t="s">
         <v>376</v>
       </c>
     </row>
@@ -13946,7 +14215,7 @@
       <c r="F296" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="G296" s="64" t="s">
+      <c r="G296" s="63" t="s">
         <v>377</v>
       </c>
     </row>
@@ -13969,7 +14238,7 @@
       <c r="F297" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="G297" s="64" t="s">
+      <c r="G297" s="63" t="s">
         <v>377</v>
       </c>
     </row>
@@ -13992,7 +14261,7 @@
       <c r="F298" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="G298" s="64" t="s">
+      <c r="G298" s="63" t="s">
         <v>377</v>
       </c>
     </row>
@@ -14015,7 +14284,7 @@
       <c r="F299" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="G299" s="64" t="s">
+      <c r="G299" s="63" t="s">
         <v>378</v>
       </c>
     </row>
@@ -14038,7 +14307,7 @@
       <c r="F300" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="G300" s="64" t="s">
+      <c r="G300" s="63" t="s">
         <v>378</v>
       </c>
     </row>
@@ -14061,11 +14330,12 @@
       <c r="F301" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="G301" s="64" t="s">
+      <c r="G301" s="63" t="s">
         <v>378</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="G1:G301" xr:uid="{7E8F22EE-2E06-6741-B451-D4EA064EAB2E}"/>
   <phoneticPr fontId="26" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C159" r:id="rId1" xr:uid="{BF63034B-E53E-AA4F-9F22-3EC9CCE474BD}"/>

</xml_diff>